<commit_message>
Vector stats, Condensed delete calls into single file
Condensed item delete calls into single file (itemDelete.rul)
Deleted more unused ufo things to clean up wiki
Updated enemy itemsets to add vector
updated version number
Vector stats/sound
Reduced ground->QD item movement cost to match ground->hand->QD, which was 1 faster
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD9858E-BB72-4436-972D-75B7692887F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0A0205-2037-4FC2-AC0B-AE48166BA516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="735" windowWidth="19440" windowHeight="15000" activeTab="6" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="28680" yWindow="735" windowWidth="19440" windowHeight="15000" firstSheet="7" activeTab="12" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1768" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="595">
   <si>
     <t>Name</t>
   </si>
@@ -1086,10 +1086,6 @@
 120</t>
   </si>
   <si>
-    <t>100000
-+ 10000</t>
-  </si>
-  <si>
     <t>1
 3</t>
   </si>
@@ -1628,27 +1624,18 @@
     <t>AR-18/G3?</t>
   </si>
   <si>
-    <t>Origin-12/Deagle/Gold Deagle</t>
-  </si>
-  <si>
     <t>M4 Carbine/SCAR L/Deagle</t>
   </si>
   <si>
     <t>Remington 870/M9/Deagle</t>
   </si>
   <si>
-    <t>Skorpion/Stechkin/Glock 17</t>
-  </si>
-  <si>
     <t>TEC-9/Glock18/Spas 12</t>
   </si>
   <si>
     <t>M16/M16 (m203 Smoke)/Deagle</t>
   </si>
   <si>
-    <t>M4 Carbine/M4 (M320 Smoke)/M4 (UBS)</t>
-  </si>
-  <si>
     <t>AR-18/Spas 12/G3</t>
   </si>
   <si>
@@ -1658,9 +1645,6 @@
     <t>RPK/RPK/AKM</t>
   </si>
   <si>
-    <t>AKs-74u/AK-74/Glock 17</t>
-  </si>
-  <si>
     <t>M249/M60/M60</t>
   </si>
   <si>
@@ -1763,12 +1747,6 @@
     <t>Shield + MK 23/Deagle/P226</t>
   </si>
   <si>
-    <t>Skorpion EVO/Deagle/Golden Deagle</t>
-  </si>
-  <si>
-    <t>MK23/M4 Carbine (Sopmod)/?</t>
-  </si>
-  <si>
     <t>Glock 18/G36C/?</t>
   </si>
   <si>
@@ -1781,9 +1759,6 @@
     <t>HK417/?/?</t>
   </si>
   <si>
-    <t>Deagle/Skorpion EVO/?</t>
-  </si>
-  <si>
     <t>Browning HP</t>
   </si>
   <si>
@@ -1962,6 +1937,40 @@
   </si>
   <si>
     <t>Movement pen.</t>
+  </si>
+  <si>
+    <t>Kriss Vector</t>
+  </si>
+  <si>
+    <t>AKs-74u/Stechkin/Glock 17</t>
+  </si>
+  <si>
+    <t>AKs-74u (Sopmod)/AK-74 (GP-25 Smoke)/AK-74 (GP-25 Frag)</t>
+  </si>
+  <si>
+    <t>AKs-74u (Sopmod)/AK-74 (GP-25 Frag)/Vektor</t>
+  </si>
+  <si>
+    <t>M4 Carbine/M4 (UBS)/Deagle</t>
+  </si>
+  <si>
+    <t>Kriss Vector/Origin-12/Gold Deagle</t>
+  </si>
+  <si>
+    <t>Skorpion EVO/Kriss Vector/Golden Deagle</t>
+  </si>
+  <si>
+    <t>Deagle/Skorpion EVO/Kriss Vector</t>
+  </si>
+  <si>
+    <t>MK23/M4 Carbine (Sopmod)/M4 Carbine (Sopmod)</t>
+  </si>
+  <si>
+    <t>100000 &lt;=vet diff 200000 &gt;vet diff</t>
+  </si>
+  <si>
+    <t>1/2 Recruit cost
++ 10000</t>
   </si>
 </sst>
 </file>
@@ -3645,8 +3654,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{EB47442F-754D-45A1-BC57-BBE7964D0858}" name="Table10" displayName="Table10" ref="A1:Z16" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17">
-  <autoFilter ref="A1:Z16" xr:uid="{EB47442F-754D-45A1-BC57-BBE7964D0858}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{EB47442F-754D-45A1-BC57-BBE7964D0858}" name="Table10" displayName="Table10" ref="A1:Z17" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17">
+  <autoFilter ref="A1:Z17" xr:uid="{EB47442F-754D-45A1-BC57-BBE7964D0858}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z15">
     <sortCondition descending="1" ref="M1:M15"/>
   </sortState>
@@ -4314,7 +4323,7 @@
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C10">
         <v>40</v>
@@ -4329,13 +4338,13 @@
         <v>1</v>
       </c>
       <c r="I10" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="56"/>
       <c r="B11" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C11">
         <v>30</v>
@@ -4769,7 +4778,7 @@
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="C24">
         <v>40</v>
@@ -4997,7 +5006,7 @@
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C29">
         <v>18</v>
@@ -5018,13 +5027,13 @@
         <v>2</v>
       </c>
       <c r="I29" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C30">
         <v>10</v>
@@ -5045,7 +5054,7 @@
         <v>11</v>
       </c>
       <c r="I30" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="M30" s="12" t="s">
         <v>41</v>
@@ -5524,7 +5533,7 @@
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
       <c r="B44" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="C44">
         <v>95</v>
@@ -5542,13 +5551,13 @@
         <v>3</v>
       </c>
       <c r="I44" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45" s="9"/>
       <c r="B45" t="s">
-        <v>550</v>
+        <v>542</v>
       </c>
       <c r="C45">
         <v>40</v>
@@ -5566,13 +5575,13 @@
         <v>3</v>
       </c>
       <c r="I45" t="s">
-        <v>549</v>
+        <v>541</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
       <c r="B46" t="s">
-        <v>551</v>
+        <v>543</v>
       </c>
       <c r="C46">
         <v>40</v>
@@ -5598,7 +5607,7 @@
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A48" s="53" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B48" t="s">
         <v>0</v>
@@ -5628,7 +5637,7 @@
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="54"/>
       <c r="B49" s="14" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C49">
         <v>40</v>
@@ -5643,7 +5652,7 @@
         <v>7</v>
       </c>
       <c r="I49" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -7199,12 +7208,13 @@
     <col min="1" max="1" width="12.42578125" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="13" max="13" width="11.85546875" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
     <col min="16" max="16" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B1" s="20" t="s">
         <v>236</v>
@@ -7252,9 +7262,9 @@
         <v>307</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B2" s="32" t="s">
         <v>294</v>
@@ -7291,16 +7301,16 @@
       </c>
       <c r="M2" s="38"/>
       <c r="N2" s="38"/>
-      <c r="O2" s="32">
-        <v>200000</v>
+      <c r="O2" s="32" t="s">
+        <v>593</v>
       </c>
       <c r="P2" s="32" t="s">
-        <v>313</v>
+        <v>594</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="96" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B3" s="26" t="s">
         <v>298</v>
@@ -7336,10 +7346,10 @@
         <v>50</v>
       </c>
       <c r="M3" s="26" t="s">
+        <v>313</v>
+      </c>
+      <c r="N3" s="26" t="s">
         <v>314</v>
-      </c>
-      <c r="N3" s="26" t="s">
-        <v>315</v>
       </c>
       <c r="O3" s="39"/>
       <c r="P3" s="39"/>
@@ -7380,10 +7390,10 @@
         <v>40</v>
       </c>
       <c r="M4" s="32" t="s">
+        <v>313</v>
+      </c>
+      <c r="N4" s="32" t="s">
         <v>314</v>
-      </c>
-      <c r="N4" s="32" t="s">
-        <v>315</v>
       </c>
       <c r="O4" s="38"/>
       <c r="P4" s="38"/>
@@ -7391,7 +7401,7 @@
     <row r="5" spans="1:16" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="97"/>
       <c r="B5" s="26" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C5" s="21">
         <v>60</v>
@@ -7424,10 +7434,10 @@
         <v>25</v>
       </c>
       <c r="M5" s="26" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="N5" s="26" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="O5" s="39"/>
       <c r="P5" s="39"/>
@@ -7435,7 +7445,7 @@
     <row r="6" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="97"/>
       <c r="B6" s="32" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C6" s="21">
         <v>65</v>
@@ -7468,10 +7478,10 @@
         <v>20</v>
       </c>
       <c r="M6" s="32" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="N6" s="32" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="O6" s="38"/>
       <c r="P6" s="38"/>
@@ -7479,7 +7489,7 @@
     <row r="7" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="97"/>
       <c r="B7" s="26" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C7" s="21">
         <v>75</v>
@@ -7512,7 +7522,7 @@
         <v>20</v>
       </c>
       <c r="M7" s="26" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N7" s="26" t="s">
         <v>255</v>
@@ -7523,7 +7533,7 @@
     <row r="8" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="97"/>
       <c r="B8" s="32" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C8" s="21">
         <v>60</v>
@@ -7556,7 +7566,7 @@
         <v>15</v>
       </c>
       <c r="M8" s="32" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="N8" s="32" t="s">
         <v>255</v>
@@ -7567,7 +7577,7 @@
     <row r="9" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="97"/>
       <c r="B9" s="26" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C9" s="21">
         <v>60</v>
@@ -7600,7 +7610,7 @@
         <v>30</v>
       </c>
       <c r="M9" s="26" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="N9" s="26" t="s">
         <v>255</v>
@@ -7611,7 +7621,7 @@
     <row r="10" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="98"/>
       <c r="B10" s="32" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C10" s="21">
         <v>60</v>
@@ -7644,17 +7654,17 @@
         <v>30</v>
       </c>
       <c r="M10" s="32" t="s">
+        <v>325</v>
+      </c>
+      <c r="N10" s="32" t="s">
         <v>326</v>
-      </c>
-      <c r="N10" s="32" t="s">
-        <v>327</v>
       </c>
       <c r="O10" s="38"/>
       <c r="P10" s="38"/>
     </row>
     <row r="11" spans="1:16" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="96" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B11" s="26" t="s">
         <v>298</v>
@@ -7710,10 +7720,10 @@
         <v>50</v>
       </c>
       <c r="M12" s="32" t="s">
+        <v>327</v>
+      </c>
+      <c r="N12" s="32" t="s">
         <v>328</v>
-      </c>
-      <c r="N12" s="32" t="s">
-        <v>329</v>
       </c>
       <c r="O12" s="38"/>
       <c r="P12" s="38"/>
@@ -7721,7 +7731,7 @@
     <row r="13" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="97"/>
       <c r="B13" s="26" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C13" s="21">
         <v>70</v>
@@ -7754,10 +7764,10 @@
         <v>30</v>
       </c>
       <c r="M13" s="26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="N13" s="26" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="O13" s="39"/>
       <c r="P13" s="39"/>
@@ -7765,7 +7775,7 @@
     <row r="14" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="97"/>
       <c r="B14" s="32" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C14" s="21">
         <v>75</v>
@@ -7798,10 +7808,10 @@
         <v>30</v>
       </c>
       <c r="M14" s="32" t="s">
+        <v>313</v>
+      </c>
+      <c r="N14" s="32" t="s">
         <v>314</v>
-      </c>
-      <c r="N14" s="32" t="s">
-        <v>315</v>
       </c>
       <c r="O14" s="38"/>
       <c r="P14" s="38"/>
@@ -7842,10 +7852,10 @@
         <v>30</v>
       </c>
       <c r="M15" s="26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="N15" s="26" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="O15" s="39"/>
       <c r="P15" s="39"/>
@@ -7853,7 +7863,7 @@
     <row r="16" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="97"/>
       <c r="B16" s="32" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C16" s="21">
         <v>75</v>
@@ -7886,10 +7896,10 @@
         <v>30</v>
       </c>
       <c r="M16" s="32" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="N16" s="32" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="O16" s="38"/>
       <c r="P16" s="38"/>
@@ -7897,7 +7907,7 @@
     <row r="17" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="97"/>
       <c r="B17" s="26" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C17" s="21">
         <v>75</v>
@@ -7930,10 +7940,10 @@
         <v>30</v>
       </c>
       <c r="M17" s="26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="N17" s="26" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="O17" s="39"/>
       <c r="P17" s="39"/>
@@ -7941,7 +7951,7 @@
     <row r="18" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="98"/>
       <c r="B18" s="32" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C18" s="21">
         <v>70</v>
@@ -7974,10 +7984,10 @@
         <v>30</v>
       </c>
       <c r="M18" s="32" t="s">
+        <v>332</v>
+      </c>
+      <c r="N18" s="32" t="s">
         <v>333</v>
-      </c>
-      <c r="N18" s="32" t="s">
-        <v>334</v>
       </c>
       <c r="O18" s="38"/>
       <c r="P18" s="38"/>
@@ -7999,8 +8009,8 @@
     <col min="2" max="2" width="12.140625" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="36.140625" customWidth="1"/>
-    <col min="6" max="6" width="42.85546875" customWidth="1"/>
+    <col min="5" max="5" width="43.140625" customWidth="1"/>
+    <col min="6" max="6" width="53.7109375" customWidth="1"/>
     <col min="7" max="7" width="46.28515625" customWidth="1"/>
     <col min="8" max="8" width="14.42578125" customWidth="1"/>
     <col min="9" max="9" width="30.140625" customWidth="1"/>
@@ -8008,25 +8018,25 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B1" s="44" t="s">
+        <v>338</v>
+      </c>
+      <c r="C1" s="44" t="s">
         <v>339</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="D1" s="44" t="s">
         <v>340</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="E1" s="44" t="s">
         <v>341</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="F1" s="44" t="s">
         <v>342</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="G1" s="44" t="s">
         <v>343</v>
-      </c>
-      <c r="G1" s="44" t="s">
-        <v>344</v>
       </c>
       <c r="H1" s="44" t="s">
         <v>237</v>
@@ -8035,7 +8045,7 @@
     </row>
     <row r="2" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="102" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B2" s="102" t="s">
         <v>298</v>
@@ -8044,19 +8054,19 @@
         <v>298</v>
       </c>
       <c r="D2" s="45" t="s">
+        <v>344</v>
+      </c>
+      <c r="E2" s="45" t="s">
+        <v>473</v>
+      </c>
+      <c r="F2" s="45" t="s">
+        <v>473</v>
+      </c>
+      <c r="G2" s="45" t="s">
         <v>345</v>
       </c>
-      <c r="E2" s="45" t="s">
-        <v>474</v>
-      </c>
-      <c r="F2" s="45" t="s">
-        <v>474</v>
-      </c>
-      <c r="G2" s="45" t="s">
+      <c r="H2" s="102" t="s">
         <v>346</v>
-      </c>
-      <c r="H2" s="102" t="s">
-        <v>347</v>
       </c>
       <c r="I2" s="62"/>
     </row>
@@ -8065,16 +8075,16 @@
       <c r="B3" s="100"/>
       <c r="C3" s="100"/>
       <c r="D3" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E3" s="46" t="s">
+        <v>474</v>
+      </c>
+      <c r="F3" s="46" t="s">
+        <v>474</v>
+      </c>
+      <c r="G3" s="46" t="s">
         <v>475</v>
-      </c>
-      <c r="F3" s="46" t="s">
-        <v>475</v>
-      </c>
-      <c r="G3" s="46" t="s">
-        <v>476</v>
       </c>
       <c r="H3" s="100"/>
     </row>
@@ -8083,16 +8093,16 @@
       <c r="B4" s="100"/>
       <c r="C4" s="100"/>
       <c r="D4" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E4" s="60" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F4" s="60" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="G4" s="60" t="s">
-        <v>480</v>
+        <v>589</v>
       </c>
       <c r="H4" s="100"/>
     </row>
@@ -8105,19 +8115,19 @@
         <v>299</v>
       </c>
       <c r="D5" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E5" s="61" t="s">
-        <v>483</v>
+        <v>585</v>
       </c>
       <c r="F5" s="61" t="s">
-        <v>490</v>
+        <v>586</v>
       </c>
       <c r="G5" s="61" t="s">
-        <v>490</v>
+        <v>587</v>
       </c>
       <c r="H5" s="99" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8125,16 +8135,16 @@
       <c r="B6" s="100"/>
       <c r="C6" s="100"/>
       <c r="D6" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="G6" s="46" t="s">
-        <v>588</v>
+        <v>580</v>
       </c>
       <c r="H6" s="100"/>
     </row>
@@ -8143,41 +8153,41 @@
       <c r="B7" s="103"/>
       <c r="C7" s="103"/>
       <c r="D7" s="59" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E7" s="59" t="s">
+        <v>480</v>
+      </c>
+      <c r="F7" s="59" t="s">
         <v>482</v>
       </c>
-      <c r="F7" s="59" t="s">
-        <v>485</v>
-      </c>
       <c r="G7" s="59" t="s">
-        <v>486</v>
+        <v>588</v>
       </c>
       <c r="H7" s="103"/>
     </row>
     <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="100"/>
       <c r="B8" s="99" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C8" s="99" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D8" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E8" s="61" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="F8" s="61" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="G8" s="61" t="s">
         <v>220</v>
       </c>
       <c r="H8" s="99" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8185,16 +8195,16 @@
       <c r="B9" s="100"/>
       <c r="C9" s="100"/>
       <c r="D9" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="F9" s="46" t="s">
+        <v>561</v>
+      </c>
+      <c r="G9" s="46" t="s">
         <v>569</v>
-      </c>
-      <c r="G9" s="46" t="s">
-        <v>577</v>
       </c>
       <c r="H9" s="100"/>
     </row>
@@ -8203,41 +8213,41 @@
       <c r="B10" s="103"/>
       <c r="C10" s="103"/>
       <c r="D10" s="59" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E10" s="59" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F10" s="59" t="s">
-        <v>578</v>
+        <v>570</v>
       </c>
       <c r="G10" s="59" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="H10" s="103"/>
     </row>
     <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="100"/>
       <c r="B11" s="99" t="s">
+        <v>355</v>
+      </c>
+      <c r="C11" s="99" t="s">
+        <v>317</v>
+      </c>
+      <c r="D11" s="61" t="s">
+        <v>344</v>
+      </c>
+      <c r="E11" s="61" t="s">
+        <v>460</v>
+      </c>
+      <c r="F11" s="61" t="s">
+        <v>460</v>
+      </c>
+      <c r="G11" s="61" t="s">
+        <v>558</v>
+      </c>
+      <c r="H11" s="99" t="s">
         <v>356</v>
-      </c>
-      <c r="C11" s="99" t="s">
-        <v>318</v>
-      </c>
-      <c r="D11" s="61" t="s">
-        <v>345</v>
-      </c>
-      <c r="E11" s="61" t="s">
-        <v>461</v>
-      </c>
-      <c r="F11" s="61" t="s">
-        <v>461</v>
-      </c>
-      <c r="G11" s="61" t="s">
-        <v>566</v>
-      </c>
-      <c r="H11" s="99" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8245,16 +8255,16 @@
       <c r="B12" s="100"/>
       <c r="C12" s="100"/>
       <c r="D12" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E12" s="46" t="s">
         <v>203</v>
       </c>
       <c r="F12" s="46" t="s">
+        <v>477</v>
+      </c>
+      <c r="G12" s="46" t="s">
         <v>478</v>
-      </c>
-      <c r="G12" s="46" t="s">
-        <v>479</v>
       </c>
       <c r="H12" s="100"/>
     </row>
@@ -8263,41 +8273,41 @@
       <c r="B13" s="100"/>
       <c r="C13" s="100"/>
       <c r="D13" s="60" t="s">
+        <v>348</v>
+      </c>
+      <c r="E13" s="60" t="s">
+        <v>357</v>
+      </c>
+      <c r="F13" s="60" t="s">
+        <v>352</v>
+      </c>
+      <c r="G13" s="60" t="s">
         <v>349</v>
-      </c>
-      <c r="E13" s="60" t="s">
-        <v>358</v>
-      </c>
-      <c r="F13" s="60" t="s">
-        <v>353</v>
-      </c>
-      <c r="G13" s="60" t="s">
-        <v>350</v>
       </c>
       <c r="H13" s="100"/>
     </row>
     <row r="14" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="100"/>
       <c r="B14" s="99" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C14" s="99" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D14" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E14" s="61" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="F14" s="61" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G14" s="61" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="H14" s="99" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8305,16 +8315,16 @@
       <c r="B15" s="100"/>
       <c r="C15" s="100"/>
       <c r="D15" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E15" s="46" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F15" s="46" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G15" s="46" t="s">
-        <v>584</v>
+        <v>576</v>
       </c>
       <c r="H15" s="100"/>
     </row>
@@ -8323,29 +8333,29 @@
       <c r="B16" s="103"/>
       <c r="C16" s="103"/>
       <c r="D16" s="59" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E16" s="59" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="F16" s="59" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G16" s="59" t="s">
-        <v>585</v>
+        <v>577</v>
       </c>
       <c r="H16" s="103"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="100"/>
       <c r="B17" s="99" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C17" s="99" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D17" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E17" s="61" t="s">
         <v>11</v>
@@ -8354,10 +8364,10 @@
         <v>111</v>
       </c>
       <c r="G17" s="61" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H17" s="99" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8365,16 +8375,16 @@
       <c r="B18" s="100"/>
       <c r="C18" s="100"/>
       <c r="D18" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E18" s="46" t="s">
-        <v>565</v>
+        <v>557</v>
       </c>
       <c r="F18" s="46" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G18" s="46" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="H18" s="100"/>
     </row>
@@ -8383,41 +8393,41 @@
       <c r="B19" s="103"/>
       <c r="C19" s="103"/>
       <c r="D19" s="59" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E19" s="59" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="F19" s="59" t="s">
-        <v>542</v>
+        <v>534</v>
       </c>
       <c r="G19" s="59" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="H19" s="103"/>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="100"/>
       <c r="B20" s="99" t="s">
+        <v>362</v>
+      </c>
+      <c r="C20" s="99" t="s">
+        <v>323</v>
+      </c>
+      <c r="D20" s="61" t="s">
+        <v>344</v>
+      </c>
+      <c r="E20" s="61" t="s">
         <v>363</v>
       </c>
-      <c r="C20" s="99" t="s">
-        <v>324</v>
-      </c>
-      <c r="D20" s="61" t="s">
-        <v>345</v>
-      </c>
-      <c r="E20" s="61" t="s">
+      <c r="F20" s="61" t="s">
+        <v>545</v>
+      </c>
+      <c r="G20" s="61" t="s">
         <v>364</v>
       </c>
-      <c r="F20" s="61" t="s">
-        <v>553</v>
-      </c>
-      <c r="G20" s="61" t="s">
-        <v>365</v>
-      </c>
       <c r="H20" s="99" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8425,16 +8435,16 @@
       <c r="B21" s="100"/>
       <c r="C21" s="100"/>
       <c r="D21" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E21" s="46" t="s">
-        <v>564</v>
+        <v>556</v>
       </c>
       <c r="F21" s="46" t="s">
-        <v>552</v>
+        <v>544</v>
       </c>
       <c r="G21" s="46" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H21" s="100"/>
     </row>
@@ -8443,41 +8453,41 @@
       <c r="B22" s="100"/>
       <c r="C22" s="100"/>
       <c r="D22" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E22" s="60" t="s">
+        <v>365</v>
+      </c>
+      <c r="F22" s="60" t="s">
         <v>366</v>
       </c>
-      <c r="F22" s="60" t="s">
+      <c r="G22" s="60" t="s">
         <v>367</v>
-      </c>
-      <c r="G22" s="60" t="s">
-        <v>368</v>
       </c>
       <c r="H22" s="101"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="100"/>
       <c r="B23" s="99" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C23" s="99" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D23" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E23" s="61" t="s">
         <v>148</v>
       </c>
       <c r="F23" s="61" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="G23" s="61" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="H23" s="102" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8485,16 +8495,16 @@
       <c r="B24" s="100"/>
       <c r="C24" s="100"/>
       <c r="D24" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E24" s="65" t="s">
-        <v>560</v>
+        <v>552</v>
       </c>
       <c r="F24" s="46" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="G24" s="46" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="H24" s="100"/>
     </row>
@@ -8503,22 +8513,22 @@
       <c r="B25" s="101"/>
       <c r="C25" s="101"/>
       <c r="D25" s="47" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E25" s="47" t="s">
-        <v>559</v>
+        <v>551</v>
       </c>
       <c r="F25" s="47" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="G25" s="47" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="H25" s="101"/>
     </row>
     <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="102" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B26" s="102" t="s">
         <v>298</v>
@@ -8527,7 +8537,7 @@
         <v>298</v>
       </c>
       <c r="D26" s="45" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E26" s="104"/>
       <c r="F26" s="105"/>
@@ -8539,7 +8549,7 @@
       <c r="B27" s="100"/>
       <c r="C27" s="100"/>
       <c r="D27" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E27" s="104"/>
       <c r="F27" s="105"/>
@@ -8551,7 +8561,7 @@
       <c r="B28" s="100"/>
       <c r="C28" s="100"/>
       <c r="D28" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E28" s="109"/>
       <c r="F28" s="110"/>
@@ -8567,19 +8577,19 @@
         <v>299</v>
       </c>
       <c r="D29" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E29" s="75" t="s">
-        <v>528</v>
+        <v>521</v>
       </c>
       <c r="F29" s="64" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="G29" s="76" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="H29" s="99" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8587,13 +8597,13 @@
       <c r="B30" s="100"/>
       <c r="C30" s="100"/>
       <c r="D30" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E30" s="79" t="s">
-        <v>527</v>
+        <v>520</v>
       </c>
       <c r="F30" s="71" t="s">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="G30" s="77" t="s">
         <v>209</v>
@@ -8605,41 +8615,41 @@
       <c r="B31" s="103"/>
       <c r="C31" s="103"/>
       <c r="D31" s="59" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E31" s="78" t="s">
-        <v>526</v>
+        <v>592</v>
       </c>
       <c r="F31" s="74" t="s">
-        <v>531</v>
+        <v>591</v>
       </c>
       <c r="G31" s="78" t="s">
-        <v>525</v>
+        <v>590</v>
       </c>
       <c r="H31" s="103"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="100"/>
       <c r="B32" s="100" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C32" s="100" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D32" s="58" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E32" s="73" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="F32" s="80" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
       <c r="G32" s="73" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="H32" s="100" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8647,16 +8657,16 @@
       <c r="B33" s="100"/>
       <c r="C33" s="100"/>
       <c r="D33" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E33" s="79" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="F33" s="71" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="G33" s="79" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="H33" s="100"/>
     </row>
@@ -8665,41 +8675,41 @@
       <c r="B34" s="100"/>
       <c r="C34" s="100"/>
       <c r="D34" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E34" s="67" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="F34" s="81" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="G34" s="67" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="H34" s="100"/>
     </row>
     <row r="35" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="100"/>
       <c r="B35" s="99" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C35" s="99" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D35" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E35" s="75" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="F35" s="75" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="G35" s="75" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="H35" s="99" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8707,16 +8717,16 @@
       <c r="B36" s="100"/>
       <c r="C36" s="100"/>
       <c r="D36" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E36" s="79" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="F36" s="79" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="G36" s="79" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="H36" s="100"/>
     </row>
@@ -8725,41 +8735,41 @@
       <c r="B37" s="100"/>
       <c r="C37" s="100"/>
       <c r="D37" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E37" s="90" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F37" s="90" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="G37" s="90" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="H37" s="100"/>
     </row>
     <row r="38" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="100"/>
       <c r="B38" s="99" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C38" s="99" t="s">
         <v>287</v>
       </c>
       <c r="D38" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E38" s="63" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="F38" s="85" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
       <c r="G38" s="63" t="s">
-        <v>567</v>
+        <v>559</v>
       </c>
       <c r="H38" s="99" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8767,16 +8777,16 @@
       <c r="B39" s="100"/>
       <c r="C39" s="100"/>
       <c r="D39" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E39" s="79" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="F39" s="71" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="G39" s="79" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="H39" s="100"/>
     </row>
@@ -8785,41 +8795,41 @@
       <c r="B40" s="100"/>
       <c r="C40" s="100"/>
       <c r="D40" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E40" s="67" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="F40" s="81" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="G40" s="67" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="H40" s="100"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="100"/>
       <c r="B41" s="99" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C41" s="99" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D41" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E41" s="86" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="F41" s="80" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
       <c r="G41" s="86" t="s">
-        <v>563</v>
+        <v>555</v>
       </c>
       <c r="H41" s="99" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8827,16 +8837,16 @@
       <c r="B42" s="100"/>
       <c r="C42" s="100"/>
       <c r="D42" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E42" s="87" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="F42" s="88" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="G42" s="87" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="H42" s="100"/>
     </row>
@@ -8845,41 +8855,41 @@
       <c r="B43" s="100"/>
       <c r="C43" s="100"/>
       <c r="D43" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E43" s="67" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="F43" s="89" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="G43" s="67" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="H43" s="100"/>
     </row>
     <row r="44" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="100"/>
       <c r="B44" s="99" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C44" s="99" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D44" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E44" s="68" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="F44" s="82" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="G44" s="68" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="H44" s="99" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8887,16 +8897,16 @@
       <c r="B45" s="100"/>
       <c r="C45" s="100"/>
       <c r="D45" s="66" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E45" s="69" t="s">
-        <v>570</v>
+        <v>562</v>
       </c>
       <c r="F45" s="69" t="s">
-        <v>581</v>
+        <v>573</v>
       </c>
       <c r="G45" s="69" t="s">
-        <v>582</v>
+        <v>574</v>
       </c>
       <c r="H45" s="100"/>
     </row>
@@ -8905,41 +8915,41 @@
       <c r="B46" s="100"/>
       <c r="C46" s="100"/>
       <c r="D46" s="60" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E46" s="67" t="s">
-        <v>579</v>
+        <v>571</v>
       </c>
       <c r="F46" s="81" t="s">
-        <v>580</v>
+        <v>572</v>
       </c>
       <c r="G46" s="67" t="s">
-        <v>583</v>
+        <v>575</v>
       </c>
       <c r="H46" s="100"/>
     </row>
     <row r="47" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="100"/>
       <c r="B47" s="99" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C47" s="99" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D47" s="61" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="E47" s="63" t="s">
         <v>158</v>
       </c>
       <c r="F47" s="80" t="s">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="G47" s="63" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="H47" s="99" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8947,16 +8957,16 @@
       <c r="B48" s="100"/>
       <c r="C48" s="100"/>
       <c r="D48" s="46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E48" s="70" t="s">
-        <v>510</v>
+        <v>505</v>
       </c>
       <c r="F48" s="83" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="G48" s="70" t="s">
-        <v>508</v>
+        <v>503</v>
       </c>
       <c r="H48" s="100"/>
     </row>
@@ -8965,16 +8975,16 @@
       <c r="B49" s="101"/>
       <c r="C49" s="101"/>
       <c r="D49" s="47" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E49" s="84" t="s">
-        <v>511</v>
+        <v>506</v>
       </c>
       <c r="F49" s="72" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="G49" s="84" t="s">
-        <v>509</v>
+        <v>504</v>
       </c>
       <c r="H49" s="101"/>
     </row>
@@ -9059,111 +9069,111 @@
         <v>236</v>
       </c>
       <c r="B1" s="20" t="s">
+        <v>370</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>371</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="D1" s="20" t="s">
         <v>372</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="E1" s="20" t="s">
         <v>373</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="F1" s="20" t="s">
         <v>374</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="G1" s="20" t="s">
         <v>375</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="H1" s="20" t="s">
         <v>376</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="I1" s="20" t="s">
         <v>377</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="J1" s="20" t="s">
         <v>378</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="K1" s="20" t="s">
         <v>379</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="L1" s="20" t="s">
         <v>380</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="M1" s="20" t="s">
         <v>381</v>
       </c>
-      <c r="M1" s="20" t="s">
+      <c r="N1" s="20" t="s">
         <v>382</v>
       </c>
-      <c r="N1" s="20" t="s">
+      <c r="O1" s="20" t="s">
         <v>383</v>
       </c>
-      <c r="O1" s="20" t="s">
+      <c r="P1" s="20" t="s">
         <v>384</v>
-      </c>
-      <c r="P1" s="20" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
+        <v>385</v>
+      </c>
+      <c r="B2" s="32" t="s">
         <v>386</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>387</v>
       </c>
       <c r="C2" s="32">
         <v>3</v>
       </c>
       <c r="D2" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="E2" s="32">
+        <v>0</v>
+      </c>
+      <c r="F2" s="32">
+        <v>0</v>
+      </c>
+      <c r="G2" s="49">
+        <v>0</v>
+      </c>
+      <c r="H2" s="49" t="s">
+        <v>410</v>
+      </c>
+      <c r="I2" s="49" t="s">
+        <v>410</v>
+      </c>
+      <c r="J2" s="49" t="s">
+        <v>410</v>
+      </c>
+      <c r="K2" s="49">
+        <v>0</v>
+      </c>
+      <c r="L2" s="49">
+        <v>0</v>
+      </c>
+      <c r="M2" s="32" t="s">
         <v>388</v>
       </c>
-      <c r="E2" s="32">
-        <v>0</v>
-      </c>
-      <c r="F2" s="32">
-        <v>0</v>
-      </c>
-      <c r="G2" s="49">
-        <v>0</v>
-      </c>
-      <c r="H2" s="49" t="s">
-        <v>411</v>
-      </c>
-      <c r="I2" s="49" t="s">
-        <v>411</v>
-      </c>
-      <c r="J2" s="49" t="s">
-        <v>411</v>
-      </c>
-      <c r="K2" s="49">
-        <v>0</v>
-      </c>
-      <c r="L2" s="49">
-        <v>0</v>
-      </c>
-      <c r="M2" s="32" t="s">
+      <c r="N2" s="32" t="s">
         <v>389</v>
-      </c>
-      <c r="N2" s="32" t="s">
-        <v>390</v>
       </c>
       <c r="O2" s="32">
         <v>300</v>
       </c>
       <c r="P2" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B3" s="39"/>
       <c r="C3" s="26">
         <v>12</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E3" s="26">
         <v>0</v>
@@ -9175,13 +9185,13 @@
         <v>0</v>
       </c>
       <c r="H3" s="50" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I3" s="50" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J3" s="50" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="K3" s="50">
         <v>0</v>
@@ -9190,80 +9200,80 @@
         <v>0</v>
       </c>
       <c r="M3" s="26" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="N3" s="26" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="O3" s="26">
         <v>400</v>
       </c>
       <c r="P3" s="26" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="32" t="s">
+        <v>393</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>386</v>
+      </c>
+      <c r="C4" s="32">
+        <v>0</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>387</v>
+      </c>
+      <c r="E4" s="32">
+        <v>0</v>
+      </c>
+      <c r="F4" s="32">
+        <v>1</v>
+      </c>
+      <c r="G4" s="49">
+        <v>1</v>
+      </c>
+      <c r="H4" s="49" t="s">
+        <v>411</v>
+      </c>
+      <c r="I4" s="49" t="s">
+        <v>411</v>
+      </c>
+      <c r="J4" s="49" t="s">
+        <v>419</v>
+      </c>
+      <c r="K4" s="49">
+        <v>0</v>
+      </c>
+      <c r="L4" s="49">
+        <v>0</v>
+      </c>
+      <c r="M4" s="32" t="s">
+        <v>392</v>
+      </c>
+      <c r="N4" s="32" t="s">
         <v>394</v>
       </c>
-      <c r="B4" s="32" t="s">
-        <v>387</v>
-      </c>
-      <c r="C4" s="32">
-        <v>0</v>
-      </c>
-      <c r="D4" s="32" t="s">
-        <v>388</v>
-      </c>
-      <c r="E4" s="32">
-        <v>0</v>
-      </c>
-      <c r="F4" s="32">
-        <v>1</v>
-      </c>
-      <c r="G4" s="49">
-        <v>1</v>
-      </c>
-      <c r="H4" s="49" t="s">
-        <v>412</v>
-      </c>
-      <c r="I4" s="49" t="s">
-        <v>412</v>
-      </c>
-      <c r="J4" s="49" t="s">
-        <v>420</v>
-      </c>
-      <c r="K4" s="49">
-        <v>0</v>
-      </c>
-      <c r="L4" s="49">
-        <v>0</v>
-      </c>
-      <c r="M4" s="32" t="s">
-        <v>393</v>
-      </c>
-      <c r="N4" s="32" t="s">
+      <c r="O4" s="32" t="s">
         <v>395</v>
       </c>
-      <c r="O4" s="32" t="s">
-        <v>396</v>
-      </c>
       <c r="P4" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
+        <v>396</v>
+      </c>
+      <c r="B5" s="26" t="s">
         <v>397</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>398</v>
       </c>
       <c r="C5" s="26">
         <v>20</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E5" s="26">
         <v>0</v>
@@ -9272,48 +9282,48 @@
         <v>1</v>
       </c>
       <c r="G5" s="50" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="H5" s="50" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="I5" s="50" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="J5" s="50" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="K5" s="50" t="s">
+        <v>423</v>
+      </c>
+      <c r="L5" s="50" t="s">
         <v>424</v>
       </c>
-      <c r="L5" s="50" t="s">
-        <v>425</v>
-      </c>
       <c r="M5" s="26" t="s">
+        <v>398</v>
+      </c>
+      <c r="N5" s="26" t="s">
+        <v>389</v>
+      </c>
+      <c r="O5" s="26" t="s">
         <v>399</v>
       </c>
-      <c r="N5" s="26" t="s">
+      <c r="P5" s="26" t="s">
         <v>390</v>
-      </c>
-      <c r="O5" s="26" t="s">
-        <v>400</v>
-      </c>
-      <c r="P5" s="26" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="32" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C6" s="32">
         <v>10</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E6" s="32">
         <v>0</v>
@@ -9325,13 +9335,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="49" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="I6" s="49" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="J6" s="49" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="K6" s="49">
         <v>0</v>
@@ -9340,30 +9350,30 @@
         <v>0</v>
       </c>
       <c r="M6" s="32" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="N6" s="32" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="O6" s="32">
         <v>500</v>
       </c>
       <c r="P6" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
+        <v>401</v>
+      </c>
+      <c r="B7" s="26" t="s">
         <v>402</v>
       </c>
-      <c r="B7" s="26" t="s">
-        <v>403</v>
-      </c>
       <c r="C7" s="26">
         <v>0</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E7" s="26">
         <v>1</v>
@@ -9372,132 +9382,132 @@
         <v>2</v>
       </c>
       <c r="G7" s="50" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="H7" s="50" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="I7" s="50" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="J7" s="50" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="K7" s="50" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="L7" s="50" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="M7" s="26" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="N7" s="26" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="O7" s="26" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="P7" s="26" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="32" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B8" s="32" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C8" s="32">
         <v>4</v>
       </c>
       <c r="D8" s="32" t="s">
+        <v>405</v>
+      </c>
+      <c r="E8" s="32">
+        <v>0</v>
+      </c>
+      <c r="F8" s="32">
+        <v>1</v>
+      </c>
+      <c r="G8" s="49">
+        <v>0</v>
+      </c>
+      <c r="H8" s="49" t="s">
+        <v>411</v>
+      </c>
+      <c r="I8" s="49" t="s">
+        <v>417</v>
+      </c>
+      <c r="J8" s="49" t="s">
+        <v>412</v>
+      </c>
+      <c r="K8" s="49">
+        <v>0</v>
+      </c>
+      <c r="L8" s="49">
+        <v>0</v>
+      </c>
+      <c r="M8" s="32" t="s">
+        <v>392</v>
+      </c>
+      <c r="N8" s="32" t="s">
         <v>406</v>
       </c>
-      <c r="E8" s="32">
-        <v>0</v>
-      </c>
-      <c r="F8" s="32">
-        <v>1</v>
-      </c>
-      <c r="G8" s="49">
-        <v>0</v>
-      </c>
-      <c r="H8" s="49" t="s">
-        <v>412</v>
-      </c>
-      <c r="I8" s="49" t="s">
-        <v>418</v>
-      </c>
-      <c r="J8" s="49" t="s">
-        <v>413</v>
-      </c>
-      <c r="K8" s="49">
-        <v>0</v>
-      </c>
-      <c r="L8" s="49">
-        <v>0</v>
-      </c>
-      <c r="M8" s="32" t="s">
-        <v>393</v>
-      </c>
-      <c r="N8" s="32" t="s">
-        <v>407</v>
-      </c>
       <c r="O8" s="32" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="P8" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B9" s="39"/>
       <c r="C9" s="26">
         <v>24</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E9" s="26">
         <v>0</v>
       </c>
       <c r="F9" s="50" t="s">
+        <v>410</v>
+      </c>
+      <c r="G9" s="50" t="s">
         <v>411</v>
       </c>
-      <c r="G9" s="50" t="s">
-        <v>412</v>
-      </c>
       <c r="H9" s="50" t="s">
+        <v>414</v>
+      </c>
+      <c r="I9" s="50" t="s">
+        <v>419</v>
+      </c>
+      <c r="J9" s="50" t="s">
+        <v>422</v>
+      </c>
+      <c r="K9" s="50" t="s">
         <v>415</v>
       </c>
-      <c r="I9" s="50" t="s">
-        <v>420</v>
-      </c>
-      <c r="J9" s="50" t="s">
-        <v>423</v>
-      </c>
-      <c r="K9" s="50" t="s">
-        <v>416</v>
-      </c>
       <c r="L9" s="50" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="M9" s="26" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="N9" s="26">
         <v>999</v>
       </c>
       <c r="O9" s="26" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P9" s="26" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
   </sheetData>
@@ -9520,7 +9530,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="112" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B1" s="112"/>
       <c r="C1" s="51"/>
@@ -9556,7 +9566,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B8" s="14"/>
     </row>
@@ -9565,7 +9575,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>589</v>
+        <v>581</v>
       </c>
       <c r="B10" s="14"/>
     </row>
@@ -9580,55 +9590,55 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="B14" s="14"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>571</v>
+        <v>563</v>
       </c>
       <c r="B15" s="14"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="B16" s="14"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
       <c r="B17" s="14"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="B18" s="14"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="B19" s="14"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="B20" s="14"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>586</v>
+        <v>578</v>
       </c>
       <c r="B21" s="14"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>587</v>
+        <v>579</v>
       </c>
       <c r="B22" s="14"/>
     </row>
@@ -9870,7 +9880,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B3">
         <v>16</v>
@@ -9933,7 +9943,7 @@
         <v>76</v>
       </c>
       <c r="V3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="W3" cm="1">
         <f t="array" aca="1" ref="W3" ca="1">INDEX(Caliber!B2:'Caliber'!C10,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B2:'Caliber'!B10,0),2)</f>
@@ -9947,7 +9957,7 @@
         <v>92</v>
       </c>
       <c r="Z3" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
@@ -10824,7 +10834,7 @@
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B15">
         <v>8</v>
@@ -10903,7 +10913,7 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="B16">
         <v>12</v>
@@ -10990,7 +11000,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{941F1AF2-A8AA-477B-ABE7-7C87546ECF29}">
-  <dimension ref="A1:Z16"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" customWidth="1"/>
@@ -11176,7 +11186,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B3">
         <v>18</v>
@@ -11413,7 +11423,7 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B6">
         <v>23</v>
@@ -11650,7 +11660,7 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B9">
         <v>21</v>
@@ -11713,7 +11723,7 @@
         <v>7</v>
       </c>
       <c r="V9" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="W9" s="10" cm="1">
         <f t="array" aca="1" ref="W9" ca="1">INDEX(Caliber!B2:'Caliber'!C11,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B2:'Caliber'!B11,0),2)</f>
@@ -11724,7 +11734,7 @@
         <v>0.35</v>
       </c>
       <c r="Y9" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
@@ -12124,7 +12134,7 @@
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B15">
         <v>22</v>
@@ -12198,12 +12208,12 @@
         <v>0</v>
       </c>
       <c r="Y15" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>541</v>
+        <v>533</v>
       </c>
       <c r="B16">
         <v>19</v>
@@ -12277,6 +12287,85 @@
         <v>0.1</v>
       </c>
       <c r="Y16" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>584</v>
+      </c>
+      <c r="B17">
+        <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>80</v>
+      </c>
+      <c r="G17">
+        <v>115</v>
+      </c>
+      <c r="H17">
+        <v>25</v>
+      </c>
+      <c r="I17">
+        <v>15</v>
+      </c>
+      <c r="J17">
+        <v>25</v>
+      </c>
+      <c r="K17">
+        <v>30</v>
+      </c>
+      <c r="L17">
+        <v>40</v>
+      </c>
+      <c r="M17">
+        <v>20</v>
+      </c>
+      <c r="N17">
+        <v>6</v>
+      </c>
+      <c r="O17">
+        <v>9</v>
+      </c>
+      <c r="P17">
+        <v>4</v>
+      </c>
+      <c r="Q17">
+        <v>20</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>5</v>
+      </c>
+      <c r="T17">
+        <v>1</v>
+      </c>
+      <c r="U17">
+        <v>10</v>
+      </c>
+      <c r="V17" t="s">
+        <v>14</v>
+      </c>
+      <c r="W17" s="10">
+        <f>INDEX(Caliber!B2:'Caliber'!C9,MATCH(V16,Caliber!B2:'Caliber'!B9,0),2)</f>
+        <v>35</v>
+      </c>
+      <c r="X17" s="10">
+        <f>INDEX(Caliber!C2:'Caliber'!D9,MATCH(V16,Caliber!B2:'Caliber'!B9,0),2)</f>
+        <v>0.1</v>
+      </c>
+      <c r="Y17" t="s">
         <v>115</v>
       </c>
     </row>
@@ -13803,7 +13892,7 @@
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B19">
         <v>23</v>
@@ -14377,7 +14466,7 @@
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B26">
         <v>30</v>
@@ -14459,7 +14548,7 @@
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B27">
         <v>32</v>
@@ -14623,7 +14712,7 @@
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B29">
         <v>30</v>
@@ -14635,7 +14724,7 @@
         <v>76</v>
       </c>
       <c r="E29" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="F29" t="b">
         <v>1</v>
@@ -14705,7 +14794,7 @@
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B30">
         <v>24</v>
@@ -16591,7 +16680,7 @@
     </row>
     <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B53">
         <v>21</v>
@@ -16673,7 +16762,7 @@
     </row>
     <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B54">
         <v>19</v>
@@ -16755,7 +16844,7 @@
     </row>
     <row r="55" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>548</v>
+        <v>540</v>
       </c>
       <c r="B55">
         <v>31</v>
@@ -16767,7 +16856,7 @@
         <v>76</v>
       </c>
       <c r="E55" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
       <c r="F55" t="b">
         <v>1</v>
@@ -16832,7 +16921,7 @@
         <v>0.3</v>
       </c>
       <c r="Z55" t="s">
-        <v>547</v>
+        <v>539</v>
       </c>
     </row>
     <row r="56" spans="1:26" x14ac:dyDescent="0.25">
@@ -17952,7 +18041,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
       <c r="B14">
         <v>35</v>
@@ -18018,7 +18107,7 @@
         <v>76</v>
       </c>
       <c r="W14" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="X14">
         <f>INDEX(Caliber!B13:'Caliber'!C24,MATCH(W14,Caliber!B13:'Caliber'!B24,0),2)</f>
@@ -18032,12 +18121,12 @@
         <v>178</v>
       </c>
       <c r="AA14" t="s">
-        <v>556</v>
+        <v>548</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>557</v>
+        <v>549</v>
       </c>
       <c r="B15">
         <v>37</v>
@@ -18103,7 +18192,7 @@
         <v>76</v>
       </c>
       <c r="W15" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="X15">
         <f>INDEX(Caliber!B13:'Caliber'!C24,MATCH(W15,Caliber!B13:'Caliber'!B24,0),2)</f>
@@ -18117,7 +18206,7 @@
         <v>178</v>
       </c>
       <c r="AA15" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
@@ -18566,7 +18655,7 @@
         <v>160</v>
       </c>
       <c r="AB3" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.25">
@@ -18655,7 +18744,7 @@
         <v>178</v>
       </c>
       <c r="AB4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
@@ -18744,7 +18833,7 @@
         <v>178</v>
       </c>
       <c r="AB5" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
@@ -19194,7 +19283,7 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B11">
         <v>24</v>
@@ -19278,7 +19367,7 @@
         <v>178</v>
       </c>
       <c r="AB11" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
   </sheetData>
@@ -19377,7 +19466,7 @@
         <v>73</v>
       </c>
       <c r="T1" s="19" t="s">
-        <v>591</v>
+        <v>583</v>
       </c>
       <c r="U1" s="19" t="s">
         <v>86</v>
@@ -20001,7 +20090,7 @@
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B9">
         <v>24</v>
@@ -20070,7 +20159,7 @@
         <v>15</v>
       </c>
       <c r="X9" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="Y9" cm="1">
         <f t="array" aca="1" ref="Y9" ca="1">INDEX(Caliber!B2:'Caliber'!C11,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B2:'Caliber'!B11,0),2)</f>
@@ -20081,12 +20170,12 @@
         <v>0.35</v>
       </c>
       <c r="AA9" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>568</v>
+        <v>560</v>
       </c>
       <c r="B10">
         <v>78</v>
@@ -20171,7 +20260,7 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>572</v>
+        <v>564</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -20256,7 +20345,7 @@
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>573</v>
+        <v>565</v>
       </c>
       <c r="B12">
         <v>39</v>
@@ -20336,12 +20425,12 @@
         <v>0.4</v>
       </c>
       <c r="AA12" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>574</v>
+        <v>566</v>
       </c>
       <c r="B13">
         <v>30</v>
@@ -20421,12 +20510,12 @@
         <v>0.4</v>
       </c>
       <c r="AA13" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>575</v>
+        <v>567</v>
       </c>
       <c r="B14">
         <v>48</v>
@@ -20506,12 +20595,12 @@
         <v>0.4</v>
       </c>
       <c r="AA14" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="B15">
         <v>47</v>
@@ -21227,7 +21316,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="B8">
         <v>30</v>
@@ -21293,7 +21382,7 @@
         <v>76</v>
       </c>
       <c r="W8" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="X8" cm="1">
         <f t="array" aca="1" ref="X8" ca="1">INDEX(Caliber!B35:'Caliber'!C45,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B45,0),2)</f>
@@ -21307,7 +21396,7 @@
         <v>82</v>
       </c>
       <c r="AA8" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
@@ -21408,7 +21497,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
M26 MASS as standalone weapon
Made M26 MASS function as standalone shotgun.
updated strings of MASS.
Updated listOrder of armor and manufacturing items to appear in correct order.
Renamed AKs-74u (SOPMOD) to AKs-74u (TACMOD) as it doesn't use SOPMOD parts.
Added more items to itemDelete.rul
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0A0205-2037-4FC2-AC0B-AE48166BA516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBB55DE-F400-4331-9138-8FD5483E3CAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="735" windowWidth="19440" windowHeight="15000" firstSheet="7" activeTab="12" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="28680" yWindow="735" windowWidth="19440" windowHeight="15000" firstSheet="4" activeTab="5" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1787" uniqueCount="596">
   <si>
     <t>Name</t>
   </si>
@@ -1971,6 +1971,9 @@
   <si>
     <t>1/2 Recruit cost
 + 10000</t>
+  </si>
+  <si>
+    <t>M26 MASS</t>
   </si>
 </sst>
 </file>
@@ -2902,13 +2905,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3767,8 +3770,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AEDA3547-9A13-4490-8F2C-86A75C183266}" name="Table1" displayName="Table1" ref="A1:AB11" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6">
-  <autoFilter ref="A1:AB11" xr:uid="{AEDA3547-9A13-4490-8F2C-86A75C183266}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AEDA3547-9A13-4490-8F2C-86A75C183266}" name="Table1" displayName="Table1" ref="A1:AB12" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6">
+  <autoFilter ref="A1:AB12" xr:uid="{AEDA3547-9A13-4490-8F2C-86A75C183266}"/>
   <tableColumns count="28">
     <tableColumn id="1" xr3:uid="{FDEE9766-F3A6-4F13-BA12-421285A2A455}" name="Name"/>
     <tableColumn id="2" xr3:uid="{D410D561-60F9-4F73-9A13-43B6913A0690}" name="weight"/>
@@ -8150,8 +8153,8 @@
     </row>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="100"/>
-      <c r="B7" s="103"/>
-      <c r="C7" s="103"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="101"/>
       <c r="D7" s="59" t="s">
         <v>348</v>
       </c>
@@ -8164,7 +8167,7 @@
       <c r="G7" s="59" t="s">
         <v>588</v>
       </c>
-      <c r="H7" s="103"/>
+      <c r="H7" s="101"/>
     </row>
     <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="100"/>
@@ -8210,8 +8213,8 @@
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="100"/>
-      <c r="B10" s="103"/>
-      <c r="C10" s="103"/>
+      <c r="B10" s="101"/>
+      <c r="C10" s="101"/>
       <c r="D10" s="59" t="s">
         <v>348</v>
       </c>
@@ -8224,7 +8227,7 @@
       <c r="G10" s="59" t="s">
         <v>486</v>
       </c>
-      <c r="H10" s="103"/>
+      <c r="H10" s="101"/>
     </row>
     <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="100"/>
@@ -8330,8 +8333,8 @@
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="100"/>
-      <c r="B16" s="103"/>
-      <c r="C16" s="103"/>
+      <c r="B16" s="101"/>
+      <c r="C16" s="101"/>
       <c r="D16" s="59" t="s">
         <v>348</v>
       </c>
@@ -8344,7 +8347,7 @@
       <c r="G16" s="59" t="s">
         <v>577</v>
       </c>
-      <c r="H16" s="103"/>
+      <c r="H16" s="101"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="100"/>
@@ -8390,8 +8393,8 @@
     </row>
     <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="100"/>
-      <c r="B19" s="103"/>
-      <c r="C19" s="103"/>
+      <c r="B19" s="101"/>
+      <c r="C19" s="101"/>
       <c r="D19" s="59" t="s">
         <v>348</v>
       </c>
@@ -8404,7 +8407,7 @@
       <c r="G19" s="59" t="s">
         <v>536</v>
       </c>
-      <c r="H19" s="103"/>
+      <c r="H19" s="101"/>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="100"/>
@@ -8464,7 +8467,7 @@
       <c r="G22" s="60" t="s">
         <v>367</v>
       </c>
-      <c r="H22" s="101"/>
+      <c r="H22" s="103"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="100"/>
@@ -8509,9 +8512,9 @@
       <c r="H24" s="100"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="101"/>
-      <c r="B25" s="101"/>
-      <c r="C25" s="101"/>
+      <c r="A25" s="103"/>
+      <c r="B25" s="103"/>
+      <c r="C25" s="103"/>
       <c r="D25" s="47" t="s">
         <v>348</v>
       </c>
@@ -8524,7 +8527,7 @@
       <c r="G25" s="47" t="s">
         <v>470</v>
       </c>
-      <c r="H25" s="101"/>
+      <c r="H25" s="103"/>
     </row>
     <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="102" t="s">
@@ -8612,8 +8615,8 @@
     </row>
     <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="100"/>
-      <c r="B31" s="103"/>
-      <c r="C31" s="103"/>
+      <c r="B31" s="101"/>
+      <c r="C31" s="101"/>
       <c r="D31" s="59" t="s">
         <v>348</v>
       </c>
@@ -8626,7 +8629,7 @@
       <c r="G31" s="78" t="s">
         <v>590</v>
       </c>
-      <c r="H31" s="103"/>
+      <c r="H31" s="101"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="100"/>
@@ -8971,9 +8974,9 @@
       <c r="H48" s="100"/>
     </row>
     <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="101"/>
-      <c r="B49" s="101"/>
-      <c r="C49" s="101"/>
+      <c r="A49" s="103"/>
+      <c r="B49" s="103"/>
+      <c r="C49" s="103"/>
       <c r="D49" s="47" t="s">
         <v>348</v>
       </c>
@@ -8986,19 +8989,38 @@
       <c r="G49" s="84" t="s">
         <v>504</v>
       </c>
-      <c r="H49" s="101"/>
+      <c r="H49" s="103"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="H44:H46"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="A2:A25"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="H2:H4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="H20:H22"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="H23:H25"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="B8:B10"/>
     <mergeCell ref="A26:A49"/>
     <mergeCell ref="B26:B28"/>
     <mergeCell ref="C26:C28"/>
@@ -9015,34 +9037,15 @@
     <mergeCell ref="B35:B37"/>
     <mergeCell ref="C35:C37"/>
     <mergeCell ref="H35:H37"/>
-    <mergeCell ref="A2:A25"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="H2:H4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="H20:H22"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="H23:H25"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="H17:H19"/>
-    <mergeCell ref="H5:H7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="H38:H40"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="H44:H46"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="H11:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -18369,7 +18372,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38CF758D-66BB-49AA-8233-CCB9E398E093}">
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -19334,7 +19337,7 @@
         <v>76</v>
       </c>
       <c r="R11">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="S11">
         <v>0</v>
@@ -19368,6 +19371,92 @@
       </c>
       <c r="AB11" t="s">
         <v>453</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>595</v>
+      </c>
+      <c r="B12">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12">
+        <v>18000</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12">
+        <v>115</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="s">
+        <v>76</v>
+      </c>
+      <c r="J12">
+        <v>30</v>
+      </c>
+      <c r="K12" t="s">
+        <v>76</v>
+      </c>
+      <c r="L12" t="s">
+        <v>76</v>
+      </c>
+      <c r="M12">
+        <v>50</v>
+      </c>
+      <c r="N12" t="s">
+        <v>76</v>
+      </c>
+      <c r="O12" t="s">
+        <v>76</v>
+      </c>
+      <c r="P12">
+        <v>7</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>76</v>
+      </c>
+      <c r="R12">
+        <v>30</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12" t="s">
+        <v>76</v>
+      </c>
+      <c r="U12">
+        <v>1</v>
+      </c>
+      <c r="V12" t="s">
+        <v>76</v>
+      </c>
+      <c r="W12" t="s">
+        <v>33</v>
+      </c>
+      <c r="X12" cm="1">
+        <f t="array" aca="1" ref="X12" ca="1">INDEX(Caliber!B26:'Caliber'!C33,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B26:'Caliber'!B33,0),2)</f>
+        <v>18</v>
+      </c>
+      <c r="Y12" cm="1">
+        <f t="array" aca="1" ref="Y12" ca="1">INDEX(Caliber!B26:'Caliber'!D33,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-2)),Caliber!B26:'Caliber'!B33,0),3)</f>
+        <v>10</v>
+      </c>
+      <c r="Z12" cm="1">
+        <f t="array" aca="1" ref="Z12" ca="1">INDEX(Caliber!B26:'Caliber'!F33,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-3)),Caliber!B26:'Caliber'!B33,0),5)</f>
+        <v>0</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PMC SAW unit sprite
PMC SAW unit armor type changed to kevlar+riot.
Organized file structure of PMC unit sprites.
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14387DD2-F104-4619-89B3-93391E157295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A65C2C-649F-4900-B7F5-667E3CCD0123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="735" windowWidth="19440" windowHeight="15000" firstSheet="6" activeTab="11" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="11" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1797" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1793" uniqueCount="595">
   <si>
     <t>Name</t>
   </si>
@@ -1918,19 +1918,7 @@
     <t>Remington 870/M3 (slug)/M3</t>
   </si>
   <si>
-    <t>Vector</t>
-  </si>
-  <si>
-    <t>Bushmaster ACR</t>
-  </si>
-  <si>
     <t>AR-18/G3/Spas 12 (Inc)</t>
-  </si>
-  <si>
-    <t>Modify gasmask terrorist sprite to show armor</t>
-  </si>
-  <si>
-    <t>MASS standalone</t>
   </si>
   <si>
     <t>Movement pen.</t>
@@ -1980,6 +1968,9 @@
   </si>
   <si>
     <t>Kriss Vector/ACR/Gold Deagle</t>
+  </si>
+  <si>
+    <t>Vest + Riot (35)</t>
   </si>
 </sst>
 </file>
@@ -2911,13 +2902,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -7311,10 +7302,10 @@
       <c r="M2" s="38"/>
       <c r="N2" s="38"/>
       <c r="O2" s="32" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="P2" s="32" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -8105,13 +8096,13 @@
         <v>348</v>
       </c>
       <c r="E4" s="60" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="F4" s="60" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="G4" s="60" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="H4" s="100"/>
     </row>
@@ -8127,13 +8118,13 @@
         <v>344</v>
       </c>
       <c r="E5" s="61" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="F5" s="61" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="G5" s="61" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H5" s="99" t="s">
         <v>346</v>
@@ -8153,14 +8144,14 @@
         <v>482</v>
       </c>
       <c r="G6" s="46" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H6" s="100"/>
     </row>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="100"/>
-      <c r="B7" s="101"/>
-      <c r="C7" s="101"/>
+      <c r="B7" s="103"/>
+      <c r="C7" s="103"/>
       <c r="D7" s="59" t="s">
         <v>348</v>
       </c>
@@ -8171,9 +8162,9 @@
         <v>481</v>
       </c>
       <c r="G7" s="59" t="s">
-        <v>587</v>
-      </c>
-      <c r="H7" s="101"/>
+        <v>583</v>
+      </c>
+      <c r="H7" s="103"/>
     </row>
     <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="100"/>
@@ -8219,8 +8210,8 @@
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="100"/>
-      <c r="B10" s="101"/>
-      <c r="C10" s="101"/>
+      <c r="B10" s="103"/>
+      <c r="C10" s="103"/>
       <c r="D10" s="59" t="s">
         <v>348</v>
       </c>
@@ -8233,7 +8224,7 @@
       <c r="G10" s="59" t="s">
         <v>485</v>
       </c>
-      <c r="H10" s="101"/>
+      <c r="H10" s="103"/>
     </row>
     <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="100"/>
@@ -8339,8 +8330,8 @@
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="100"/>
-      <c r="B16" s="101"/>
-      <c r="C16" s="101"/>
+      <c r="B16" s="103"/>
+      <c r="C16" s="103"/>
       <c r="D16" s="59" t="s">
         <v>348</v>
       </c>
@@ -8353,7 +8344,7 @@
       <c r="G16" s="59" t="s">
         <v>576</v>
       </c>
-      <c r="H16" s="101"/>
+      <c r="H16" s="103"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="100"/>
@@ -8399,8 +8390,8 @@
     </row>
     <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="100"/>
-      <c r="B19" s="101"/>
-      <c r="C19" s="101"/>
+      <c r="B19" s="103"/>
+      <c r="C19" s="103"/>
       <c r="D19" s="59" t="s">
         <v>348</v>
       </c>
@@ -8413,7 +8404,7 @@
       <c r="G19" s="59" t="s">
         <v>535</v>
       </c>
-      <c r="H19" s="101"/>
+      <c r="H19" s="103"/>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="100"/>
@@ -8473,7 +8464,7 @@
       <c r="G22" s="60" t="s">
         <v>367</v>
       </c>
-      <c r="H22" s="103"/>
+      <c r="H22" s="101"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="100"/>
@@ -8518,9 +8509,9 @@
       <c r="H24" s="100"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="103"/>
-      <c r="B25" s="103"/>
-      <c r="C25" s="103"/>
+      <c r="A25" s="101"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="101"/>
       <c r="D25" s="47" t="s">
         <v>348</v>
       </c>
@@ -8533,7 +8524,7 @@
       <c r="G25" s="47" t="s">
         <v>470</v>
       </c>
-      <c r="H25" s="103"/>
+      <c r="H25" s="101"/>
     </row>
     <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="102" t="s">
@@ -8621,21 +8612,21 @@
     </row>
     <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="100"/>
-      <c r="B31" s="101"/>
-      <c r="C31" s="101"/>
+      <c r="B31" s="103"/>
+      <c r="C31" s="103"/>
       <c r="D31" s="59" t="s">
         <v>348</v>
       </c>
       <c r="E31" s="78" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="F31" s="74" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="G31" s="78" t="s">
-        <v>588</v>
-      </c>
-      <c r="H31" s="101"/>
+        <v>584</v>
+      </c>
+      <c r="H31" s="103"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="100"/>
@@ -8898,7 +8889,7 @@
         <v>510</v>
       </c>
       <c r="H44" s="99" t="s">
-        <v>346</v>
+        <v>594</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8980,9 +8971,9 @@
       <c r="H48" s="100"/>
     </row>
     <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="103"/>
-      <c r="B49" s="103"/>
-      <c r="C49" s="103"/>
+      <c r="A49" s="101"/>
+      <c r="B49" s="101"/>
+      <c r="C49" s="101"/>
       <c r="D49" s="47" t="s">
         <v>348</v>
       </c>
@@ -8995,22 +8986,35 @@
       <c r="G49" s="84" t="s">
         <v>503</v>
       </c>
-      <c r="H49" s="103"/>
+      <c r="H49" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="H44:H46"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="A26:A49"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="H35:H37"/>
     <mergeCell ref="A2:A25"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C2:C4"/>
@@ -9027,31 +9031,18 @@
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="H5:H7"/>
     <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A26:A49"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="H35:H37"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="H44:H46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9583,9 +9574,6 @@
       <c r="B9" s="14"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>580</v>
-      </c>
       <c r="B10" s="14"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -9616,9 +9604,6 @@
       <c r="B16" s="14"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>581</v>
-      </c>
       <c r="B17" s="14"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -9640,15 +9625,9 @@
       <c r="B20" s="14"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>577</v>
-      </c>
       <c r="B21" s="14"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>578</v>
-      </c>
       <c r="B22" s="14"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -12301,7 +12280,7 @@
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="B17">
         <v>26</v>
@@ -16935,7 +16914,7 @@
     </row>
     <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="B56">
         <v>24</v>
@@ -19463,7 +19442,7 @@
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="B12">
         <v>8</v>
@@ -19643,7 +19622,7 @@
         <v>73</v>
       </c>
       <c r="T1" s="19" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="U1" s="19" t="s">
         <v>86</v>

</xml_diff>

<commit_message>
bomb defusal scoring and bombsites
Still need to make one more bomb site.
East EU terrains and 1 USA terrain is set up currently.
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A65C2C-649F-4900-B7F5-667E3CCD0123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F12E85-25D4-47A5-A532-E59E34312984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="11" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="9810" yWindow="2325" windowWidth="14400" windowHeight="11385" firstSheet="5" activeTab="13" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1793" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1797" uniqueCount="599">
   <si>
     <t>Name</t>
   </si>
@@ -1971,6 +1971,18 @@
   </si>
   <si>
     <t>Vest + Riot (35)</t>
+  </si>
+  <si>
+    <t>M79</t>
+  </si>
+  <si>
+    <t>FN2000</t>
+  </si>
+  <si>
+    <t>QLZ-87/QLU-11</t>
+  </si>
+  <si>
+    <t>Beretta 93R</t>
   </si>
 </sst>
 </file>
@@ -2902,13 +2914,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -8150,8 +8162,8 @@
     </row>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="100"/>
-      <c r="B7" s="103"/>
-      <c r="C7" s="103"/>
+      <c r="B7" s="101"/>
+      <c r="C7" s="101"/>
       <c r="D7" s="59" t="s">
         <v>348</v>
       </c>
@@ -8164,7 +8176,7 @@
       <c r="G7" s="59" t="s">
         <v>583</v>
       </c>
-      <c r="H7" s="103"/>
+      <c r="H7" s="101"/>
     </row>
     <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="100"/>
@@ -8210,8 +8222,8 @@
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="100"/>
-      <c r="B10" s="103"/>
-      <c r="C10" s="103"/>
+      <c r="B10" s="101"/>
+      <c r="C10" s="101"/>
       <c r="D10" s="59" t="s">
         <v>348</v>
       </c>
@@ -8224,7 +8236,7 @@
       <c r="G10" s="59" t="s">
         <v>485</v>
       </c>
-      <c r="H10" s="103"/>
+      <c r="H10" s="101"/>
     </row>
     <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="100"/>
@@ -8330,8 +8342,8 @@
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="100"/>
-      <c r="B16" s="103"/>
-      <c r="C16" s="103"/>
+      <c r="B16" s="101"/>
+      <c r="C16" s="101"/>
       <c r="D16" s="59" t="s">
         <v>348</v>
       </c>
@@ -8344,7 +8356,7 @@
       <c r="G16" s="59" t="s">
         <v>576</v>
       </c>
-      <c r="H16" s="103"/>
+      <c r="H16" s="101"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="100"/>
@@ -8390,8 +8402,8 @@
     </row>
     <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="100"/>
-      <c r="B19" s="103"/>
-      <c r="C19" s="103"/>
+      <c r="B19" s="101"/>
+      <c r="C19" s="101"/>
       <c r="D19" s="59" t="s">
         <v>348</v>
       </c>
@@ -8404,7 +8416,7 @@
       <c r="G19" s="59" t="s">
         <v>535</v>
       </c>
-      <c r="H19" s="103"/>
+      <c r="H19" s="101"/>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="100"/>
@@ -8464,7 +8476,7 @@
       <c r="G22" s="60" t="s">
         <v>367</v>
       </c>
-      <c r="H22" s="101"/>
+      <c r="H22" s="103"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="100"/>
@@ -8509,9 +8521,9 @@
       <c r="H24" s="100"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="101"/>
-      <c r="B25" s="101"/>
-      <c r="C25" s="101"/>
+      <c r="A25" s="103"/>
+      <c r="B25" s="103"/>
+      <c r="C25" s="103"/>
       <c r="D25" s="47" t="s">
         <v>348</v>
       </c>
@@ -8524,7 +8536,7 @@
       <c r="G25" s="47" t="s">
         <v>470</v>
       </c>
-      <c r="H25" s="101"/>
+      <c r="H25" s="103"/>
     </row>
     <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="102" t="s">
@@ -8612,8 +8624,8 @@
     </row>
     <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="100"/>
-      <c r="B31" s="103"/>
-      <c r="C31" s="103"/>
+      <c r="B31" s="101"/>
+      <c r="C31" s="101"/>
       <c r="D31" s="59" t="s">
         <v>348</v>
       </c>
@@ -8626,7 +8638,7 @@
       <c r="G31" s="78" t="s">
         <v>584</v>
       </c>
-      <c r="H31" s="103"/>
+      <c r="H31" s="101"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="100"/>
@@ -8971,9 +8983,9 @@
       <c r="H48" s="100"/>
     </row>
     <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="101"/>
-      <c r="B49" s="101"/>
-      <c r="C49" s="101"/>
+      <c r="A49" s="103"/>
+      <c r="B49" s="103"/>
+      <c r="C49" s="103"/>
       <c r="D49" s="47" t="s">
         <v>348</v>
       </c>
@@ -8986,19 +8998,38 @@
       <c r="G49" s="84" t="s">
         <v>503</v>
       </c>
-      <c r="H49" s="101"/>
+      <c r="H49" s="103"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="H44:H46"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="A2:A25"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="H2:H4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="H20:H22"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="H23:H25"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="B8:B10"/>
     <mergeCell ref="A26:A49"/>
     <mergeCell ref="B26:B28"/>
     <mergeCell ref="C26:C28"/>
@@ -9015,34 +9046,15 @@
     <mergeCell ref="B35:B37"/>
     <mergeCell ref="C35:C37"/>
     <mergeCell ref="H35:H37"/>
-    <mergeCell ref="A2:A25"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="H2:H4"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="C5:C7"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="H20:H22"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="C23:C25"/>
-    <mergeCell ref="H23:H25"/>
-    <mergeCell ref="C17:C19"/>
-    <mergeCell ref="H17:H19"/>
-    <mergeCell ref="H5:H7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="H38:H40"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="H44:H46"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="H11:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9604,6 +9616,9 @@
       <c r="B16" s="14"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>597</v>
+      </c>
       <c r="B17" s="14"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -9625,12 +9640,21 @@
       <c r="B20" s="14"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>595</v>
+      </c>
       <c r="B21" s="14"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>596</v>
+      </c>
       <c r="B22" s="14"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>598</v>
+      </c>
       <c r="B23" s="14"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Ammo included in weapon categories + misc changes
Ammo included in weapon categories.
C4 ufopaedia added to language files.
Reordered ufopaedia + added listOrder sorting system (like WeaponsEquipment.rul).
Loaded ammo now defaults to highest capacity magazine.
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F12E85-25D4-47A5-A532-E59E34312984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{283A7799-5E07-4DA4-B491-B3E8F0445A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9810" yWindow="2325" windowWidth="14400" windowHeight="11385" firstSheet="5" activeTab="13" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1797" uniqueCount="599">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1799" uniqueCount="601">
   <si>
     <t>Name</t>
   </si>
@@ -1983,6 +1983,12 @@
   </si>
   <si>
     <t>Beretta 93R</t>
+  </si>
+  <si>
+    <t>Styer scout</t>
+  </si>
+  <si>
+    <t>EOD suit</t>
   </si>
 </sst>
 </file>
@@ -2914,13 +2920,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -8162,8 +8168,8 @@
     </row>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="100"/>
-      <c r="B7" s="101"/>
-      <c r="C7" s="101"/>
+      <c r="B7" s="103"/>
+      <c r="C7" s="103"/>
       <c r="D7" s="59" t="s">
         <v>348</v>
       </c>
@@ -8176,7 +8182,7 @@
       <c r="G7" s="59" t="s">
         <v>583</v>
       </c>
-      <c r="H7" s="101"/>
+      <c r="H7" s="103"/>
     </row>
     <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="100"/>
@@ -8222,8 +8228,8 @@
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="100"/>
-      <c r="B10" s="101"/>
-      <c r="C10" s="101"/>
+      <c r="B10" s="103"/>
+      <c r="C10" s="103"/>
       <c r="D10" s="59" t="s">
         <v>348</v>
       </c>
@@ -8236,7 +8242,7 @@
       <c r="G10" s="59" t="s">
         <v>485</v>
       </c>
-      <c r="H10" s="101"/>
+      <c r="H10" s="103"/>
     </row>
     <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="100"/>
@@ -8342,8 +8348,8 @@
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="100"/>
-      <c r="B16" s="101"/>
-      <c r="C16" s="101"/>
+      <c r="B16" s="103"/>
+      <c r="C16" s="103"/>
       <c r="D16" s="59" t="s">
         <v>348</v>
       </c>
@@ -8356,7 +8362,7 @@
       <c r="G16" s="59" t="s">
         <v>576</v>
       </c>
-      <c r="H16" s="101"/>
+      <c r="H16" s="103"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="100"/>
@@ -8402,8 +8408,8 @@
     </row>
     <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="100"/>
-      <c r="B19" s="101"/>
-      <c r="C19" s="101"/>
+      <c r="B19" s="103"/>
+      <c r="C19" s="103"/>
       <c r="D19" s="59" t="s">
         <v>348</v>
       </c>
@@ -8416,7 +8422,7 @@
       <c r="G19" s="59" t="s">
         <v>535</v>
       </c>
-      <c r="H19" s="101"/>
+      <c r="H19" s="103"/>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="100"/>
@@ -8476,7 +8482,7 @@
       <c r="G22" s="60" t="s">
         <v>367</v>
       </c>
-      <c r="H22" s="103"/>
+      <c r="H22" s="101"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="100"/>
@@ -8521,9 +8527,9 @@
       <c r="H24" s="100"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="103"/>
-      <c r="B25" s="103"/>
-      <c r="C25" s="103"/>
+      <c r="A25" s="101"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="101"/>
       <c r="D25" s="47" t="s">
         <v>348</v>
       </c>
@@ -8536,7 +8542,7 @@
       <c r="G25" s="47" t="s">
         <v>470</v>
       </c>
-      <c r="H25" s="103"/>
+      <c r="H25" s="101"/>
     </row>
     <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="102" t="s">
@@ -8624,8 +8630,8 @@
     </row>
     <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="100"/>
-      <c r="B31" s="101"/>
-      <c r="C31" s="101"/>
+      <c r="B31" s="103"/>
+      <c r="C31" s="103"/>
       <c r="D31" s="59" t="s">
         <v>348</v>
       </c>
@@ -8638,7 +8644,7 @@
       <c r="G31" s="78" t="s">
         <v>584</v>
       </c>
-      <c r="H31" s="101"/>
+      <c r="H31" s="103"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="100"/>
@@ -8983,9 +8989,9 @@
       <c r="H48" s="100"/>
     </row>
     <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="103"/>
-      <c r="B49" s="103"/>
-      <c r="C49" s="103"/>
+      <c r="A49" s="101"/>
+      <c r="B49" s="101"/>
+      <c r="C49" s="101"/>
       <c r="D49" s="47" t="s">
         <v>348</v>
       </c>
@@ -8998,22 +9004,35 @@
       <c r="G49" s="84" t="s">
         <v>503</v>
       </c>
-      <c r="H49" s="103"/>
+      <c r="H49" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="H44:H46"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="A26:A49"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="H35:H37"/>
     <mergeCell ref="A2:A25"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C2:C4"/>
@@ -9030,31 +9049,18 @@
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="H5:H7"/>
     <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A26:A49"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="H35:H37"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="H44:H46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9658,9 +9664,15 @@
       <c r="B23" s="14"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>599</v>
+      </c>
       <c r="B24" s="14"/>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>600</v>
+      </c>
       <c r="B25" s="14"/>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
10x 5.56 mag, Steyr scout acquisition
Moved dragunov in enemy weapon sets to later in the game.
Steyr scout acquisition added.
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37FB118-D426-4C25-827F-B208A28C96DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D1C437-2680-4BCB-A0F3-EA0B1A6B7E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="2" activeTab="4" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="4" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1809" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1810" uniqueCount="600">
   <si>
     <t>Name</t>
   </si>
@@ -1582,12 +1582,6 @@
     <t>M16 (Scoped)/SKS/M14 (Scoped)</t>
   </si>
   <si>
-    <t>SKS/Dragunov/SKS</t>
-  </si>
-  <si>
-    <t>FN FAL (scoped)/Dragunov/FN FAL (scoped)</t>
-  </si>
-  <si>
     <t>M82 Barret/M24 SWS/AWM</t>
   </si>
   <si>
@@ -1970,9 +1964,6 @@
     <t>Beretta 93R</t>
   </si>
   <si>
-    <t>Styer scout</t>
-  </si>
-  <si>
     <t>EOD suit</t>
   </si>
   <si>
@@ -1980,13 +1971,28 @@
   </si>
   <si>
     <t>Styer Scout</t>
+  </si>
+  <si>
+    <t>VSS/OSV 96/Dragunov</t>
+  </si>
+  <si>
+    <t>SKS/SKS/SKS</t>
+  </si>
+  <si>
+    <t>FN FAL (scoped)/FN FAL (scoped)/FN FAL (scoped)</t>
+  </si>
+  <si>
+    <t>SV-98</t>
+  </si>
+  <si>
+    <t>SSG 08</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2027,12 +2033,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="25">
@@ -2953,7 +2953,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4117,20 +4117,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6695E0F0-C0B0-45B8-AA00-1AE0F467FE87}">
   <dimension ref="A1:S49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.109375" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" customWidth="1"/>
-    <col min="5" max="5" width="14.88671875" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="14.88671875" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" customWidth="1"/>
-    <col min="9" max="9" width="131.88671875" customWidth="1"/>
-    <col min="12" max="12" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
+    <col min="9" max="9" width="131.85546875" customWidth="1"/>
+    <col min="12" max="12" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>17</v>
       </c>
@@ -4159,7 +4159,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="1" t="s">
         <v>8</v>
@@ -4187,7 +4187,7 @@
       <c r="P2" s="13"/>
       <c r="Q2" s="13"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" t="s">
         <v>10</v>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="M3" s="14"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" t="s">
         <v>95</v>
@@ -4229,7 +4229,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" t="s">
         <v>12</v>
@@ -4248,7 +4248,7 @@
       </c>
       <c r="M5" s="14"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" t="s">
         <v>16</v>
@@ -4271,7 +4271,7 @@
       <c r="P6" s="10"/>
       <c r="Q6" s="10"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" t="s">
         <v>15</v>
@@ -4290,7 +4290,7 @@
       </c>
       <c r="M7" s="14"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" t="s">
         <v>13</v>
@@ -4313,7 +4313,7 @@
       <c r="P8" s="10"/>
       <c r="Q8" s="10"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" t="s">
         <v>14</v>
@@ -4336,7 +4336,7 @@
       <c r="P9" s="11"/>
       <c r="Q9" s="11"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" t="s">
         <v>423</v>
@@ -4357,7 +4357,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="56"/>
       <c r="B11" t="s">
         <v>439</v>
@@ -4390,7 +4390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="55" t="s">
         <v>22</v>
       </c>
@@ -4434,7 +4434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="1" t="s">
         <v>18</v>
@@ -4470,7 +4470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" t="s">
         <v>19</v>
@@ -4503,7 +4503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" t="s">
         <v>120</v>
@@ -4536,7 +4536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" t="s">
         <v>23</v>
@@ -4569,7 +4569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" t="s">
         <v>25</v>
@@ -4602,7 +4602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" t="s">
         <v>26</v>
@@ -4635,7 +4635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" t="s">
         <v>27</v>
@@ -4668,7 +4668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" t="s">
         <v>28</v>
@@ -4701,7 +4701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
       <c r="B21" t="s">
         <v>30</v>
@@ -4734,7 +4734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" t="s">
         <v>29</v>
@@ -4752,7 +4752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" t="s">
         <v>31</v>
@@ -4791,10 +4791,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C24">
         <v>40</v>
@@ -4830,7 +4830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>32</v>
       </c>
@@ -4880,7 +4880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="1" t="s">
         <v>33</v>
@@ -4926,7 +4926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" t="s">
         <v>34</v>
@@ -4971,7 +4971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" t="s">
         <v>35</v>
@@ -5019,7 +5019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" t="s">
         <v>444</v>
@@ -5046,7 +5046,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" t="s">
         <v>447</v>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="S30" s="13"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
       <c r="B31" t="s">
         <v>37</v>
@@ -5134,7 +5134,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
       <c r="B32" t="s">
         <v>38</v>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="S32" s="10"/>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
       <c r="B33" t="s">
         <v>39</v>
@@ -5222,7 +5222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>40</v>
       </c>
@@ -5270,7 +5270,7 @@
       </c>
       <c r="S34" s="10"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="8"/>
       <c r="B35" s="1" t="s">
         <v>41</v>
@@ -5313,7 +5313,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
       <c r="B36" t="s">
         <v>43</v>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="S36" s="10"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
       <c r="B37" t="s">
         <v>45</v>
@@ -5398,7 +5398,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
       <c r="B38" t="s">
         <v>47</v>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="S38" s="10"/>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
       <c r="B39" t="s">
         <v>49</v>
@@ -5462,7 +5462,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
       <c r="B40" t="s">
         <v>50</v>
@@ -5483,7 +5483,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="9"/>
       <c r="B41" t="s">
         <v>51</v>
@@ -5504,7 +5504,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
       <c r="B42" t="s">
         <v>52</v>
@@ -5525,7 +5525,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
       <c r="B43" t="s">
         <v>53</v>
@@ -5546,10 +5546,10 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
       <c r="B44" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="C44">
         <v>95</v>
@@ -5567,13 +5567,13 @@
         <v>3</v>
       </c>
       <c r="I44" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45" s="9"/>
       <c r="B45" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C45">
         <v>40</v>
@@ -5591,13 +5591,13 @@
         <v>3</v>
       </c>
       <c r="I45" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46" s="9"/>
       <c r="B46" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C46">
         <v>40</v>
@@ -5618,10 +5618,10 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47" s="9"/>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A48" s="53" t="s">
         <v>446</v>
       </c>
@@ -5650,7 +5650,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="54"/>
       <c r="B49" s="14" t="s">
         <v>437</v>
@@ -5685,18 +5685,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BABADE2C-4009-4AB7-BED9-B450B00DFD85}">
   <dimension ref="A1:P32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" customWidth="1"/>
-    <col min="11" max="11" width="14.109375" customWidth="1"/>
-    <col min="12" max="12" width="10.44140625" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" customWidth="1"/>
+    <col min="11" max="11" width="14.140625" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" customWidth="1"/>
     <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="10.44140625" customWidth="1"/>
-    <col min="15" max="15" width="13.33203125" customWidth="1"/>
-    <col min="16" max="16" width="11.109375" customWidth="1"/>
+    <col min="14" max="14" width="10.42578125" customWidth="1"/>
+    <col min="15" max="15" width="13.28515625" customWidth="1"/>
+    <col min="16" max="16" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="91" t="s">
         <v>236</v>
       </c>
@@ -5732,7 +5732,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="92"/>
       <c r="B2" s="20" t="s">
         <v>245</v>
@@ -5768,7 +5768,7 @@
       <c r="O2" s="92"/>
       <c r="P2" s="92"/>
     </row>
-    <row r="3" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
         <v>254</v>
       </c>
@@ -5808,7 +5808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="32" t="s">
         <v>257</v>
       </c>
@@ -5852,7 +5852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
         <v>258</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="32" t="s">
         <v>259</v>
       </c>
@@ -5948,7 +5948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>260</v>
       </c>
@@ -5996,7 +5996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="32" t="s">
         <v>262</v>
       </c>
@@ -6044,7 +6044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>263</v>
       </c>
@@ -6092,7 +6092,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="32" t="s">
         <v>266</v>
       </c>
@@ -6140,7 +6140,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="32" t="s">
         <v>291</v>
       </c>
@@ -6190,7 +6190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="32" t="s">
         <v>292</v>
       </c>
@@ -6240,7 +6240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="33" t="s">
         <v>267</v>
       </c>
@@ -6280,7 +6280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="33" t="s">
         <v>269</v>
       </c>
@@ -6324,7 +6324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33" t="s">
         <v>270</v>
       </c>
@@ -6372,7 +6372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33" t="s">
         <v>271</v>
       </c>
@@ -6420,7 +6420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33" t="s">
         <v>272</v>
       </c>
@@ -6468,7 +6468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33" t="s">
         <v>273</v>
       </c>
@@ -6516,7 +6516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33" t="s">
         <v>274</v>
       </c>
@@ -6564,7 +6564,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="33" t="s">
         <v>275</v>
       </c>
@@ -6612,7 +6612,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="33" t="s">
         <v>276</v>
       </c>
@@ -6654,7 +6654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="33" t="s">
         <v>278</v>
       </c>
@@ -6700,7 +6700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="33" t="s">
         <v>279</v>
       </c>
@@ -6750,7 +6750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="33" t="s">
         <v>280</v>
       </c>
@@ -6800,7 +6800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="33" t="s">
         <v>281</v>
       </c>
@@ -6850,7 +6850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="33" t="s">
         <v>283</v>
       </c>
@@ -6900,7 +6900,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="33" t="s">
         <v>284</v>
       </c>
@@ -6950,7 +6950,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="33" t="s">
         <v>286</v>
       </c>
@@ -7000,7 +7000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="26" t="s">
         <v>287</v>
       </c>
@@ -7050,7 +7050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="32" t="s">
         <v>288</v>
       </c>
@@ -7100,7 +7100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="26" t="s">
         <v>289</v>
       </c>
@@ -7150,7 +7150,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="33" t="s">
         <v>290</v>
       </c>
@@ -7219,16 +7219,16 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C092F238-A859-4DAF-9B24-82DF047DC2BE}">
   <dimension ref="A1:P18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
-    <col min="13" max="13" width="11.88671875" customWidth="1"/>
-    <col min="15" max="15" width="16.33203125" customWidth="1"/>
-    <col min="16" max="16" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="11.85546875" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>334</v>
       </c>
@@ -7278,7 +7278,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
         <v>335</v>
       </c>
@@ -7318,13 +7318,13 @@
       <c r="M2" s="38"/>
       <c r="N2" s="38"/>
       <c r="O2" s="32" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="P2" s="32" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="96" t="s">
         <v>336</v>
       </c>
@@ -7370,7 +7370,7 @@
       <c r="O3" s="39"/>
       <c r="P3" s="39"/>
     </row>
-    <row r="4" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="97"/>
       <c r="B4" s="32" t="s">
         <v>299</v>
@@ -7414,7 +7414,7 @@
       <c r="O4" s="38"/>
       <c r="P4" s="38"/>
     </row>
-    <row r="5" spans="1:16" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="97"/>
       <c r="B5" s="26" t="s">
         <v>315</v>
@@ -7458,7 +7458,7 @@
       <c r="O5" s="39"/>
       <c r="P5" s="39"/>
     </row>
-    <row r="6" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="97"/>
       <c r="B6" s="32" t="s">
         <v>317</v>
@@ -7502,7 +7502,7 @@
       <c r="O6" s="38"/>
       <c r="P6" s="38"/>
     </row>
-    <row r="7" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="97"/>
       <c r="B7" s="26" t="s">
         <v>319</v>
@@ -7546,7 +7546,7 @@
       <c r="O7" s="39"/>
       <c r="P7" s="39"/>
     </row>
-    <row r="8" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="97"/>
       <c r="B8" s="32" t="s">
         <v>321</v>
@@ -7590,7 +7590,7 @@
       <c r="O8" s="38"/>
       <c r="P8" s="38"/>
     </row>
-    <row r="9" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="97"/>
       <c r="B9" s="26" t="s">
         <v>323</v>
@@ -7634,7 +7634,7 @@
       <c r="O9" s="39"/>
       <c r="P9" s="39"/>
     </row>
-    <row r="10" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="98"/>
       <c r="B10" s="32" t="s">
         <v>324</v>
@@ -7678,7 +7678,7 @@
       <c r="O10" s="38"/>
       <c r="P10" s="38"/>
     </row>
-    <row r="11" spans="1:16" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="96" t="s">
         <v>337</v>
       </c>
@@ -7700,7 +7700,7 @@
       <c r="O11" s="39"/>
       <c r="P11" s="39"/>
     </row>
-    <row r="12" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="97"/>
       <c r="B12" s="32" t="s">
         <v>299</v>
@@ -7744,7 +7744,7 @@
       <c r="O12" s="38"/>
       <c r="P12" s="38"/>
     </row>
-    <row r="13" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="97"/>
       <c r="B13" s="26" t="s">
         <v>329</v>
@@ -7788,7 +7788,7 @@
       <c r="O13" s="39"/>
       <c r="P13" s="39"/>
     </row>
-    <row r="14" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="97"/>
       <c r="B14" s="32" t="s">
         <v>317</v>
@@ -7832,7 +7832,7 @@
       <c r="O14" s="38"/>
       <c r="P14" s="38"/>
     </row>
-    <row r="15" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="97"/>
       <c r="B15" s="26" t="s">
         <v>287</v>
@@ -7876,7 +7876,7 @@
       <c r="O15" s="39"/>
       <c r="P15" s="39"/>
     </row>
-    <row r="16" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="97"/>
       <c r="B16" s="32" t="s">
         <v>321</v>
@@ -7920,7 +7920,7 @@
       <c r="O16" s="38"/>
       <c r="P16" s="38"/>
     </row>
-    <row r="17" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="97"/>
       <c r="B17" s="26" t="s">
         <v>315</v>
@@ -7964,7 +7964,7 @@
       <c r="O17" s="39"/>
       <c r="P17" s="39"/>
     </row>
-    <row r="18" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="98"/>
       <c r="B18" s="32" t="s">
         <v>324</v>
@@ -8020,19 +8020,19 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D21C18DE-CCD8-4ABA-9B3B-CCD73CA8C93E}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16.5546875" customWidth="1"/>
-    <col min="5" max="5" width="43.109375" customWidth="1"/>
-    <col min="6" max="6" width="53.6640625" customWidth="1"/>
-    <col min="7" max="7" width="46.33203125" customWidth="1"/>
-    <col min="8" max="8" width="14.44140625" customWidth="1"/>
-    <col min="9" max="9" width="30.109375" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
+    <col min="5" max="5" width="43.140625" customWidth="1"/>
+    <col min="6" max="6" width="53.7109375" customWidth="1"/>
+    <col min="7" max="7" width="46.28515625" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="44" t="s">
         <v>334</v>
       </c>
@@ -8059,7 +8059,7 @@
       </c>
       <c r="I1" s="48"/>
     </row>
-    <row r="2" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="102" t="s">
         <v>384</v>
       </c>
@@ -8073,10 +8073,10 @@
         <v>344</v>
       </c>
       <c r="E2" s="45" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="F2" s="45" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="G2" s="45" t="s">
         <v>345</v>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="I2" s="62"/>
     </row>
-    <row r="3" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="100"/>
       <c r="B3" s="100"/>
       <c r="C3" s="100"/>
@@ -8094,17 +8094,17 @@
         <v>347</v>
       </c>
       <c r="E3" s="46" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="F3" s="46" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="G3" s="46" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="H3" s="100"/>
     </row>
-    <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="100"/>
       <c r="B4" s="100"/>
       <c r="C4" s="100"/>
@@ -8112,17 +8112,17 @@
         <v>348</v>
       </c>
       <c r="E4" s="60" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="F4" s="60" t="s">
+        <v>584</v>
+      </c>
+      <c r="G4" s="60" t="s">
         <v>586</v>
       </c>
-      <c r="G4" s="60" t="s">
-        <v>588</v>
-      </c>
       <c r="H4" s="100"/>
     </row>
-    <row r="5" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="100"/>
       <c r="B5" s="99" t="s">
         <v>299</v>
@@ -8134,19 +8134,19 @@
         <v>344</v>
       </c>
       <c r="E5" s="61" t="s">
+        <v>573</v>
+      </c>
+      <c r="F5" s="61" t="s">
+        <v>574</v>
+      </c>
+      <c r="G5" s="61" t="s">
         <v>575</v>
-      </c>
-      <c r="F5" s="61" t="s">
-        <v>576</v>
-      </c>
-      <c r="G5" s="61" t="s">
-        <v>577</v>
       </c>
       <c r="H5" s="99" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="100"/>
       <c r="B6" s="100"/>
       <c r="C6" s="100"/>
@@ -8154,17 +8154,17 @@
         <v>347</v>
       </c>
       <c r="E6" s="46" t="s">
+        <v>475</v>
+      </c>
+      <c r="F6" s="46" t="s">
         <v>477</v>
       </c>
-      <c r="F6" s="46" t="s">
-        <v>479</v>
-      </c>
       <c r="G6" s="46" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H6" s="100"/>
     </row>
-    <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="100"/>
       <c r="B7" s="101"/>
       <c r="C7" s="101"/>
@@ -8172,17 +8172,17 @@
         <v>348</v>
       </c>
       <c r="E7" s="59" t="s">
+        <v>474</v>
+      </c>
+      <c r="F7" s="59" t="s">
         <v>476</v>
       </c>
-      <c r="F7" s="59" t="s">
-        <v>478</v>
-      </c>
       <c r="G7" s="59" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="H7" s="101"/>
     </row>
-    <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="100"/>
       <c r="B8" s="99" t="s">
         <v>352</v>
@@ -8194,10 +8194,10 @@
         <v>344</v>
       </c>
       <c r="E8" s="61" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="F8" s="61" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="G8" s="61" t="s">
         <v>220</v>
@@ -8206,7 +8206,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="100"/>
       <c r="B9" s="100"/>
       <c r="C9" s="100"/>
@@ -8217,14 +8217,14 @@
         <v>350</v>
       </c>
       <c r="F9" s="46" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="G9" s="46" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="H9" s="100"/>
     </row>
-    <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="100"/>
       <c r="B10" s="101"/>
       <c r="C10" s="101"/>
@@ -8235,14 +8235,14 @@
         <v>351</v>
       </c>
       <c r="F10" s="59" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="G10" s="59" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="H10" s="101"/>
     </row>
-    <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="100"/>
       <c r="B11" s="99" t="s">
         <v>354</v>
@@ -8260,13 +8260,13 @@
         <v>457</v>
       </c>
       <c r="G11" s="61" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="H11" s="99" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="100"/>
       <c r="B12" s="100"/>
       <c r="C12" s="100"/>
@@ -8277,14 +8277,14 @@
         <v>203</v>
       </c>
       <c r="F12" s="46" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="G12" s="46" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="H12" s="100"/>
     </row>
-    <row r="13" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="100"/>
       <c r="B13" s="100"/>
       <c r="C13" s="100"/>
@@ -8302,7 +8302,7 @@
       </c>
       <c r="H13" s="100"/>
     </row>
-    <row r="14" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="100"/>
       <c r="B14" s="99" t="s">
         <v>357</v>
@@ -8326,7 +8326,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="100"/>
       <c r="B15" s="100"/>
       <c r="C15" s="100"/>
@@ -8340,11 +8340,11 @@
         <v>460</v>
       </c>
       <c r="G15" s="46" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="H15" s="100"/>
     </row>
-    <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="100"/>
       <c r="B16" s="101"/>
       <c r="C16" s="101"/>
@@ -8352,17 +8352,17 @@
         <v>348</v>
       </c>
       <c r="E16" s="59" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="F16" s="59" t="s">
         <v>459</v>
       </c>
       <c r="G16" s="59" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H16" s="101"/>
     </row>
-    <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="100"/>
       <c r="B17" s="99" t="s">
         <v>358</v>
@@ -8386,7 +8386,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="100"/>
       <c r="B18" s="100"/>
       <c r="C18" s="100"/>
@@ -8394,17 +8394,17 @@
         <v>347</v>
       </c>
       <c r="E18" s="46" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="F18" s="46" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="G18" s="46" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="H18" s="100"/>
     </row>
-    <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="100"/>
       <c r="B19" s="101"/>
       <c r="C19" s="101"/>
@@ -8415,14 +8415,14 @@
         <v>458</v>
       </c>
       <c r="F19" s="59" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="G19" s="59" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="H19" s="101"/>
     </row>
-    <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="100"/>
       <c r="B20" s="99" t="s">
         <v>359</v>
@@ -8437,7 +8437,7 @@
         <v>360</v>
       </c>
       <c r="F20" s="61" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="G20" s="61" t="s">
         <v>361</v>
@@ -8446,7 +8446,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="100"/>
       <c r="B21" s="100"/>
       <c r="C21" s="100"/>
@@ -8454,17 +8454,17 @@
         <v>347</v>
       </c>
       <c r="E21" s="46" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="F21" s="46" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="G21" s="46" t="s">
         <v>361</v>
       </c>
       <c r="H21" s="100"/>
     </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="100"/>
       <c r="B22" s="100"/>
       <c r="C22" s="100"/>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="H22" s="103"/>
     </row>
-    <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="100"/>
       <c r="B23" s="99" t="s">
         <v>365</v>
@@ -8497,16 +8497,16 @@
         <v>148</v>
       </c>
       <c r="F23" s="61" t="s">
-        <v>465</v>
+        <v>596</v>
       </c>
       <c r="G23" s="61" t="s">
-        <v>469</v>
+        <v>595</v>
       </c>
       <c r="H23" s="102" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="100"/>
       <c r="B24" s="100"/>
       <c r="C24" s="100"/>
@@ -8514,17 +8514,17 @@
         <v>347</v>
       </c>
       <c r="E24" s="65" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="F24" s="46" t="s">
+        <v>597</v>
+      </c>
+      <c r="G24" s="46" t="s">
         <v>466</v>
       </c>
-      <c r="G24" s="46" t="s">
-        <v>468</v>
-      </c>
       <c r="H24" s="100"/>
     </row>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="103"/>
       <c r="B25" s="103"/>
       <c r="C25" s="103"/>
@@ -8532,17 +8532,17 @@
         <v>348</v>
       </c>
       <c r="E25" s="47" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="F25" s="47" t="s">
         <v>464</v>
       </c>
       <c r="G25" s="47" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="H25" s="103"/>
     </row>
-    <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="102" t="s">
         <v>337</v>
       </c>
@@ -8560,7 +8560,7 @@
       <c r="G26" s="106"/>
       <c r="H26" s="107"/>
     </row>
-    <row r="27" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="100"/>
       <c r="B27" s="100"/>
       <c r="C27" s="100"/>
@@ -8572,7 +8572,7 @@
       <c r="G27" s="106"/>
       <c r="H27" s="108"/>
     </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="100"/>
       <c r="B28" s="100"/>
       <c r="C28" s="100"/>
@@ -8584,7 +8584,7 @@
       <c r="G28" s="111"/>
       <c r="H28" s="108"/>
     </row>
-    <row r="29" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="100"/>
       <c r="B29" s="99" t="s">
         <v>299</v>
@@ -8596,10 +8596,10 @@
         <v>344</v>
       </c>
       <c r="E29" s="75" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="F29" s="64" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="G29" s="76" t="s">
         <v>451</v>
@@ -8608,7 +8608,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="100"/>
       <c r="B30" s="100"/>
       <c r="C30" s="100"/>
@@ -8616,17 +8616,17 @@
         <v>347</v>
       </c>
       <c r="E30" s="79" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="F30" s="71" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="G30" s="77" t="s">
         <v>209</v>
       </c>
       <c r="H30" s="100"/>
     </row>
-    <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="100"/>
       <c r="B31" s="101"/>
       <c r="C31" s="101"/>
@@ -8634,17 +8634,17 @@
         <v>348</v>
       </c>
       <c r="E31" s="78" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="F31" s="74" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="G31" s="78" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H31" s="101"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="100"/>
       <c r="B32" s="100" t="s">
         <v>352</v>
@@ -8656,19 +8656,19 @@
         <v>344</v>
       </c>
       <c r="E32" s="73" t="s">
+        <v>509</v>
+      </c>
+      <c r="F32" s="80" t="s">
+        <v>510</v>
+      </c>
+      <c r="G32" s="73" t="s">
         <v>511</v>
-      </c>
-      <c r="F32" s="80" t="s">
-        <v>512</v>
-      </c>
-      <c r="G32" s="73" t="s">
-        <v>513</v>
       </c>
       <c r="H32" s="100" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="100"/>
       <c r="B33" s="100"/>
       <c r="C33" s="100"/>
@@ -8676,17 +8676,17 @@
         <v>347</v>
       </c>
       <c r="E33" s="79" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="F33" s="71" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="G33" s="79" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="H33" s="100"/>
     </row>
-    <row r="34" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="100"/>
       <c r="B34" s="100"/>
       <c r="C34" s="100"/>
@@ -8694,17 +8694,17 @@
         <v>348</v>
       </c>
       <c r="E34" s="67" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="F34" s="81" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="G34" s="67" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="H34" s="100"/>
     </row>
-    <row r="35" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="100"/>
       <c r="B35" s="99" t="s">
         <v>354</v>
@@ -8716,19 +8716,19 @@
         <v>344</v>
       </c>
       <c r="E35" s="75" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="F35" s="75" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="G35" s="75" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="H35" s="99" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="100"/>
       <c r="B36" s="100"/>
       <c r="C36" s="100"/>
@@ -8736,17 +8736,17 @@
         <v>347</v>
       </c>
       <c r="E36" s="79" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="F36" s="79" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="G36" s="79" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="H36" s="100"/>
     </row>
-    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="100"/>
       <c r="B37" s="100"/>
       <c r="C37" s="100"/>
@@ -8754,17 +8754,17 @@
         <v>348</v>
       </c>
       <c r="E37" s="90" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="F37" s="90" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="G37" s="90" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="H37" s="100"/>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="100"/>
       <c r="B38" s="99" t="s">
         <v>357</v>
@@ -8776,19 +8776,19 @@
         <v>344</v>
       </c>
       <c r="E38" s="63" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="F38" s="85" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="G38" s="63" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="H38" s="99" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="100"/>
       <c r="B39" s="100"/>
       <c r="C39" s="100"/>
@@ -8796,17 +8796,17 @@
         <v>347</v>
       </c>
       <c r="E39" s="79" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="F39" s="71" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="G39" s="79" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="H39" s="100"/>
     </row>
-    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="100"/>
       <c r="B40" s="100"/>
       <c r="C40" s="100"/>
@@ -8814,17 +8814,17 @@
         <v>348</v>
       </c>
       <c r="E40" s="67" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="F40" s="81" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="G40" s="67" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="H40" s="100"/>
     </row>
-    <row r="41" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="100"/>
       <c r="B41" s="99" t="s">
         <v>358</v>
@@ -8836,19 +8836,19 @@
         <v>344</v>
       </c>
       <c r="E41" s="86" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F41" s="80" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="G41" s="86" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="H41" s="99" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="100"/>
       <c r="B42" s="100"/>
       <c r="C42" s="100"/>
@@ -8856,17 +8856,17 @@
         <v>347</v>
       </c>
       <c r="E42" s="87" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="F42" s="88" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="G42" s="87" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="H42" s="100"/>
     </row>
-    <row r="43" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="100"/>
       <c r="B43" s="100"/>
       <c r="C43" s="100"/>
@@ -8874,17 +8874,17 @@
         <v>348</v>
       </c>
       <c r="E43" s="67" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="F43" s="89" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="G43" s="67" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="H43" s="100"/>
     </row>
-    <row r="44" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="100"/>
       <c r="B44" s="99" t="s">
         <v>359</v>
@@ -8896,19 +8896,19 @@
         <v>344</v>
       </c>
       <c r="E44" s="68" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="F44" s="82" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="G44" s="68" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="H44" s="99" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="100"/>
       <c r="B45" s="100"/>
       <c r="C45" s="100"/>
@@ -8916,17 +8916,17 @@
         <v>347</v>
       </c>
       <c r="E45" s="69" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="F45" s="69" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="G45" s="69" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H45" s="100"/>
     </row>
-    <row r="46" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="100"/>
       <c r="B46" s="100"/>
       <c r="C46" s="100"/>
@@ -8934,17 +8934,17 @@
         <v>348</v>
       </c>
       <c r="E46" s="67" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="F46" s="81" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="G46" s="67" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="H46" s="100"/>
     </row>
-    <row r="47" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="100"/>
       <c r="B47" s="99" t="s">
         <v>365</v>
@@ -8959,16 +8959,16 @@
         <v>158</v>
       </c>
       <c r="F47" s="80" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="G47" s="63" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="H47" s="99" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="100"/>
       <c r="B48" s="100"/>
       <c r="C48" s="100"/>
@@ -8976,17 +8976,17 @@
         <v>347</v>
       </c>
       <c r="E48" s="70" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="F48" s="83" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="G48" s="70" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="H48" s="100"/>
     </row>
-    <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="103"/>
       <c r="B49" s="103"/>
       <c r="C49" s="103"/>
@@ -8994,13 +8994,13 @@
         <v>348</v>
       </c>
       <c r="E49" s="84" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="F49" s="72" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="G49" s="84" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="H49" s="103"/>
     </row>
@@ -9067,20 +9067,20 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC8BAE7-4B1E-4B8C-8AF9-C5EAA5B2467F}">
   <dimension ref="A1:P9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
-    <col min="2" max="2" width="8.44140625" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" customWidth="1"/>
-    <col min="9" max="9" width="13.88671875" customWidth="1"/>
-    <col min="11" max="11" width="15.109375" customWidth="1"/>
-    <col min="12" max="12" width="10.88671875" customWidth="1"/>
-    <col min="14" max="14" width="13.5546875" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" customWidth="1"/>
+    <col min="11" max="11" width="15.140625" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" customWidth="1"/>
     <col min="15" max="15" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="20" t="s">
         <v>236</v>
       </c>
@@ -9130,7 +9130,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
         <v>382</v>
       </c>
@@ -9180,7 +9180,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
         <v>388</v>
       </c>
@@ -9228,7 +9228,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="32" t="s">
         <v>390</v>
       </c>
@@ -9278,7 +9278,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
         <v>393</v>
       </c>
@@ -9328,7 +9328,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="32" t="s">
         <v>397</v>
       </c>
@@ -9378,7 +9378,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
         <v>398</v>
       </c>
@@ -9428,7 +9428,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="32" t="s">
         <v>401</v>
       </c>
@@ -9478,7 +9478,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
         <v>404</v>
       </c>
@@ -9538,13 +9538,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6FEC12-ED84-4F38-9B1C-DC3BDC099D3A}">
   <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.88671875" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" customWidth="1"/>
+    <col min="1" max="1" width="40.85546875" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="112" t="s">
         <v>436</v>
       </c>
@@ -9553,154 +9553,157 @@
       <c r="D1" s="51"/>
       <c r="E1" s="51"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="112"/>
       <c r="B2" s="112"/>
       <c r="C2" s="51"/>
       <c r="D2" s="51"/>
       <c r="E2" s="51"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="112"/>
       <c r="B3" s="112"/>
       <c r="C3" s="51"/>
       <c r="D3" s="51"/>
       <c r="E3" s="51"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="52"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="14"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B6" s="14"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B7" s="14"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>453</v>
       </c>
       <c r="B8" s="14"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B9" s="14"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" s="14"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" s="14"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" s="14"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B13" s="14"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>520</v>
+      </c>
+      <c r="B14" s="14"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>555</v>
+      </c>
+      <c r="B15" s="14"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>522</v>
       </c>
-      <c r="B14" s="14"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>557</v>
-      </c>
-      <c r="B15" s="14"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="B16" s="14"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>590</v>
+      </c>
+      <c r="B17" s="14"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>523</v>
+      </c>
+      <c r="B18" s="14"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>524</v>
       </c>
-      <c r="B16" s="14"/>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="B19" s="14"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>538</v>
+      </c>
+      <c r="B20" s="14"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>588</v>
+      </c>
+      <c r="B21" s="14"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>589</v>
+      </c>
+      <c r="B22" s="14"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>591</v>
+      </c>
+      <c r="B23" s="14"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B24" s="14"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>592</v>
       </c>
-      <c r="B17" s="14"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>525</v>
-      </c>
-      <c r="B18" s="14"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>526</v>
-      </c>
-      <c r="B19" s="14"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>540</v>
-      </c>
-      <c r="B20" s="14"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>590</v>
-      </c>
-      <c r="B21" s="14"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>591</v>
-      </c>
-      <c r="B22" s="14"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>593</v>
-      </c>
-      <c r="B23" s="14"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>594</v>
-      </c>
-      <c r="B24" s="14"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>595</v>
-      </c>
       <c r="B25" s="14"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>598</v>
+      </c>
       <c r="B26" s="14"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>599</v>
+      </c>
       <c r="B27" s="14"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B28" s="14"/>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B29" s="14"/>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B30" s="14"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B31" s="14"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B32" s="14"/>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="14"/>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="14"/>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="14"/>
     </row>
   </sheetData>
@@ -9714,34 +9717,34 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6FC119D-A7BC-46FE-BE1D-3900F19AB624}">
   <dimension ref="A1:Z16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="3" max="3" width="6.5546875" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10.88671875" customWidth="1"/>
-    <col min="9" max="10" width="9.33203125" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" customWidth="1"/>
-    <col min="12" max="13" width="10.109375" customWidth="1"/>
+    <col min="8" max="8" width="10.85546875" customWidth="1"/>
+    <col min="9" max="10" width="9.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" customWidth="1"/>
+    <col min="12" max="13" width="10.140625" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="16" width="12.44140625" customWidth="1"/>
-    <col min="17" max="17" width="12.33203125" customWidth="1"/>
+    <col min="15" max="16" width="12.42578125" customWidth="1"/>
+    <col min="17" max="17" width="12.28515625" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="19" width="14.109375" customWidth="1"/>
-    <col min="20" max="20" width="12.44140625" customWidth="1"/>
-    <col min="21" max="21" width="12.33203125" customWidth="1"/>
-    <col min="22" max="22" width="13.44140625" customWidth="1"/>
-    <col min="23" max="23" width="8.88671875" customWidth="1"/>
-    <col min="24" max="24" width="13.5546875" customWidth="1"/>
-    <col min="25" max="25" width="11.5546875" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" customWidth="1"/>
+    <col min="20" max="20" width="12.42578125" customWidth="1"/>
+    <col min="21" max="21" width="12.28515625" customWidth="1"/>
+    <col min="22" max="22" width="13.42578125" customWidth="1"/>
+    <col min="23" max="23" width="8.85546875" customWidth="1"/>
+    <col min="24" max="24" width="13.5703125" customWidth="1"/>
+    <col min="25" max="25" width="11.5703125" customWidth="1"/>
     <col min="26" max="26" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -9821,7 +9824,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -9900,7 +9903,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>422</v>
       </c>
@@ -9982,7 +9985,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>99</v>
       </c>
@@ -10061,7 +10064,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -10143,7 +10146,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>102</v>
       </c>
@@ -10222,7 +10225,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>97</v>
       </c>
@@ -10301,7 +10304,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>93</v>
       </c>
@@ -10380,7 +10383,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -10459,7 +10462,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>89</v>
       </c>
@@ -10538,7 +10541,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>77</v>
       </c>
@@ -10617,7 +10620,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -10696,7 +10699,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>103</v>
       </c>
@@ -10775,7 +10778,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>83</v>
       </c>
@@ -10854,7 +10857,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>456</v>
       </c>
@@ -10933,9 +10936,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="B16">
         <v>12</v>
@@ -11023,31 +11026,31 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{941F1AF2-A8AA-477B-ABE7-7C87546ECF29}">
   <dimension ref="A1:Z17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10.88671875" customWidth="1"/>
-    <col min="9" max="10" width="9.33203125" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" customWidth="1"/>
-    <col min="12" max="13" width="10.109375" customWidth="1"/>
+    <col min="8" max="8" width="10.85546875" customWidth="1"/>
+    <col min="9" max="10" width="9.28515625" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" customWidth="1"/>
+    <col min="12" max="13" width="10.140625" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="16" width="12.44140625" customWidth="1"/>
-    <col min="17" max="17" width="12.33203125" customWidth="1"/>
+    <col min="15" max="16" width="12.42578125" customWidth="1"/>
+    <col min="17" max="17" width="12.28515625" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="19" width="14.109375" customWidth="1"/>
-    <col min="20" max="20" width="12.44140625" customWidth="1"/>
-    <col min="21" max="21" width="12.33203125" customWidth="1"/>
-    <col min="22" max="22" width="13.5546875" customWidth="1"/>
-    <col min="24" max="24" width="13.5546875" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" customWidth="1"/>
+    <col min="20" max="20" width="12.42578125" customWidth="1"/>
+    <col min="21" max="21" width="12.28515625" customWidth="1"/>
+    <col min="22" max="22" width="13.5703125" customWidth="1"/>
+    <col min="24" max="24" width="13.5703125" customWidth="1"/>
     <col min="25" max="25" width="12" customWidth="1"/>
-    <col min="26" max="26" width="26.5546875" customWidth="1"/>
+    <col min="26" max="26" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -11127,7 +11130,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>107</v>
       </c>
@@ -11206,7 +11209,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>433</v>
       </c>
@@ -11285,7 +11288,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="57" t="s">
         <v>108</v>
       </c>
@@ -11364,7 +11367,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>110</v>
       </c>
@@ -11443,7 +11446,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>452</v>
       </c>
@@ -11522,7 +11525,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>116</v>
       </c>
@@ -11601,7 +11604,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>106</v>
       </c>
@@ -11680,7 +11683,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>442</v>
       </c>
@@ -11759,7 +11762,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -11838,7 +11841,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>112</v>
       </c>
@@ -11917,7 +11920,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>111</v>
       </c>
@@ -11996,7 +11999,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>114</v>
       </c>
@@ -12075,7 +12078,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>104</v>
       </c>
@@ -12154,7 +12157,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>428</v>
       </c>
@@ -12233,9 +12236,9 @@
         <v>429</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="B16">
         <v>19</v>
@@ -12312,9 +12315,9 @@
         <v>115</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B17">
         <v>26</v>
@@ -12402,34 +12405,34 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E308052D-1B88-4699-843E-12AA607B59B8}">
   <dimension ref="A1:AA57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.109375" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" customWidth="1"/>
-    <col min="10" max="11" width="9.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" customWidth="1"/>
-    <col min="13" max="13" width="10.109375" customWidth="1"/>
-    <col min="14" max="14" width="11.33203125" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="11" width="9.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="10.140625" customWidth="1"/>
+    <col min="14" max="14" width="11.28515625" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.44140625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" customWidth="1"/>
+    <col min="16" max="17" width="12.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12.28515625" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="14.109375" customWidth="1"/>
-    <col min="21" max="21" width="12.44140625" customWidth="1"/>
-    <col min="22" max="22" width="12.33203125" customWidth="1"/>
-    <col min="23" max="23" width="14.44140625" customWidth="1"/>
-    <col min="24" max="24" width="11.5546875" customWidth="1"/>
-    <col min="25" max="25" width="13.5546875" customWidth="1"/>
-    <col min="26" max="26" width="11.6640625" customWidth="1"/>
-    <col min="27" max="27" width="29.6640625" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" customWidth="1"/>
+    <col min="21" max="21" width="12.42578125" customWidth="1"/>
+    <col min="22" max="22" width="12.28515625" customWidth="1"/>
+    <col min="23" max="23" width="14.42578125" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" customWidth="1"/>
+    <col min="25" max="25" width="13.5703125" customWidth="1"/>
+    <col min="26" max="26" width="11.7109375" customWidth="1"/>
+    <col min="27" max="27" width="29.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -12512,7 +12515,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>205</v>
       </c>
@@ -12594,7 +12597,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>133</v>
       </c>
@@ -12676,7 +12679,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>135</v>
       </c>
@@ -12758,7 +12761,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>136</v>
       </c>
@@ -12840,7 +12843,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>138</v>
       </c>
@@ -12922,9 +12925,9 @@
         <v>137</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B7">
         <v>31</v>
@@ -12936,7 +12939,7 @@
         <v>76</v>
       </c>
       <c r="E7" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -13001,10 +13004,10 @@
         <v>0.3</v>
       </c>
       <c r="Z7" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -13086,7 +13089,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>454</v>
       </c>
@@ -13168,7 +13171,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>455</v>
       </c>
@@ -13250,7 +13253,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>201</v>
       </c>
@@ -13332,7 +13335,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>202</v>
       </c>
@@ -13414,7 +13417,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>139</v>
       </c>
@@ -13499,7 +13502,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>141</v>
       </c>
@@ -13584,7 +13587,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>206</v>
       </c>
@@ -13666,7 +13669,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>147</v>
       </c>
@@ -13748,7 +13751,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>189</v>
       </c>
@@ -13830,7 +13833,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>197</v>
       </c>
@@ -13912,7 +13915,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>207</v>
       </c>
@@ -13994,7 +13997,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>142</v>
       </c>
@@ -14076,7 +14079,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>143</v>
       </c>
@@ -14158,7 +14161,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>427</v>
       </c>
@@ -14240,7 +14243,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>144</v>
       </c>
@@ -14322,7 +14325,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>146</v>
       </c>
@@ -14404,7 +14407,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>174</v>
       </c>
@@ -14486,7 +14489,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>145</v>
       </c>
@@ -14568,7 +14571,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>209</v>
       </c>
@@ -14650,7 +14653,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>210</v>
       </c>
@@ -14732,7 +14735,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>434</v>
       </c>
@@ -14814,7 +14817,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>435</v>
       </c>
@@ -14896,7 +14899,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>200</v>
       </c>
@@ -14978,7 +14981,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>431</v>
       </c>
@@ -15060,7 +15063,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>430</v>
       </c>
@@ -15142,7 +15145,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>130</v>
       </c>
@@ -15224,7 +15227,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>132</v>
       </c>
@@ -15306,7 +15309,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>172</v>
       </c>
@@ -15388,7 +15391,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>131</v>
       </c>
@@ -15470,7 +15473,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>169</v>
       </c>
@@ -15552,7 +15555,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>171</v>
       </c>
@@ -15634,7 +15637,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>173</v>
       </c>
@@ -15716,7 +15719,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>170</v>
       </c>
@@ -15798,7 +15801,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>204</v>
       </c>
@@ -15880,7 +15883,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>193</v>
       </c>
@@ -15962,7 +15965,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>195</v>
       </c>
@@ -16044,7 +16047,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>194</v>
       </c>
@@ -16126,7 +16129,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>190</v>
       </c>
@@ -16208,7 +16211,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>192</v>
       </c>
@@ -16290,7 +16293,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>191</v>
       </c>
@@ -16372,7 +16375,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>198</v>
       </c>
@@ -16454,7 +16457,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>199</v>
       </c>
@@ -16536,7 +16539,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>121</v>
       </c>
@@ -16618,7 +16621,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>122</v>
       </c>
@@ -16700,7 +16703,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>126</v>
       </c>
@@ -16782,7 +16785,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>127</v>
       </c>
@@ -16864,7 +16867,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>128</v>
       </c>
@@ -16946,9 +16949,9 @@
         <v>117</v>
       </c>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B56">
         <v>24</v>
@@ -17028,7 +17031,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X57" t="e" cm="1">
         <f t="array" aca="1" ref="X57" ca="1">INDEX(Caliber!B13:'Caliber'!C23,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -17049,34 +17052,34 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E52ABDA0-E560-473A-9AD2-E06CBFB7AB92}">
   <dimension ref="A1:AA30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.109375" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="3" max="3" width="6.88671875" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="3" max="3" width="6.85546875" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" customWidth="1"/>
-    <col min="7" max="7" width="16.109375" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" customWidth="1"/>
-    <col min="10" max="11" width="9.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" customWidth="1"/>
-    <col min="13" max="14" width="10.109375" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="11" width="9.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="14" width="10.140625" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.44140625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" customWidth="1"/>
+    <col min="16" max="17" width="12.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12.28515625" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="14.109375" customWidth="1"/>
-    <col min="21" max="21" width="12.44140625" customWidth="1"/>
-    <col min="22" max="22" width="12.33203125" customWidth="1"/>
-    <col min="23" max="23" width="19.109375" customWidth="1"/>
-    <col min="25" max="25" width="13.5546875" customWidth="1"/>
-    <col min="26" max="26" width="11.6640625" customWidth="1"/>
-    <col min="27" max="27" width="21.33203125" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" customWidth="1"/>
+    <col min="21" max="21" width="12.42578125" customWidth="1"/>
+    <col min="22" max="22" width="12.28515625" customWidth="1"/>
+    <col min="23" max="23" width="19.140625" customWidth="1"/>
+    <col min="25" max="25" width="13.5703125" customWidth="1"/>
+    <col min="26" max="26" width="11.7109375" customWidth="1"/>
+    <col min="27" max="27" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -17159,7 +17162,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>148</v>
       </c>
@@ -17241,7 +17244,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>151</v>
       </c>
@@ -17323,7 +17326,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>155</v>
       </c>
@@ -17405,7 +17408,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>154</v>
       </c>
@@ -17487,7 +17490,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>157</v>
       </c>
@@ -17569,7 +17572,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>158</v>
       </c>
@@ -17651,7 +17654,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>159</v>
       </c>
@@ -17733,7 +17736,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>161</v>
       </c>
@@ -17815,7 +17818,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>162</v>
       </c>
@@ -17897,7 +17900,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>163</v>
       </c>
@@ -17979,7 +17982,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>164</v>
       </c>
@@ -18061,7 +18064,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>165</v>
       </c>
@@ -18143,9 +18146,9 @@
         <v>166</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="B14">
         <v>35</v>
@@ -18211,7 +18214,7 @@
         <v>76</v>
       </c>
       <c r="W14" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="X14">
         <f>INDEX(Caliber!B13:'Caliber'!C24,MATCH(W14,Caliber!B13:'Caliber'!B24,0),2)</f>
@@ -18225,12 +18228,12 @@
         <v>178</v>
       </c>
       <c r="AA14" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="B15">
         <v>37</v>
@@ -18296,7 +18299,7 @@
         <v>76</v>
       </c>
       <c r="W15" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="X15">
         <f>INDEX(Caliber!B13:'Caliber'!C24,MATCH(W15,Caliber!B13:'Caliber'!B24,0),2)</f>
@@ -18310,12 +18313,12 @@
         <v>178</v>
       </c>
       <c r="AA15" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A16" s="113" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="B16">
         <v>24</v>
@@ -18395,7 +18398,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="17" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X17" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W17,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18405,7 +18408,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="18" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="18" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X18" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W18,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18415,7 +18418,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="19" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="19" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X19" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W19,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18425,7 +18428,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="20" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="20" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X20" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W20,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18435,7 +18438,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="21" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="21" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X21" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W21,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18445,7 +18448,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="22" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="22" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X22" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W22,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18455,7 +18458,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="23" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="23" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X23" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W23,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18465,7 +18468,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="24" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="24" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X24" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W24,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18475,7 +18478,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="25" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="25" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X25" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W25,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18485,7 +18488,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="26" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="26" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X26" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W26,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18495,7 +18498,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="27" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="27" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X27" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W27,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18505,7 +18508,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="28" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="28" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X28" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W28,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18515,7 +18518,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="29" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="29" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X29" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W29,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18525,7 +18528,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="30" spans="24:25" x14ac:dyDescent="0.3">
+    <row r="30" spans="24:25" x14ac:dyDescent="0.25">
       <c r="X30" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W30,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18547,34 +18550,34 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38CF758D-66BB-49AA-8233-CCB9E398E093}">
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" customWidth="1"/>
-    <col min="10" max="11" width="9.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" customWidth="1"/>
-    <col min="13" max="13" width="10.109375" customWidth="1"/>
-    <col min="14" max="14" width="11.44140625" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="11" width="9.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="10.140625" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.44140625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" customWidth="1"/>
+    <col min="16" max="17" width="12.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12.28515625" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="14.109375" customWidth="1"/>
-    <col min="21" max="21" width="12.44140625" customWidth="1"/>
-    <col min="22" max="22" width="12.33203125" customWidth="1"/>
-    <col min="23" max="23" width="15.6640625" customWidth="1"/>
-    <col min="24" max="24" width="11.5546875" customWidth="1"/>
-    <col min="25" max="25" width="11.33203125" customWidth="1"/>
-    <col min="26" max="26" width="13.5546875" customWidth="1"/>
-    <col min="27" max="27" width="11.6640625" customWidth="1"/>
-    <col min="28" max="28" width="25.109375" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" customWidth="1"/>
+    <col min="21" max="21" width="12.42578125" customWidth="1"/>
+    <col min="22" max="22" width="12.28515625" customWidth="1"/>
+    <col min="23" max="23" width="15.7109375" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" customWidth="1"/>
+    <col min="25" max="25" width="11.28515625" customWidth="1"/>
+    <col min="26" max="26" width="13.5703125" customWidth="1"/>
+    <col min="27" max="27" width="11.7109375" customWidth="1"/>
+    <col min="28" max="28" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -18660,7 +18663,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>168</v>
       </c>
@@ -18746,7 +18749,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>176</v>
       </c>
@@ -18835,7 +18838,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>177</v>
       </c>
@@ -18924,7 +18927,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>180</v>
       </c>
@@ -19013,7 +19016,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>181</v>
       </c>
@@ -19102,7 +19105,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>183</v>
       </c>
@@ -19191,7 +19194,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>186</v>
       </c>
@@ -19280,7 +19283,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>187</v>
       </c>
@@ -19369,7 +19372,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>188</v>
       </c>
@@ -19458,7 +19461,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>443</v>
       </c>
@@ -19547,9 +19550,9 @@
         <v>450</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B12">
         <v>8</v>
@@ -19644,33 +19647,33 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0094531B-7BBB-4DD3-8835-99962592A6C6}">
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="3" max="3" width="6.5546875" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" customWidth="1"/>
-    <col min="7" max="7" width="16.109375" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" customWidth="1"/>
-    <col min="10" max="11" width="9.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" customWidth="1"/>
-    <col min="13" max="14" width="10.109375" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="11" width="9.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="14" width="10.140625" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.44140625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" customWidth="1"/>
+    <col min="16" max="17" width="12.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12.28515625" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="17.33203125" customWidth="1"/>
-    <col min="21" max="21" width="12.44140625" customWidth="1"/>
-    <col min="22" max="22" width="12.33203125" customWidth="1"/>
-    <col min="23" max="23" width="18.5546875" customWidth="1"/>
-    <col min="25" max="25" width="13.5546875" customWidth="1"/>
-    <col min="26" max="26" width="11.6640625" customWidth="1"/>
+    <col min="20" max="20" width="17.28515625" customWidth="1"/>
+    <col min="21" max="21" width="12.42578125" customWidth="1"/>
+    <col min="22" max="22" width="12.28515625" customWidth="1"/>
+    <col min="23" max="23" width="18.5703125" customWidth="1"/>
+    <col min="25" max="25" width="13.5703125" customWidth="1"/>
+    <col min="26" max="26" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -19729,7 +19732,7 @@
         <v>73</v>
       </c>
       <c r="T1" s="19" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="U1" s="19" t="s">
         <v>86</v>
@@ -19756,7 +19759,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>211</v>
       </c>
@@ -19841,7 +19844,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>215</v>
       </c>
@@ -19926,7 +19929,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>220</v>
       </c>
@@ -20011,7 +20014,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>217</v>
       </c>
@@ -20096,7 +20099,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>216</v>
       </c>
@@ -20181,7 +20184,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>222</v>
       </c>
@@ -20266,7 +20269,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>218</v>
       </c>
@@ -20351,7 +20354,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>441</v>
       </c>
@@ -20436,9 +20439,9 @@
         <v>440</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B10">
         <v>78</v>
@@ -20521,9 +20524,9 @@
         <v>213</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -20606,9 +20609,9 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B12">
         <v>39</v>
@@ -20691,9 +20694,9 @@
         <v>440</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B13">
         <v>30</v>
@@ -20776,9 +20779,9 @@
         <v>440</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B14">
         <v>48</v>
@@ -20861,9 +20864,9 @@
         <v>440</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B15">
         <v>47</v>
@@ -20959,32 +20962,32 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B2364D-F43A-47E4-8B6C-A03FB84E628E}">
   <dimension ref="A1:AA16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" customWidth="1"/>
-    <col min="7" max="7" width="16.109375" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" customWidth="1"/>
-    <col min="10" max="11" width="9.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" customWidth="1"/>
-    <col min="13" max="14" width="10.109375" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="11" width="9.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="14" width="10.140625" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.44140625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" customWidth="1"/>
+    <col min="16" max="17" width="12.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12.28515625" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="14.109375" customWidth="1"/>
-    <col min="21" max="21" width="12.44140625" customWidth="1"/>
-    <col min="22" max="22" width="12.33203125" customWidth="1"/>
-    <col min="23" max="23" width="15.5546875" customWidth="1"/>
-    <col min="25" max="25" width="13.5546875" customWidth="1"/>
-    <col min="26" max="26" width="11.6640625" customWidth="1"/>
-    <col min="27" max="27" width="17.88671875" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" customWidth="1"/>
+    <col min="21" max="21" width="12.42578125" customWidth="1"/>
+    <col min="22" max="22" width="12.28515625" customWidth="1"/>
+    <col min="23" max="23" width="15.5703125" customWidth="1"/>
+    <col min="25" max="25" width="13.5703125" customWidth="1"/>
+    <col min="26" max="26" width="11.7109375" customWidth="1"/>
+    <col min="27" max="27" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -21067,7 +21070,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>223</v>
       </c>
@@ -21152,7 +21155,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>225</v>
       </c>
@@ -21237,7 +21240,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>229</v>
       </c>
@@ -21322,7 +21325,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>232</v>
       </c>
@@ -21407,7 +21410,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>233</v>
       </c>
@@ -21492,7 +21495,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>234</v>
       </c>
@@ -21577,9 +21580,9 @@
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="B8">
         <v>30</v>
@@ -21645,7 +21648,7 @@
         <v>76</v>
       </c>
       <c r="W8" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="X8" cm="1">
         <f t="array" aca="1" ref="X8" ca="1">INDEX(Caliber!B35:'Caliber'!C45,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B45,0),2)</f>
@@ -21659,10 +21662,10 @@
         <v>82</v>
       </c>
       <c r="AA8" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="X9" t="e" cm="1">
         <f t="array" aca="1" ref="X9" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -21672,7 +21675,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="X10" t="e" cm="1">
         <f t="array" aca="1" ref="X10" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -21682,7 +21685,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="X11" t="e" cm="1">
         <f t="array" aca="1" ref="X11" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -21692,7 +21695,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="X12" t="e" cm="1">
         <f t="array" aca="1" ref="X12" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -21702,7 +21705,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="X13" t="e" cm="1">
         <f t="array" aca="1" ref="X13" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -21712,7 +21715,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
       <c r="X14" t="e" cm="1">
         <f t="array" aca="1" ref="X14" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -21722,7 +21725,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
       <c r="X15" t="e" cm="1">
         <f t="array" aca="1" ref="X15" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -21732,7 +21735,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
       <c r="X16" t="e" cm="1">
         <f t="array" aca="1" ref="X16" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -21753,12 +21756,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD9C29F4-F90E-490E-8D34-BB5E6787CD6C}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>424</v>
       </c>

</xml_diff>

<commit_message>
SSG 08 + lategame major attacks
SSG 08 added.
Late game major attacks now show up after month 9.
Updated tech tree .drawio file.
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D1C437-2680-4BCB-A0F3-EA0B1A6B7E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543F4D48-48C5-4135-AE27-4F516F433596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="4" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="13" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1810" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1817" uniqueCount="600">
   <si>
     <t>Name</t>
   </si>
@@ -2665,7 +2665,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2917,13 +2917,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2953,7 +2953,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8166,8 +8165,8 @@
     </row>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="100"/>
-      <c r="B7" s="101"/>
-      <c r="C7" s="101"/>
+      <c r="B7" s="103"/>
+      <c r="C7" s="103"/>
       <c r="D7" s="59" t="s">
         <v>348</v>
       </c>
@@ -8180,7 +8179,7 @@
       <c r="G7" s="59" t="s">
         <v>576</v>
       </c>
-      <c r="H7" s="101"/>
+      <c r="H7" s="103"/>
     </row>
     <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="100"/>
@@ -8226,8 +8225,8 @@
     </row>
     <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="100"/>
-      <c r="B10" s="101"/>
-      <c r="C10" s="101"/>
+      <c r="B10" s="103"/>
+      <c r="C10" s="103"/>
       <c r="D10" s="59" t="s">
         <v>348</v>
       </c>
@@ -8240,7 +8239,7 @@
       <c r="G10" s="59" t="s">
         <v>480</v>
       </c>
-      <c r="H10" s="101"/>
+      <c r="H10" s="103"/>
     </row>
     <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="100"/>
@@ -8346,8 +8345,8 @@
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="100"/>
-      <c r="B16" s="101"/>
-      <c r="C16" s="101"/>
+      <c r="B16" s="103"/>
+      <c r="C16" s="103"/>
       <c r="D16" s="59" t="s">
         <v>348</v>
       </c>
@@ -8360,7 +8359,7 @@
       <c r="G16" s="59" t="s">
         <v>569</v>
       </c>
-      <c r="H16" s="101"/>
+      <c r="H16" s="103"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="100"/>
@@ -8406,8 +8405,8 @@
     </row>
     <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="100"/>
-      <c r="B19" s="101"/>
-      <c r="C19" s="101"/>
+      <c r="B19" s="103"/>
+      <c r="C19" s="103"/>
       <c r="D19" s="59" t="s">
         <v>348</v>
       </c>
@@ -8420,7 +8419,7 @@
       <c r="G19" s="59" t="s">
         <v>528</v>
       </c>
-      <c r="H19" s="101"/>
+      <c r="H19" s="103"/>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="100"/>
@@ -8480,7 +8479,7 @@
       <c r="G22" s="60" t="s">
         <v>364</v>
       </c>
-      <c r="H22" s="103"/>
+      <c r="H22" s="101"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="100"/>
@@ -8525,9 +8524,9 @@
       <c r="H24" s="100"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="103"/>
-      <c r="B25" s="103"/>
-      <c r="C25" s="103"/>
+      <c r="A25" s="101"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="101"/>
       <c r="D25" s="47" t="s">
         <v>348</v>
       </c>
@@ -8540,7 +8539,7 @@
       <c r="G25" s="47" t="s">
         <v>465</v>
       </c>
-      <c r="H25" s="103"/>
+      <c r="H25" s="101"/>
     </row>
     <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="102" t="s">
@@ -8628,8 +8627,8 @@
     </row>
     <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="100"/>
-      <c r="B31" s="101"/>
-      <c r="C31" s="101"/>
+      <c r="B31" s="103"/>
+      <c r="C31" s="103"/>
       <c r="D31" s="59" t="s">
         <v>348</v>
       </c>
@@ -8642,7 +8641,7 @@
       <c r="G31" s="78" t="s">
         <v>577</v>
       </c>
-      <c r="H31" s="101"/>
+      <c r="H31" s="103"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="100"/>
@@ -8987,9 +8986,9 @@
       <c r="H48" s="100"/>
     </row>
     <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="103"/>
-      <c r="B49" s="103"/>
-      <c r="C49" s="103"/>
+      <c r="A49" s="101"/>
+      <c r="B49" s="101"/>
+      <c r="C49" s="101"/>
       <c r="D49" s="47" t="s">
         <v>348</v>
       </c>
@@ -9002,22 +9001,35 @@
       <c r="G49" s="84" t="s">
         <v>498</v>
       </c>
-      <c r="H49" s="103"/>
+      <c r="H49" s="101"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="H44:H46"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="A26:A49"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="H35:H37"/>
     <mergeCell ref="A2:A25"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C2:C4"/>
@@ -9034,31 +9046,18 @@
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="H5:H7"/>
     <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A26:A49"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="H35:H37"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="H44:H46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9677,9 +9676,6 @@
       <c r="B26" s="14"/>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>599</v>
-      </c>
       <c r="B27" s="14"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -18317,7 +18313,7 @@
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A16" s="113" t="s">
+      <c r="A16" s="57" t="s">
         <v>594</v>
       </c>
       <c r="B16">
@@ -18326,8 +18322,8 @@
       <c r="C16" t="s">
         <v>90</v>
       </c>
-      <c r="D16" t="s">
-        <v>76</v>
+      <c r="D16">
+        <v>45000</v>
       </c>
       <c r="E16" t="b">
         <v>1</v>
@@ -18398,17 +18394,89 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="24:25" x14ac:dyDescent="0.25">
-      <c r="X17" t="e">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>599</v>
+      </c>
+      <c r="B17">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>90</v>
+      </c>
+      <c r="D17">
+        <v>49000</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="s">
+        <v>76</v>
+      </c>
+      <c r="H17">
+        <v>145</v>
+      </c>
+      <c r="I17">
+        <v>75</v>
+      </c>
+      <c r="J17">
+        <v>50</v>
+      </c>
+      <c r="K17" t="s">
+        <v>76</v>
+      </c>
+      <c r="L17">
+        <v>125</v>
+      </c>
+      <c r="M17">
+        <v>90</v>
+      </c>
+      <c r="N17" t="s">
+        <v>76</v>
+      </c>
+      <c r="O17">
+        <v>200</v>
+      </c>
+      <c r="P17">
+        <v>35</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>76</v>
+      </c>
+      <c r="R17">
+        <v>200</v>
+      </c>
+      <c r="S17">
+        <v>5</v>
+      </c>
+      <c r="T17">
+        <v>1</v>
+      </c>
+      <c r="U17">
+        <v>1</v>
+      </c>
+      <c r="V17" t="s">
+        <v>76</v>
+      </c>
+      <c r="W17" t="s">
+        <v>152</v>
+      </c>
+      <c r="X17">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W17,Caliber!B13:'Caliber'!B23,0),2)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Y17" t="e">
+        <v>45</v>
+      </c>
+      <c r="Y17">
         <f>INDEX(Caliber!C13:'Caliber'!D23,MATCH(W17,Caliber!B13:'Caliber'!B23,0),2)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="18" spans="24:25" x14ac:dyDescent="0.25">
+        <v>0.6</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X18" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W18,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18418,7 +18486,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="19" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X19" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W19,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18428,7 +18496,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="20" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X20" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W20,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18438,7 +18506,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="21" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X21" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W21,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18448,7 +18516,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="22" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X22" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W22,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18458,7 +18526,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="23" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X23" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W23,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18468,7 +18536,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="24" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X24" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W24,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18478,7 +18546,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="25" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X25" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W25,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18488,7 +18556,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="26" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X26" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W26,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18498,7 +18566,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="27" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X27" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W27,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18508,7 +18576,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="28" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X28" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W28,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18518,7 +18586,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="29" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X29" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W29,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -18528,7 +18596,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="30" spans="24:25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="X30" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W30,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>

</xml_diff>

<commit_message>
Weapon range in ufopaedia
SSG 08 sprite bug fixed
FMG 9 now unfolds properly
FMG9 weight reduced from 22->17
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09950D76-C716-4B06-B24C-6E8309944B32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E997E6BA-9920-4158-8B4B-A15B5C584C39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="735" windowWidth="19440" windowHeight="15000" firstSheet="6" activeTab="11" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="2" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -120,7 +120,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1841" uniqueCount="605">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1839" uniqueCount="603">
   <si>
     <t>Name</t>
   </si>
@@ -1980,12 +1980,6 @@
   </si>
   <si>
     <t>AR-18</t>
-  </si>
-  <si>
-    <t>Saiga rifle (5.45)</t>
-  </si>
-  <si>
-    <t>cz 858</t>
   </si>
   <si>
     <t>ak 104</t>
@@ -8268,10 +8262,10 @@
         <v>344</v>
       </c>
       <c r="E11" s="61" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="F11" s="61" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="G11" s="61" t="s">
         <v>546</v>
@@ -8288,10 +8282,10 @@
         <v>347</v>
       </c>
       <c r="E12" s="46" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F12" s="46" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="G12" s="46" t="s">
         <v>203</v>
@@ -9697,20 +9691,14 @@
       <c r="B27" s="14"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>598</v>
-      </c>
       <c r="B28" s="14"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>599</v>
-      </c>
       <c r="B29" s="14"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="B30" s="14"/>
     </row>
@@ -11237,7 +11225,7 @@
         <v>433</v>
       </c>
       <c r="B3">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
         <v>75</v>
@@ -17056,7 +17044,7 @@
     </row>
     <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B57">
         <v>22</v>
@@ -17138,7 +17126,7 @@
     </row>
     <row r="58" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="B58">
         <v>23</v>

</xml_diff>

<commit_message>
EOD suit in campaign
EOD suit research, name string, item, and ufopaedia page
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F54F9D-6BFF-4BA5-A2BA-2F50361B7694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEBB1E07-853B-4A8E-B290-7E3A5C675546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="8" activeTab="11" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="13" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -2051,9 +2051,6 @@
     <t>Beretta 93R</t>
   </si>
   <si>
-    <t>EOD suit</t>
-  </si>
-  <si>
     <t>TEC-9/TEC-9/Skorpion</t>
   </si>
   <si>
@@ -2228,6 +2225,9 @@
   </si>
   <si>
     <t>HK417/?/G11</t>
+  </si>
+  <si>
+    <t>Ending slides</t>
   </si>
 </sst>
 </file>
@@ -3207,13 +3207,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4406,20 +4406,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6695E0F0-C0B0-45B8-AA00-1AE0F467FE87}">
   <dimension ref="A1:S49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.109375" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
-    <col min="8" max="8" width="14.7109375" customWidth="1"/>
-    <col min="9" max="9" width="131.85546875" customWidth="1"/>
-    <col min="12" max="12" width="20.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="5" max="5" width="14.88671875" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.88671875" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" customWidth="1"/>
+    <col min="9" max="9" width="131.88671875" customWidth="1"/>
+    <col min="12" max="12" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>17</v>
       </c>
@@ -4448,7 +4448,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="1" t="s">
         <v>8</v>
@@ -4476,7 +4476,7 @@
       <c r="P2" s="13"/>
       <c r="Q2" s="13"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" t="s">
         <v>10</v>
@@ -4495,7 +4495,7 @@
       </c>
       <c r="M3" s="14"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" t="s">
         <v>95</v>
@@ -4518,7 +4518,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" t="s">
         <v>12</v>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="M5" s="14"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" t="s">
         <v>16</v>
@@ -4560,7 +4560,7 @@
       <c r="P6" s="10"/>
       <c r="Q6" s="10"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" t="s">
         <v>15</v>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="M7" s="14"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" t="s">
         <v>13</v>
@@ -4602,7 +4602,7 @@
       <c r="P8" s="10"/>
       <c r="Q8" s="10"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" t="s">
         <v>14</v>
@@ -4625,7 +4625,7 @@
       <c r="P9" s="11"/>
       <c r="Q9" s="11"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" t="s">
         <v>411</v>
@@ -4646,7 +4646,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="56"/>
       <c r="B11" t="s">
         <v>427</v>
@@ -4679,7 +4679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="55" t="s">
         <v>22</v>
       </c>
@@ -4723,7 +4723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="1" t="s">
         <v>18</v>
@@ -4759,7 +4759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" t="s">
         <v>19</v>
@@ -4792,7 +4792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" t="s">
         <v>120</v>
@@ -4825,7 +4825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" t="s">
         <v>23</v>
@@ -4858,7 +4858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" t="s">
         <v>25</v>
@@ -4891,7 +4891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" t="s">
         <v>26</v>
@@ -4924,7 +4924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="B19" t="s">
         <v>27</v>
@@ -4957,7 +4957,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" t="s">
         <v>28</v>
@@ -4990,7 +4990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
       <c r="B21" t="s">
         <v>30</v>
@@ -5023,7 +5023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
       <c r="B22" t="s">
         <v>29</v>
@@ -5041,7 +5041,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
       <c r="B23" t="s">
         <v>31</v>
@@ -5080,7 +5080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" t="s">
         <v>523</v>
@@ -5119,7 +5119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>32</v>
       </c>
@@ -5169,7 +5169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" s="6"/>
       <c r="B26" s="1" t="s">
         <v>33</v>
@@ -5215,7 +5215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A27" s="7"/>
       <c r="B27" t="s">
         <v>34</v>
@@ -5260,7 +5260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A28" s="7"/>
       <c r="B28" t="s">
         <v>35</v>
@@ -5308,7 +5308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A29" s="7"/>
       <c r="B29" t="s">
         <v>432</v>
@@ -5335,7 +5335,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" s="7"/>
       <c r="B30" t="s">
         <v>435</v>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="S30" s="13"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" s="7"/>
       <c r="B31" t="s">
         <v>37</v>
@@ -5423,7 +5423,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A32" s="7"/>
       <c r="B32" t="s">
         <v>38</v>
@@ -5466,7 +5466,7 @@
       </c>
       <c r="S32" s="10"/>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A33" s="7"/>
       <c r="B33" t="s">
         <v>39</v>
@@ -5511,7 +5511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>40</v>
       </c>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="S34" s="10"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" s="8"/>
       <c r="B35" s="1" t="s">
         <v>41</v>
@@ -5602,7 +5602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" s="9"/>
       <c r="B36" t="s">
         <v>43</v>
@@ -5645,7 +5645,7 @@
       </c>
       <c r="S36" s="10"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" s="9"/>
       <c r="B37" t="s">
         <v>45</v>
@@ -5687,7 +5687,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A38" s="9"/>
       <c r="B38" t="s">
         <v>47</v>
@@ -5730,7 +5730,7 @@
       </c>
       <c r="S38" s="10"/>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A39" s="9"/>
       <c r="B39" t="s">
         <v>49</v>
@@ -5751,7 +5751,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" s="9"/>
       <c r="B40" t="s">
         <v>50</v>
@@ -5772,7 +5772,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" s="9"/>
       <c r="B41" t="s">
         <v>51</v>
@@ -5793,7 +5793,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" s="9"/>
       <c r="B42" t="s">
         <v>52</v>
@@ -5814,7 +5814,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A43" s="9"/>
       <c r="B43" t="s">
         <v>53</v>
@@ -5835,7 +5835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" s="9"/>
       <c r="B44" t="s">
         <v>503</v>
@@ -5859,7 +5859,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" s="9"/>
       <c r="B45" t="s">
         <v>519</v>
@@ -5883,7 +5883,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" s="9"/>
       <c r="B46" t="s">
         <v>520</v>
@@ -5907,10 +5907,10 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A47" s="9"/>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A48" s="53" t="s">
         <v>434</v>
       </c>
@@ -5939,7 +5939,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="54"/>
       <c r="B49" s="14" t="s">
         <v>425</v>
@@ -5974,18 +5974,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BABADE2C-4009-4AB7-BED9-B450B00DFD85}">
   <dimension ref="A1:P32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" customWidth="1"/>
-    <col min="11" max="11" width="14.140625" customWidth="1"/>
-    <col min="12" max="12" width="10.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" customWidth="1"/>
+    <col min="11" max="11" width="14.109375" customWidth="1"/>
+    <col min="12" max="12" width="10.44140625" customWidth="1"/>
     <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="10.42578125" customWidth="1"/>
-    <col min="15" max="15" width="13.28515625" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" customWidth="1"/>
+    <col min="14" max="14" width="10.44140625" customWidth="1"/>
+    <col min="15" max="15" width="13.33203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="108" t="s">
         <v>236</v>
       </c>
@@ -6021,7 +6021,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="109"/>
       <c r="B2" s="20" t="s">
         <v>245</v>
@@ -6057,7 +6057,7 @@
       <c r="O2" s="109"/>
       <c r="P2" s="109"/>
     </row>
-    <row r="3" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
         <v>254</v>
       </c>
@@ -6097,7 +6097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="32" t="s">
         <v>257</v>
       </c>
@@ -6141,7 +6141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
         <v>258</v>
       </c>
@@ -6189,7 +6189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="32" t="s">
         <v>259</v>
       </c>
@@ -6237,7 +6237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="26" t="s">
         <v>260</v>
       </c>
@@ -6285,7 +6285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="32" t="s">
         <v>262</v>
       </c>
@@ -6333,7 +6333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="26" t="s">
         <v>263</v>
       </c>
@@ -6381,7 +6381,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="32" t="s">
         <v>266</v>
       </c>
@@ -6429,7 +6429,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="32" t="s">
         <v>291</v>
       </c>
@@ -6479,7 +6479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="32" t="s">
         <v>292</v>
       </c>
@@ -6529,7 +6529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="33" t="s">
         <v>267</v>
       </c>
@@ -6569,7 +6569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="33" t="s">
         <v>269</v>
       </c>
@@ -6613,7 +6613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="33" t="s">
         <v>270</v>
       </c>
@@ -6661,7 +6661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="33" t="s">
         <v>271</v>
       </c>
@@ -6709,7 +6709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="33" t="s">
         <v>272</v>
       </c>
@@ -6757,7 +6757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="33" t="s">
         <v>273</v>
       </c>
@@ -6805,7 +6805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="33" t="s">
         <v>274</v>
       </c>
@@ -6853,7 +6853,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="33" t="s">
         <v>275</v>
       </c>
@@ -6901,7 +6901,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="33" t="s">
         <v>276</v>
       </c>
@@ -6943,7 +6943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="33" t="s">
         <v>278</v>
       </c>
@@ -6989,7 +6989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="33" t="s">
         <v>279</v>
       </c>
@@ -7039,7 +7039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="33" t="s">
         <v>280</v>
       </c>
@@ -7089,7 +7089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="33" t="s">
         <v>281</v>
       </c>
@@ -7139,7 +7139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="33" t="s">
         <v>283</v>
       </c>
@@ -7189,7 +7189,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="33" t="s">
         <v>284</v>
       </c>
@@ -7239,7 +7239,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="33" t="s">
         <v>286</v>
       </c>
@@ -7289,7 +7289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="26" t="s">
         <v>287</v>
       </c>
@@ -7339,7 +7339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="32" t="s">
         <v>288</v>
       </c>
@@ -7389,7 +7389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="26" t="s">
         <v>289</v>
       </c>
@@ -7439,7 +7439,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="104" t="s">
         <v>290</v>
       </c>
@@ -7508,16 +7508,16 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C092F238-A859-4DAF-9B24-82DF047DC2BE}">
   <dimension ref="A1:Q19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="14" max="14" width="11.85546875" customWidth="1"/>
-    <col min="16" max="16" width="16.28515625" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="14" max="14" width="11.88671875" customWidth="1"/>
+    <col min="16" max="16" width="16.33203125" customWidth="1"/>
+    <col min="17" max="17" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>333</v>
       </c>
@@ -7570,7 +7570,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="32" t="s">
         <v>334</v>
       </c>
@@ -7617,7 +7617,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="113" t="s">
         <v>335</v>
       </c>
@@ -7655,7 +7655,7 @@
         <v>50</v>
       </c>
       <c r="M3" s="26" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N3" s="26" t="s">
         <v>313</v>
@@ -7666,7 +7666,7 @@
       <c r="P3" s="39"/>
       <c r="Q3" s="39"/>
     </row>
-    <row r="4" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="114"/>
       <c r="B4" s="32" t="s">
         <v>299</v>
@@ -7702,7 +7702,7 @@
         <v>40</v>
       </c>
       <c r="M4" s="32" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N4" s="32" t="s">
         <v>313</v>
@@ -7713,7 +7713,7 @@
       <c r="P4" s="38"/>
       <c r="Q4" s="38"/>
     </row>
-    <row r="5" spans="1:17" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="114"/>
       <c r="B5" s="26" t="s">
         <v>315</v>
@@ -7753,12 +7753,12 @@
         <v>318</v>
       </c>
       <c r="O5" s="26" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="P5" s="39"/>
       <c r="Q5" s="39"/>
     </row>
-    <row r="6" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="114"/>
       <c r="B6" s="32" t="s">
         <v>317</v>
@@ -7798,12 +7798,12 @@
         <v>316</v>
       </c>
       <c r="O6" s="32" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="P6" s="38"/>
       <c r="Q6" s="38"/>
     </row>
-    <row r="7" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="114"/>
       <c r="B7" s="26" t="s">
         <v>319</v>
@@ -7839,7 +7839,7 @@
         <v>20</v>
       </c>
       <c r="M7" s="26" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N7" s="26" t="s">
         <v>320</v>
@@ -7850,7 +7850,7 @@
       <c r="P7" s="39"/>
       <c r="Q7" s="39"/>
     </row>
-    <row r="8" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="114"/>
       <c r="B8" s="32" t="s">
         <v>321</v>
@@ -7890,12 +7890,12 @@
         <v>322</v>
       </c>
       <c r="O8" s="32" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="P8" s="38"/>
       <c r="Q8" s="38"/>
     </row>
-    <row r="9" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="114"/>
       <c r="B9" s="26" t="s">
         <v>323</v>
@@ -7935,12 +7935,12 @@
         <v>320</v>
       </c>
       <c r="O9" s="26" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="P9" s="39"/>
       <c r="Q9" s="39"/>
     </row>
-    <row r="10" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="115"/>
       <c r="B10" s="32" t="s">
         <v>324</v>
@@ -7980,12 +7980,12 @@
         <v>325</v>
       </c>
       <c r="O10" s="32" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="P10" s="38"/>
       <c r="Q10" s="38"/>
     </row>
-    <row r="11" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="113" t="s">
         <v>336</v>
       </c>
@@ -8008,7 +8008,7 @@
       <c r="P11" s="39"/>
       <c r="Q11" s="39"/>
     </row>
-    <row r="12" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="114"/>
       <c r="B12" s="32" t="s">
         <v>299</v>
@@ -8044,7 +8044,7 @@
         <v>50</v>
       </c>
       <c r="M12" s="32" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="N12" s="32" t="s">
         <v>326</v>
@@ -8055,7 +8055,7 @@
       <c r="P12" s="38"/>
       <c r="Q12" s="38"/>
     </row>
-    <row r="13" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="114"/>
       <c r="B13" s="26" t="s">
         <v>328</v>
@@ -8102,7 +8102,7 @@
       <c r="P13" s="39"/>
       <c r="Q13" s="39"/>
     </row>
-    <row r="14" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="114"/>
       <c r="B14" s="32" t="s">
         <v>317</v>
@@ -8138,7 +8138,7 @@
         <v>30</v>
       </c>
       <c r="M14" s="32" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N14" s="32" t="s">
         <v>313</v>
@@ -8149,7 +8149,7 @@
       <c r="P14" s="38"/>
       <c r="Q14" s="38"/>
     </row>
-    <row r="15" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="114"/>
       <c r="B15" s="26" t="s">
         <v>287</v>
@@ -8196,7 +8196,7 @@
       <c r="P15" s="39"/>
       <c r="Q15" s="39"/>
     </row>
-    <row r="16" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="114"/>
       <c r="B16" s="32" t="s">
         <v>321</v>
@@ -8232,7 +8232,7 @@
         <v>30</v>
       </c>
       <c r="M16" s="32" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N16" s="32" t="s">
         <v>313</v>
@@ -8243,7 +8243,7 @@
       <c r="P16" s="38"/>
       <c r="Q16" s="38"/>
     </row>
-    <row r="17" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="114"/>
       <c r="B17" s="26" t="s">
         <v>315</v>
@@ -8279,7 +8279,7 @@
         <v>30</v>
       </c>
       <c r="M17" s="26" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="N17" s="26" t="s">
         <v>313</v>
@@ -8290,7 +8290,7 @@
       <c r="P17" s="39"/>
       <c r="Q17" s="39"/>
     </row>
-    <row r="18" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="115"/>
       <c r="B18" s="32" t="s">
         <v>324</v>
@@ -8326,7 +8326,7 @@
         <v>30</v>
       </c>
       <c r="M18" s="32" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N18" s="32" t="s">
         <v>331</v>
@@ -8337,12 +8337,12 @@
       <c r="P18" s="38"/>
       <c r="Q18" s="38"/>
     </row>
-    <row r="19" spans="1:17" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="26" t="s">
         <v>434</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="C19" s="94">
         <v>100</v>
@@ -8375,13 +8375,13 @@
         <v>50</v>
       </c>
       <c r="M19" s="91" t="s">
+        <v>623</v>
+      </c>
+      <c r="N19" s="32" t="s">
         <v>624</v>
       </c>
-      <c r="N19" s="32" t="s">
-        <v>625</v>
-      </c>
       <c r="O19" s="32" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="P19" s="103"/>
       <c r="Q19" s="103"/>
@@ -8398,19 +8398,19 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D21C18DE-CCD8-4ABA-9B3B-CCD73CA8C93E}">
   <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="43.140625" customWidth="1"/>
-    <col min="6" max="6" width="53.7109375" customWidth="1"/>
-    <col min="7" max="7" width="46.28515625" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" customWidth="1"/>
-    <col min="9" max="9" width="30.140625" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="43.109375" customWidth="1"/>
+    <col min="6" max="6" width="53.6640625" customWidth="1"/>
+    <col min="7" max="7" width="46.33203125" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" customWidth="1"/>
+    <col min="9" max="9" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="44" t="s">
         <v>333</v>
       </c>
@@ -8437,7 +8437,7 @@
       </c>
       <c r="I1" s="48"/>
     </row>
-    <row r="2" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="119" t="s">
         <v>381</v>
       </c>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="I2" s="62"/>
     </row>
-    <row r="3" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="117"/>
       <c r="B3" s="117"/>
       <c r="C3" s="117"/>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="H3" s="117"/>
     </row>
-    <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="117"/>
       <c r="B4" s="117"/>
       <c r="C4" s="117"/>
@@ -8500,7 +8500,7 @@
       </c>
       <c r="H4" s="117"/>
     </row>
-    <row r="5" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="117"/>
       <c r="B5" s="116" t="s">
         <v>299</v>
@@ -8524,7 +8524,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="117"/>
       <c r="B6" s="117"/>
       <c r="C6" s="117"/>
@@ -8542,10 +8542,10 @@
       </c>
       <c r="H6" s="117"/>
     </row>
-    <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="117"/>
-      <c r="B7" s="118"/>
-      <c r="C7" s="118"/>
+      <c r="B7" s="120"/>
+      <c r="C7" s="120"/>
       <c r="D7" s="59" t="s">
         <v>347</v>
       </c>
@@ -8558,9 +8558,9 @@
       <c r="G7" s="59" t="s">
         <v>560</v>
       </c>
-      <c r="H7" s="118"/>
-    </row>
-    <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H7" s="120"/>
+    </row>
+    <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="117"/>
       <c r="B8" s="116" t="s">
         <v>351</v>
@@ -8584,7 +8584,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="117"/>
       <c r="B9" s="117"/>
       <c r="C9" s="117"/>
@@ -8592,7 +8592,7 @@
         <v>346</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="F9" s="46" t="s">
         <v>537</v>
@@ -8602,10 +8602,10 @@
       </c>
       <c r="H9" s="117"/>
     </row>
-    <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="117"/>
-      <c r="B10" s="118"/>
-      <c r="C10" s="118"/>
+      <c r="B10" s="120"/>
+      <c r="C10" s="120"/>
       <c r="D10" s="59" t="s">
         <v>347</v>
       </c>
@@ -8618,9 +8618,9 @@
       <c r="G10" s="59" t="s">
         <v>464</v>
       </c>
-      <c r="H10" s="118"/>
-    </row>
-    <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H10" s="120"/>
+    </row>
+    <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="117"/>
       <c r="B11" s="116" t="s">
         <v>353</v>
@@ -8632,10 +8632,10 @@
         <v>343</v>
       </c>
       <c r="E11" s="61" t="s">
+        <v>587</v>
+      </c>
+      <c r="F11" s="61" t="s">
         <v>588</v>
-      </c>
-      <c r="F11" s="61" t="s">
-        <v>589</v>
       </c>
       <c r="G11" s="61" t="s">
         <v>534</v>
@@ -8644,7 +8644,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="117"/>
       <c r="B12" s="117"/>
       <c r="C12" s="117"/>
@@ -8652,17 +8652,17 @@
         <v>346</v>
       </c>
       <c r="E12" s="46" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="F12" s="46" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G12" s="46" t="s">
         <v>203</v>
       </c>
       <c r="H12" s="117"/>
     </row>
-    <row r="13" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="117"/>
       <c r="B13" s="117"/>
       <c r="C13" s="117"/>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="H13" s="117"/>
     </row>
-    <row r="14" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="117"/>
       <c r="B14" s="116" t="s">
         <v>356</v>
@@ -8704,7 +8704,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="117"/>
       <c r="B15" s="117"/>
       <c r="C15" s="117"/>
@@ -8722,10 +8722,10 @@
       </c>
       <c r="H15" s="117"/>
     </row>
-    <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="117"/>
-      <c r="B16" s="118"/>
-      <c r="C16" s="118"/>
+      <c r="B16" s="120"/>
+      <c r="C16" s="120"/>
       <c r="D16" s="59" t="s">
         <v>347</v>
       </c>
@@ -8738,9 +8738,9 @@
       <c r="G16" s="59" t="s">
         <v>553</v>
       </c>
-      <c r="H16" s="118"/>
-    </row>
-    <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H16" s="120"/>
+    </row>
+    <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="117"/>
       <c r="B17" s="116" t="s">
         <v>357</v>
@@ -8764,7 +8764,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="117"/>
       <c r="B18" s="117"/>
       <c r="C18" s="117"/>
@@ -8775,17 +8775,17 @@
         <v>533</v>
       </c>
       <c r="F18" s="46" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="G18" s="46" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="H18" s="117"/>
     </row>
-    <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="117"/>
-      <c r="B19" s="118"/>
-      <c r="C19" s="118"/>
+      <c r="B19" s="120"/>
+      <c r="C19" s="120"/>
       <c r="D19" s="59" t="s">
         <v>347</v>
       </c>
@@ -8798,9 +8798,9 @@
       <c r="G19" s="59" t="s">
         <v>512</v>
       </c>
-      <c r="H19" s="118"/>
-    </row>
-    <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H19" s="120"/>
+    </row>
+    <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="117"/>
       <c r="B20" s="116" t="s">
         <v>358</v>
@@ -8818,13 +8818,13 @@
         <v>521</v>
       </c>
       <c r="G20" s="61" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="H20" s="116" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="117"/>
       <c r="B21" s="117"/>
       <c r="C21" s="117"/>
@@ -8842,7 +8842,7 @@
       </c>
       <c r="H21" s="117"/>
     </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="117"/>
       <c r="B22" s="117"/>
       <c r="C22" s="117"/>
@@ -8850,17 +8850,17 @@
         <v>347</v>
       </c>
       <c r="E22" s="60" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="F22" s="60" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="G22" s="60" t="s">
         <v>361</v>
       </c>
-      <c r="H22" s="120"/>
-    </row>
-    <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="118"/>
+    </row>
+    <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="117"/>
       <c r="B23" s="116" t="s">
         <v>362</v>
@@ -8875,16 +8875,16 @@
         <v>148</v>
       </c>
       <c r="F23" s="61" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="G23" s="61" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="H23" s="119" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="117"/>
       <c r="B24" s="117"/>
       <c r="C24" s="117"/>
@@ -8895,17 +8895,17 @@
         <v>528</v>
       </c>
       <c r="F24" s="46" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="G24" s="46" t="s">
         <v>453</v>
       </c>
       <c r="H24" s="117"/>
     </row>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="120"/>
-      <c r="B25" s="120"/>
-      <c r="C25" s="120"/>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="118"/>
+      <c r="B25" s="118"/>
+      <c r="C25" s="118"/>
       <c r="D25" s="47" t="s">
         <v>347</v>
       </c>
@@ -8918,9 +8918,9 @@
       <c r="G25" s="47" t="s">
         <v>452</v>
       </c>
-      <c r="H25" s="120"/>
-    </row>
-    <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H25" s="118"/>
+    </row>
+    <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="119" t="s">
         <v>336</v>
       </c>
@@ -8938,7 +8938,7 @@
       <c r="G26" s="123"/>
       <c r="H26" s="124"/>
     </row>
-    <row r="27" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="117"/>
       <c r="B27" s="117"/>
       <c r="C27" s="117"/>
@@ -8950,7 +8950,7 @@
       <c r="G27" s="123"/>
       <c r="H27" s="125"/>
     </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="117"/>
       <c r="B28" s="117"/>
       <c r="C28" s="117"/>
@@ -8962,7 +8962,7 @@
       <c r="G28" s="128"/>
       <c r="H28" s="125"/>
     </row>
-    <row r="29" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="117"/>
       <c r="B29" s="116" t="s">
         <v>299</v>
@@ -8986,7 +8986,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="117"/>
       <c r="B30" s="117"/>
       <c r="C30" s="117"/>
@@ -9000,14 +9000,14 @@
         <v>501</v>
       </c>
       <c r="G30" s="77" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="H30" s="117"/>
     </row>
-    <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="117"/>
-      <c r="B31" s="118"/>
-      <c r="C31" s="118"/>
+      <c r="B31" s="120"/>
+      <c r="C31" s="120"/>
       <c r="D31" s="59" t="s">
         <v>347</v>
       </c>
@@ -9020,9 +9020,9 @@
       <c r="G31" s="78" t="s">
         <v>561</v>
       </c>
-      <c r="H31" s="118"/>
-    </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H31" s="120"/>
+    </row>
+    <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="117"/>
       <c r="B32" s="117" t="s">
         <v>351</v>
@@ -9046,7 +9046,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="117"/>
       <c r="B33" s="117"/>
       <c r="C33" s="117"/>
@@ -9064,7 +9064,7 @@
       </c>
       <c r="H33" s="117"/>
     </row>
-    <row r="34" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="117"/>
       <c r="B34" s="117"/>
       <c r="C34" s="117"/>
@@ -9082,7 +9082,7 @@
       </c>
       <c r="H34" s="117"/>
     </row>
-    <row r="35" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="117"/>
       <c r="B35" s="116" t="s">
         <v>353</v>
@@ -9106,7 +9106,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="117"/>
       <c r="B36" s="117"/>
       <c r="C36" s="117"/>
@@ -9124,7 +9124,7 @@
       </c>
       <c r="H36" s="117"/>
     </row>
-    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="117"/>
       <c r="B37" s="117"/>
       <c r="C37" s="117"/>
@@ -9142,7 +9142,7 @@
       </c>
       <c r="H37" s="117"/>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="117"/>
       <c r="B38" s="116" t="s">
         <v>356</v>
@@ -9166,7 +9166,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="117"/>
       <c r="B39" s="117"/>
       <c r="C39" s="117"/>
@@ -9184,7 +9184,7 @@
       </c>
       <c r="H39" s="117"/>
     </row>
-    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="117"/>
       <c r="B40" s="117"/>
       <c r="C40" s="117"/>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="H40" s="117"/>
     </row>
-    <row r="41" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="117"/>
       <c r="B41" s="116" t="s">
         <v>357</v>
@@ -9226,7 +9226,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="117"/>
       <c r="B42" s="117"/>
       <c r="C42" s="117"/>
@@ -9244,7 +9244,7 @@
       </c>
       <c r="H42" s="117"/>
     </row>
-    <row r="43" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="117"/>
       <c r="B43" s="117"/>
       <c r="C43" s="117"/>
@@ -9262,7 +9262,7 @@
       </c>
       <c r="H43" s="117"/>
     </row>
-    <row r="44" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="117"/>
       <c r="B44" s="116" t="s">
         <v>358</v>
@@ -9286,7 +9286,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="117"/>
       <c r="B45" s="117"/>
       <c r="C45" s="117"/>
@@ -9304,7 +9304,7 @@
       </c>
       <c r="H45" s="117"/>
     </row>
-    <row r="46" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="117"/>
       <c r="B46" s="117"/>
       <c r="C46" s="117"/>
@@ -9322,7 +9322,7 @@
       </c>
       <c r="H46" s="117"/>
     </row>
-    <row r="47" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="117"/>
       <c r="B47" s="116" t="s">
         <v>362</v>
@@ -9346,7 +9346,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="117"/>
       <c r="B48" s="117"/>
       <c r="C48" s="117"/>
@@ -9364,10 +9364,10 @@
       </c>
       <c r="H48" s="117"/>
     </row>
-    <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="120"/>
-      <c r="B49" s="120"/>
-      <c r="C49" s="120"/>
+    <row r="49" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="118"/>
+      <c r="B49" s="118"/>
+      <c r="C49" s="118"/>
       <c r="D49" s="47" t="s">
         <v>347</v>
       </c>
@@ -9380,22 +9380,35 @@
       <c r="G49" s="84" t="s">
         <v>482</v>
       </c>
-      <c r="H49" s="120"/>
+      <c r="H49" s="118"/>
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="H47:H49"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="H44:H46"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="H41:H43"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="A26:A49"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="H35:H37"/>
     <mergeCell ref="A2:A25"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C2:C4"/>
@@ -9412,31 +9425,18 @@
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="H5:H7"/>
     <mergeCell ref="B8:B10"/>
-    <mergeCell ref="A26:A49"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="C26:C28"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:H28"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="H35:H37"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="H14:H16"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:C13"/>
-    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="H41:H43"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="H38:H40"/>
+    <mergeCell ref="B47:B49"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="H47:H49"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="H44:H46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -9446,20 +9446,20 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC8BAE7-4B1E-4B8C-8AF9-C5EAA5B2467F}">
   <dimension ref="A1:P11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="8.44140625" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
-    <col min="9" max="9" width="13.85546875" customWidth="1"/>
-    <col min="11" max="11" width="15.140625" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" customWidth="1"/>
+    <col min="11" max="11" width="15.109375" customWidth="1"/>
+    <col min="12" max="12" width="10.88671875" customWidth="1"/>
+    <col min="14" max="14" width="13.5546875" customWidth="1"/>
     <col min="15" max="15" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
         <v>236</v>
       </c>
@@ -9509,7 +9509,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="32" t="s">
         <v>379</v>
       </c>
@@ -9559,12 +9559,12 @@
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
         <v>385</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C3" s="26">
         <v>12</v>
@@ -9609,12 +9609,12 @@
         <v>384</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="32" t="s">
         <v>387</v>
       </c>
       <c r="B4" s="32" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="C4" s="32">
         <v>0</v>
@@ -9638,7 +9638,7 @@
         <v>406</v>
       </c>
       <c r="J4" s="49" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="K4" s="49">
         <v>0</v>
@@ -9659,7 +9659,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
         <v>390</v>
       </c>
@@ -9682,13 +9682,13 @@
         <v>404</v>
       </c>
       <c r="H5" s="50" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="I5" s="50" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="J5" s="50" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="K5" s="50" t="s">
         <v>408</v>
@@ -9709,12 +9709,12 @@
         <v>384</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="32" t="s">
         <v>394</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="C6" s="32">
         <v>10</v>
@@ -9759,7 +9759,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="26" t="s">
         <v>395</v>
       </c>
@@ -9779,28 +9779,28 @@
         <v>2</v>
       </c>
       <c r="G7" s="50" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="H7" s="50" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="I7" s="50" t="s">
         <v>407</v>
       </c>
       <c r="J7" s="50" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="K7" s="50" t="s">
         <v>408</v>
       </c>
       <c r="L7" s="50" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="M7" s="26" t="s">
         <v>392</v>
       </c>
       <c r="N7" s="26" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="O7" s="26" t="s">
         <v>397</v>
@@ -9809,7 +9809,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="32" t="s">
         <v>398</v>
       </c>
@@ -9838,7 +9838,7 @@
         <v>406</v>
       </c>
       <c r="J8" s="49" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="K8" s="49">
         <v>0</v>
@@ -9850,7 +9850,7 @@
         <v>386</v>
       </c>
       <c r="N8" s="32" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="O8" s="32" t="s">
         <v>397</v>
@@ -9859,12 +9859,12 @@
         <v>384</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="26" t="s">
         <v>400</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="C9" s="26">
         <v>12</v>
@@ -9882,13 +9882,13 @@
         <v>406</v>
       </c>
       <c r="H9" s="50" t="s">
+        <v>602</v>
+      </c>
+      <c r="I9" s="50" t="s">
+        <v>602</v>
+      </c>
+      <c r="J9" s="50" t="s">
         <v>603</v>
-      </c>
-      <c r="I9" s="50" t="s">
-        <v>603</v>
-      </c>
-      <c r="J9" s="50" t="s">
-        <v>604</v>
       </c>
       <c r="K9" s="50" t="s">
         <v>404</v>
@@ -9900,7 +9900,7 @@
         <v>401</v>
       </c>
       <c r="N9" s="26" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="O9" s="26" t="s">
         <v>402</v>
@@ -9909,9 +9909,9 @@
         <v>384</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="32" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B10" s="32" t="s">
         <v>391</v>
@@ -9932,13 +9932,13 @@
         <v>404</v>
       </c>
       <c r="H10" s="49" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="I10" s="49" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="J10" s="49" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="K10" s="49" t="s">
         <v>409</v>
@@ -9950,7 +9950,7 @@
         <v>392</v>
       </c>
       <c r="N10" s="32" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="O10" s="32" t="s">
         <v>393</v>
@@ -9959,9 +9959,9 @@
         <v>384</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="26" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B11" s="26" t="s">
         <v>391</v>
@@ -9982,13 +9982,13 @@
         <v>404</v>
       </c>
       <c r="H11" s="50" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="I11" s="50" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="J11" s="50" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="K11" s="50" t="s">
         <v>408</v>
@@ -10003,7 +10003,7 @@
         <v>383</v>
       </c>
       <c r="O11" s="26" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="P11" s="26" t="s">
         <v>384</v>
@@ -10021,13 +10021,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6FEC12-ED84-4F38-9B1C-DC3BDC099D3A}">
   <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.85546875" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" customWidth="1"/>
+    <col min="1" max="1" width="40.88671875" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="129" t="s">
         <v>424</v>
       </c>
@@ -10036,180 +10036,180 @@
       <c r="D1" s="51"/>
       <c r="E1" s="51"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="129"/>
       <c r="B2" s="129"/>
       <c r="C2" s="51"/>
       <c r="D2" s="51"/>
       <c r="E2" s="51"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="129"/>
       <c r="B3" s="129"/>
       <c r="C3" s="51"/>
       <c r="D3" s="51"/>
       <c r="E3" s="51"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="105" t="s">
+        <v>629</v>
+      </c>
+      <c r="B4" s="52"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="106" t="s">
+        <v>625</v>
+      </c>
+      <c r="B5" s="14"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="106" t="s">
+        <v>626</v>
+      </c>
+      <c r="B6" s="14"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="106" t="s">
+        <v>627</v>
+      </c>
+      <c r="B7" s="14"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="106" t="s">
+        <v>628</v>
+      </c>
+      <c r="B8" s="14"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="106" t="s">
+        <v>632</v>
+      </c>
+      <c r="B9" s="14"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B10" s="14"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="107" t="s">
         <v>630</v>
       </c>
-      <c r="B4" s="52"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="106" t="s">
-        <v>626</v>
-      </c>
-      <c r="B5" s="14"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="106" t="s">
-        <v>627</v>
-      </c>
-      <c r="B6" s="14"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="106" t="s">
-        <v>628</v>
-      </c>
-      <c r="B7" s="14"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="106" t="s">
-        <v>629</v>
-      </c>
-      <c r="B8" s="14"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="14"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="14"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="107" t="s">
-        <v>631</v>
-      </c>
       <c r="B11" s="14"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>441</v>
       </c>
       <c r="B12" s="14"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B13" s="14"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>504</v>
       </c>
       <c r="B14" s="14"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>539</v>
       </c>
       <c r="B15" s="14"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>506</v>
       </c>
       <c r="B16" s="14"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>574</v>
       </c>
       <c r="B17" s="14"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>507</v>
       </c>
       <c r="B18" s="14"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>508</v>
       </c>
       <c r="B19" s="14"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>522</v>
       </c>
       <c r="B20" s="14"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B21" s="14"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>573</v>
       </c>
       <c r="B22" s="14"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>575</v>
       </c>
       <c r="B23" s="14"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B24" s="14"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>576</v>
-      </c>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B25" s="14"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B26" s="14"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B27" s="14"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>597</v>
+      </c>
+      <c r="B28" s="14"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>598</v>
       </c>
-      <c r="B28" s="14"/>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>599</v>
-      </c>
       <c r="B29" s="14"/>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B30" s="14"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B31" s="14"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B32" s="14"/>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="14"/>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B34" s="14"/>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" s="14"/>
     </row>
   </sheetData>
@@ -10223,34 +10223,34 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6FC119D-A7BC-46FE-BE1D-3900F19AB624}">
   <dimension ref="A1:Z16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" customWidth="1"/>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" customWidth="1"/>
-    <col min="9" max="10" width="9.28515625" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" customWidth="1"/>
-    <col min="12" max="13" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" customWidth="1"/>
+    <col min="9" max="10" width="9.33203125" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" customWidth="1"/>
+    <col min="12" max="13" width="10.109375" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="16" width="12.42578125" customWidth="1"/>
-    <col min="17" max="17" width="12.28515625" customWidth="1"/>
+    <col min="15" max="16" width="12.44140625" customWidth="1"/>
+    <col min="17" max="17" width="12.33203125" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="19" width="14.140625" customWidth="1"/>
-    <col min="20" max="20" width="12.42578125" customWidth="1"/>
-    <col min="21" max="21" width="12.28515625" customWidth="1"/>
-    <col min="22" max="22" width="13.42578125" customWidth="1"/>
-    <col min="23" max="23" width="8.85546875" customWidth="1"/>
-    <col min="24" max="24" width="13.5703125" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" customWidth="1"/>
+    <col min="19" max="19" width="14.109375" customWidth="1"/>
+    <col min="20" max="20" width="12.44140625" customWidth="1"/>
+    <col min="21" max="21" width="12.33203125" customWidth="1"/>
+    <col min="22" max="22" width="13.44140625" customWidth="1"/>
+    <col min="23" max="23" width="8.88671875" customWidth="1"/>
+    <col min="24" max="24" width="13.5546875" customWidth="1"/>
+    <col min="25" max="25" width="11.5546875" customWidth="1"/>
     <col min="26" max="26" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -10330,7 +10330,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -10409,7 +10409,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>410</v>
       </c>
@@ -10491,7 +10491,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>99</v>
       </c>
@@ -10570,7 +10570,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -10652,7 +10652,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>102</v>
       </c>
@@ -10731,7 +10731,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>97</v>
       </c>
@@ -10810,7 +10810,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>93</v>
       </c>
@@ -10889,7 +10889,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -10968,7 +10968,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>89</v>
       </c>
@@ -11047,7 +11047,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>77</v>
       </c>
@@ -11126,7 +11126,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -11205,7 +11205,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>103</v>
       </c>
@@ -11284,7 +11284,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>83</v>
       </c>
@@ -11363,7 +11363,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>444</v>
       </c>
@@ -11442,7 +11442,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>502</v>
       </c>
@@ -11532,31 +11532,31 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{941F1AF2-A8AA-477B-ABE7-7C87546ECF29}">
   <dimension ref="A1:Z17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" customWidth="1"/>
-    <col min="9" max="10" width="9.28515625" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" customWidth="1"/>
-    <col min="12" max="13" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" customWidth="1"/>
+    <col min="9" max="10" width="9.33203125" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" customWidth="1"/>
+    <col min="12" max="13" width="10.109375" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="16" width="12.42578125" customWidth="1"/>
-    <col min="17" max="17" width="12.28515625" customWidth="1"/>
+    <col min="15" max="16" width="12.44140625" customWidth="1"/>
+    <col min="17" max="17" width="12.33203125" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="19" width="14.140625" customWidth="1"/>
-    <col min="20" max="20" width="12.42578125" customWidth="1"/>
-    <col min="21" max="21" width="12.28515625" customWidth="1"/>
-    <col min="22" max="22" width="13.5703125" customWidth="1"/>
-    <col min="24" max="24" width="13.5703125" customWidth="1"/>
+    <col min="19" max="19" width="14.109375" customWidth="1"/>
+    <col min="20" max="20" width="12.44140625" customWidth="1"/>
+    <col min="21" max="21" width="12.33203125" customWidth="1"/>
+    <col min="22" max="22" width="13.5546875" customWidth="1"/>
+    <col min="24" max="24" width="13.5546875" customWidth="1"/>
     <col min="25" max="25" width="12" customWidth="1"/>
-    <col min="26" max="26" width="26.5703125" customWidth="1"/>
+    <col min="26" max="26" width="26.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -11636,7 +11636,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>107</v>
       </c>
@@ -11715,7 +11715,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>421</v>
       </c>
@@ -11794,7 +11794,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" s="57" t="s">
         <v>108</v>
       </c>
@@ -11873,7 +11873,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>110</v>
       </c>
@@ -11952,7 +11952,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>440</v>
       </c>
@@ -12031,7 +12031,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>116</v>
       </c>
@@ -12110,7 +12110,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>106</v>
       </c>
@@ -12189,7 +12189,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>430</v>
       </c>
@@ -12268,7 +12268,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -12347,7 +12347,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>112</v>
       </c>
@@ -12426,7 +12426,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>111</v>
       </c>
@@ -12505,7 +12505,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>114</v>
       </c>
@@ -12584,7 +12584,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>104</v>
       </c>
@@ -12663,7 +12663,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>416</v>
       </c>
@@ -12742,7 +12742,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>511</v>
       </c>
@@ -12821,7 +12821,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>556</v>
       </c>
@@ -12911,34 +12911,34 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E308052D-1B88-4699-843E-12AA607B59B8}">
   <dimension ref="A1:AA58"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="18.5546875" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="11" width="9.28515625" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" customWidth="1"/>
-    <col min="13" max="13" width="10.140625" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" customWidth="1"/>
+    <col min="10" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="11.6640625" customWidth="1"/>
+    <col min="13" max="13" width="10.109375" customWidth="1"/>
+    <col min="14" max="14" width="11.33203125" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.42578125" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" customWidth="1"/>
+    <col min="16" max="17" width="12.44140625" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="14.140625" customWidth="1"/>
-    <col min="21" max="21" width="12.42578125" customWidth="1"/>
-    <col min="22" max="22" width="12.28515625" customWidth="1"/>
-    <col min="23" max="23" width="14.42578125" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" customWidth="1"/>
-    <col min="25" max="25" width="13.5703125" customWidth="1"/>
-    <col min="26" max="26" width="11.7109375" customWidth="1"/>
-    <col min="27" max="27" width="29.7109375" customWidth="1"/>
+    <col min="20" max="20" width="14.109375" customWidth="1"/>
+    <col min="21" max="21" width="12.44140625" customWidth="1"/>
+    <col min="22" max="22" width="12.33203125" customWidth="1"/>
+    <col min="23" max="23" width="14.44140625" customWidth="1"/>
+    <col min="24" max="24" width="11.5546875" customWidth="1"/>
+    <col min="25" max="25" width="13.5546875" customWidth="1"/>
+    <col min="26" max="26" width="11.6640625" customWidth="1"/>
+    <col min="27" max="27" width="29.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -13021,7 +13021,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>205</v>
       </c>
@@ -13103,7 +13103,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>133</v>
       </c>
@@ -13185,7 +13185,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>135</v>
       </c>
@@ -13267,7 +13267,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>136</v>
       </c>
@@ -13349,7 +13349,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>138</v>
       </c>
@@ -13431,7 +13431,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>517</v>
       </c>
@@ -13513,7 +13513,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -13595,7 +13595,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>442</v>
       </c>
@@ -13677,7 +13677,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>443</v>
       </c>
@@ -13759,7 +13759,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>201</v>
       </c>
@@ -13841,7 +13841,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>202</v>
       </c>
@@ -13923,7 +13923,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>139</v>
       </c>
@@ -14008,7 +14008,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>141</v>
       </c>
@@ -14093,7 +14093,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>206</v>
       </c>
@@ -14175,7 +14175,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>147</v>
       </c>
@@ -14257,7 +14257,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>189</v>
       </c>
@@ -14339,7 +14339,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>197</v>
       </c>
@@ -14421,7 +14421,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>207</v>
       </c>
@@ -14503,7 +14503,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>142</v>
       </c>
@@ -14585,7 +14585,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>143</v>
       </c>
@@ -14667,7 +14667,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>415</v>
       </c>
@@ -14749,7 +14749,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>144</v>
       </c>
@@ -14831,7 +14831,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>146</v>
       </c>
@@ -14913,7 +14913,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>174</v>
       </c>
@@ -14995,7 +14995,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>145</v>
       </c>
@@ -15077,7 +15077,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>209</v>
       </c>
@@ -15159,7 +15159,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>210</v>
       </c>
@@ -15241,7 +15241,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>422</v>
       </c>
@@ -15323,7 +15323,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>423</v>
       </c>
@@ -15405,7 +15405,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>200</v>
       </c>
@@ -15487,7 +15487,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>419</v>
       </c>
@@ -15569,7 +15569,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>418</v>
       </c>
@@ -15651,7 +15651,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>130</v>
       </c>
@@ -15733,7 +15733,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>132</v>
       </c>
@@ -15815,7 +15815,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>172</v>
       </c>
@@ -15897,7 +15897,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>131</v>
       </c>
@@ -15979,7 +15979,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>169</v>
       </c>
@@ -16061,7 +16061,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>171</v>
       </c>
@@ -16143,7 +16143,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>173</v>
       </c>
@@ -16225,7 +16225,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>170</v>
       </c>
@@ -16307,7 +16307,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>204</v>
       </c>
@@ -16389,7 +16389,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>193</v>
       </c>
@@ -16471,7 +16471,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>195</v>
       </c>
@@ -16553,7 +16553,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>194</v>
       </c>
@@ -16635,7 +16635,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>190</v>
       </c>
@@ -16717,7 +16717,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>192</v>
       </c>
@@ -16799,7 +16799,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>191</v>
       </c>
@@ -16881,7 +16881,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>198</v>
       </c>
@@ -16963,7 +16963,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>199</v>
       </c>
@@ -17045,7 +17045,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>121</v>
       </c>
@@ -17127,7 +17127,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>122</v>
       </c>
@@ -17209,7 +17209,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>126</v>
       </c>
@@ -17291,7 +17291,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>127</v>
       </c>
@@ -17373,7 +17373,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>128</v>
       </c>
@@ -17455,7 +17455,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>567</v>
       </c>
@@ -17537,9 +17537,9 @@
         <v>117</v>
       </c>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B57">
         <v>22</v>
@@ -17619,9 +17619,9 @@
         <v>137</v>
       </c>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B58">
         <v>23</v>
@@ -17712,34 +17712,34 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E52ABDA0-E560-473A-9AD2-E06CBFB7AB92}">
   <dimension ref="A1:AA30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
-    <col min="3" max="3" width="6.85546875" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="3" max="3" width="6.88671875" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="11" width="9.28515625" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" customWidth="1"/>
-    <col min="13" max="14" width="10.140625" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" customWidth="1"/>
+    <col min="10" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="11.6640625" customWidth="1"/>
+    <col min="13" max="14" width="10.109375" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.42578125" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" customWidth="1"/>
+    <col min="16" max="17" width="12.44140625" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="14.140625" customWidth="1"/>
-    <col min="21" max="21" width="12.42578125" customWidth="1"/>
-    <col min="22" max="22" width="12.28515625" customWidth="1"/>
-    <col min="23" max="23" width="19.140625" customWidth="1"/>
-    <col min="25" max="25" width="13.5703125" customWidth="1"/>
-    <col min="26" max="26" width="11.7109375" customWidth="1"/>
-    <col min="27" max="27" width="21.28515625" customWidth="1"/>
+    <col min="20" max="20" width="14.109375" customWidth="1"/>
+    <col min="21" max="21" width="12.44140625" customWidth="1"/>
+    <col min="22" max="22" width="12.33203125" customWidth="1"/>
+    <col min="23" max="23" width="19.109375" customWidth="1"/>
+    <col min="25" max="25" width="13.5546875" customWidth="1"/>
+    <col min="26" max="26" width="11.6640625" customWidth="1"/>
+    <col min="27" max="27" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -17822,7 +17822,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>148</v>
       </c>
@@ -17904,7 +17904,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>151</v>
       </c>
@@ -17986,7 +17986,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>155</v>
       </c>
@@ -18068,7 +18068,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>154</v>
       </c>
@@ -18150,7 +18150,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>157</v>
       </c>
@@ -18232,7 +18232,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>158</v>
       </c>
@@ -18314,7 +18314,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>159</v>
       </c>
@@ -18396,7 +18396,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>161</v>
       </c>
@@ -18478,7 +18478,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>162</v>
       </c>
@@ -18560,7 +18560,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>163</v>
       </c>
@@ -18642,7 +18642,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>164</v>
       </c>
@@ -18724,7 +18724,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>165</v>
       </c>
@@ -18806,7 +18806,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>505</v>
       </c>
@@ -18891,7 +18891,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>525</v>
       </c>
@@ -18976,9 +18976,9 @@
         <v>526</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="57" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B16">
         <v>24</v>
@@ -19058,9 +19058,9 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B17">
         <v>27</v>
@@ -19140,7 +19140,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X18" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W18,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19150,7 +19150,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X19" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W19,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19160,7 +19160,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X20" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W20,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19170,7 +19170,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X21" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W21,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19180,7 +19180,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X22" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W22,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19190,7 +19190,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X23" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W23,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19200,7 +19200,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X24" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W24,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19210,7 +19210,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X25" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W25,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19220,7 +19220,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X26" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W26,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19230,7 +19230,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X27" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W27,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19240,7 +19240,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X28" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W28,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19250,7 +19250,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X29" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W29,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19260,7 +19260,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.3">
       <c r="X30" t="e">
         <f>INDEX(Caliber!B13:'Caliber'!C23,MATCH(W30,Caliber!B13:'Caliber'!B23,0),2)</f>
         <v>#N/A</v>
@@ -19282,34 +19282,34 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38CF758D-66BB-49AA-8233-CCB9E398E093}">
   <dimension ref="A1:AB12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="11" width="9.28515625" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" customWidth="1"/>
-    <col min="13" max="13" width="10.140625" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" customWidth="1"/>
+    <col min="10" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="11.6640625" customWidth="1"/>
+    <col min="13" max="13" width="10.109375" customWidth="1"/>
+    <col min="14" max="14" width="11.44140625" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.42578125" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" customWidth="1"/>
+    <col min="16" max="17" width="12.44140625" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="14.140625" customWidth="1"/>
-    <col min="21" max="21" width="12.42578125" customWidth="1"/>
-    <col min="22" max="22" width="12.28515625" customWidth="1"/>
-    <col min="23" max="23" width="15.7109375" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" customWidth="1"/>
-    <col min="25" max="25" width="11.28515625" customWidth="1"/>
-    <col min="26" max="26" width="13.5703125" customWidth="1"/>
-    <col min="27" max="27" width="11.7109375" customWidth="1"/>
-    <col min="28" max="28" width="25.140625" customWidth="1"/>
+    <col min="20" max="20" width="14.109375" customWidth="1"/>
+    <col min="21" max="21" width="12.44140625" customWidth="1"/>
+    <col min="22" max="22" width="12.33203125" customWidth="1"/>
+    <col min="23" max="23" width="15.6640625" customWidth="1"/>
+    <col min="24" max="24" width="11.5546875" customWidth="1"/>
+    <col min="25" max="25" width="11.33203125" customWidth="1"/>
+    <col min="26" max="26" width="13.5546875" customWidth="1"/>
+    <col min="27" max="27" width="11.6640625" customWidth="1"/>
+    <col min="28" max="28" width="25.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -19395,7 +19395,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>168</v>
       </c>
@@ -19481,7 +19481,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>176</v>
       </c>
@@ -19570,7 +19570,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>177</v>
       </c>
@@ -19659,7 +19659,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>180</v>
       </c>
@@ -19748,7 +19748,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>181</v>
       </c>
@@ -19837,7 +19837,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>183</v>
       </c>
@@ -19926,7 +19926,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>186</v>
       </c>
@@ -20015,7 +20015,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>187</v>
       </c>
@@ -20104,7 +20104,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>188</v>
       </c>
@@ -20193,7 +20193,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>431</v>
       </c>
@@ -20282,7 +20282,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>566</v>
       </c>
@@ -20379,33 +20379,33 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0094531B-7BBB-4DD3-8835-99962592A6C6}">
   <dimension ref="A1:AB15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" customWidth="1"/>
     <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="11" width="9.28515625" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" customWidth="1"/>
-    <col min="13" max="14" width="10.140625" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" customWidth="1"/>
+    <col min="10" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="11.6640625" customWidth="1"/>
+    <col min="13" max="14" width="10.109375" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.42578125" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" customWidth="1"/>
+    <col min="16" max="17" width="12.44140625" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="17.28515625" customWidth="1"/>
-    <col min="21" max="21" width="12.42578125" customWidth="1"/>
-    <col min="22" max="22" width="12.28515625" customWidth="1"/>
-    <col min="23" max="23" width="18.5703125" customWidth="1"/>
-    <col min="25" max="25" width="13.5703125" customWidth="1"/>
-    <col min="26" max="26" width="11.7109375" customWidth="1"/>
+    <col min="20" max="20" width="17.33203125" customWidth="1"/>
+    <col min="21" max="21" width="12.44140625" customWidth="1"/>
+    <col min="22" max="22" width="12.33203125" customWidth="1"/>
+    <col min="23" max="23" width="18.5546875" customWidth="1"/>
+    <col min="25" max="25" width="13.5546875" customWidth="1"/>
+    <col min="26" max="26" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -20491,7 +20491,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>211</v>
       </c>
@@ -20576,7 +20576,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>215</v>
       </c>
@@ -20661,7 +20661,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>220</v>
       </c>
@@ -20746,7 +20746,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>217</v>
       </c>
@@ -20831,7 +20831,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>216</v>
       </c>
@@ -20916,7 +20916,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>222</v>
       </c>
@@ -21001,7 +21001,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>218</v>
       </c>
@@ -21086,7 +21086,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>429</v>
       </c>
@@ -21171,7 +21171,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>536</v>
       </c>
@@ -21256,7 +21256,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>540</v>
       </c>
@@ -21341,7 +21341,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>541</v>
       </c>
@@ -21426,7 +21426,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>542</v>
       </c>
@@ -21511,7 +21511,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>543</v>
       </c>
@@ -21596,7 +21596,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>544</v>
       </c>
@@ -21694,32 +21694,32 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B2364D-F43A-47E4-8B6C-A03FB84E628E}">
   <dimension ref="A1:AA16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="11" width="9.28515625" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" customWidth="1"/>
-    <col min="13" max="14" width="10.140625" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" customWidth="1"/>
+    <col min="10" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="11.6640625" customWidth="1"/>
+    <col min="13" max="14" width="10.109375" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="17" width="12.42578125" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" customWidth="1"/>
+    <col min="16" max="17" width="12.44140625" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="14.140625" customWidth="1"/>
-    <col min="21" max="21" width="12.42578125" customWidth="1"/>
-    <col min="22" max="22" width="12.28515625" customWidth="1"/>
-    <col min="23" max="23" width="15.5703125" customWidth="1"/>
-    <col min="25" max="25" width="13.5703125" customWidth="1"/>
-    <col min="26" max="26" width="11.7109375" customWidth="1"/>
-    <col min="27" max="27" width="17.85546875" customWidth="1"/>
+    <col min="20" max="20" width="14.109375" customWidth="1"/>
+    <col min="21" max="21" width="12.44140625" customWidth="1"/>
+    <col min="22" max="22" width="12.33203125" customWidth="1"/>
+    <col min="23" max="23" width="15.5546875" customWidth="1"/>
+    <col min="25" max="25" width="13.5546875" customWidth="1"/>
+    <col min="26" max="26" width="11.6640625" customWidth="1"/>
+    <col min="27" max="27" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -21802,7 +21802,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>223</v>
       </c>
@@ -21887,7 +21887,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>225</v>
       </c>
@@ -21972,7 +21972,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>229</v>
       </c>
@@ -22057,7 +22057,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>232</v>
       </c>
@@ -22142,7 +22142,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>233</v>
       </c>
@@ -22227,7 +22227,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>234</v>
       </c>
@@ -22312,7 +22312,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>503</v>
       </c>
@@ -22397,7 +22397,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>572</v>
       </c>
@@ -22479,12 +22479,12 @@
         <v>82</v>
       </c>
       <c r="AA9" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B10">
         <v>48</v>
@@ -22561,13 +22561,13 @@
         <v>0.4</v>
       </c>
       <c r="Z10" t="s">
+        <v>594</v>
+      </c>
+      <c r="AA10" t="s">
         <v>595</v>
       </c>
-      <c r="AA10" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="X11" t="e" cm="1">
         <f t="array" aca="1" ref="X11" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -22577,7 +22577,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="X12" t="e" cm="1">
         <f t="array" aca="1" ref="X12" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -22587,7 +22587,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="X13" t="e" cm="1">
         <f t="array" aca="1" ref="X13" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -22597,7 +22597,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="X14" t="e" cm="1">
         <f t="array" aca="1" ref="X14" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -22607,7 +22607,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="X15" t="e" cm="1">
         <f t="array" aca="1" ref="X15" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -22617,7 +22617,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="X16" t="e" cm="1">
         <f t="array" aca="1" ref="X16" ca="1">INDEX(Caliber!B35:'Caliber'!C43,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B43,0),2)</f>
         <v>#N/A</v>
@@ -22638,12 +22638,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD9C29F4-F90E-490E-8D34-BB5E6787CD6C}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>412</v>
       </c>

</xml_diff>

<commit_message>
Technical no longer spawns on edge of the map
Technical no longer spawns on edge of the map (when possible).
mapScritpts.rul split into mapScripts, mapScripts_Obj, and mapScripts_Tec for readability.
Ballistic knife melee stats now properly mirror knife stats again.
Fixed weight on 6x VOG-25 caseless grenades.
Fixed some missions executionOdds (house raid and office are now once a month).
</commit_message>
<xml_diff>
--- a/CTO Wepon stat spreadsheet.xlsx
+++ b/CTO Wepon stat spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethan\Documents\OpenXcom\mods\IDT_Counter_Terrorist_Operations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E48FB3C-DDEF-448B-BDF8-DC0A45EB1FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39ACC6E9-9319-413F-BEEF-A4011A7C41D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="6" activeTab="11" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="11" xr2:uid="{5CCF0F11-6EA0-4BA3-9FDA-51D6C50FE267}"/>
   </bookViews>
   <sheets>
     <sheet name="Caliber" sheetId="1" r:id="rId1"/>
@@ -257,7 +257,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1927" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1927" uniqueCount="644">
   <si>
     <t>Name</t>
   </si>
@@ -1300,10 +1300,6 @@
   </si>
   <si>
     <t>Player</t>
-  </si>
-  <si>
-    <t>European/American
-Generic</t>
   </si>
   <si>
     <t>Private Security</t>
@@ -4664,7 +4660,7 @@
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C10">
         <v>40</v>
@@ -4679,13 +4675,13 @@
         <v>1</v>
       </c>
       <c r="I10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="56"/>
       <c r="B11" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C11">
         <v>30</v>
@@ -5119,7 +5115,7 @@
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
       <c r="B24" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C24">
         <v>40</v>
@@ -5347,7 +5343,7 @@
     <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A29" s="7"/>
       <c r="B29" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C29">
         <v>18</v>
@@ -5368,13 +5364,13 @@
         <v>2</v>
       </c>
       <c r="I29" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" s="7"/>
       <c r="B30" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C30">
         <v>10</v>
@@ -5395,7 +5391,7 @@
         <v>11</v>
       </c>
       <c r="I30" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="M30" s="12" t="s">
         <v>41</v>
@@ -5874,7 +5870,7 @@
     <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" s="9"/>
       <c r="B44" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C44">
         <v>95</v>
@@ -5892,13 +5888,13 @@
         <v>3</v>
       </c>
       <c r="I44" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" s="9"/>
       <c r="B45" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C45">
         <v>40</v>
@@ -5916,13 +5912,13 @@
         <v>3</v>
       </c>
       <c r="I45" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" s="9"/>
       <c r="B46" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C46">
         <v>40</v>
@@ -5948,7 +5944,7 @@
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A48" s="53" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B48" t="s">
         <v>0</v>
@@ -5978,7 +5974,7 @@
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="54"/>
       <c r="B49" s="14" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C49">
         <v>40</v>
@@ -5993,7 +5989,7 @@
         <v>7</v>
       </c>
       <c r="I49" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -7480,34 +7476,34 @@
         <v>290</v>
       </c>
       <c r="B32" s="32">
+        <v>35</v>
+      </c>
+      <c r="C32" s="32">
         <v>30</v>
       </c>
-      <c r="C32" s="32">
-        <v>25</v>
-      </c>
       <c r="D32" s="32">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E32" s="32">
         <v>20</v>
       </c>
       <c r="F32" s="21">
-        <v>-20</v>
+        <v>-10</v>
       </c>
       <c r="G32" s="22">
-        <v>-30</v>
+        <v>-25</v>
       </c>
       <c r="H32" s="23">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I32" s="24">
-        <v>-40</v>
+        <v>-10</v>
       </c>
       <c r="J32" s="25">
-        <v>-20</v>
+        <v>-15</v>
       </c>
       <c r="K32" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L32" s="32">
         <v>0.05</v>
@@ -7647,15 +7643,15 @@
       <c r="N2" s="38"/>
       <c r="O2" s="38"/>
       <c r="P2" s="32" t="s">
+        <v>563</v>
+      </c>
+      <c r="Q2" s="32" t="s">
         <v>564</v>
-      </c>
-      <c r="Q2" s="32" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="113" t="s">
-        <v>335</v>
+        <v>380</v>
       </c>
       <c r="B3" s="26" t="s">
         <v>298</v>
@@ -7691,7 +7687,7 @@
         <v>50</v>
       </c>
       <c r="M3" s="26" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="N3" s="26" t="s">
         <v>313</v>
@@ -7738,7 +7734,7 @@
         <v>40</v>
       </c>
       <c r="M4" s="32" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="N4" s="32" t="s">
         <v>313</v>
@@ -7789,7 +7785,7 @@
         <v>318</v>
       </c>
       <c r="O5" s="26" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="P5" s="39"/>
       <c r="Q5" s="39"/>
@@ -7834,7 +7830,7 @@
         <v>316</v>
       </c>
       <c r="O6" s="32" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="P6" s="38"/>
       <c r="Q6" s="38"/>
@@ -7875,7 +7871,7 @@
         <v>20</v>
       </c>
       <c r="M7" s="26" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="N7" s="26" t="s">
         <v>320</v>
@@ -7926,7 +7922,7 @@
         <v>322</v>
       </c>
       <c r="O8" s="32" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="P8" s="38"/>
       <c r="Q8" s="38"/>
@@ -7971,7 +7967,7 @@
         <v>320</v>
       </c>
       <c r="O9" s="26" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="P9" s="39"/>
       <c r="Q9" s="39"/>
@@ -8016,14 +8012,14 @@
         <v>325</v>
       </c>
       <c r="O10" s="32" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="P10" s="38"/>
       <c r="Q10" s="38"/>
     </row>
     <row r="11" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="113" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B11" s="26" t="s">
         <v>298</v>
@@ -8080,7 +8076,7 @@
         <v>50</v>
       </c>
       <c r="M12" s="32" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="N12" s="32" t="s">
         <v>326</v>
@@ -8174,7 +8170,7 @@
         <v>30</v>
       </c>
       <c r="M14" s="32" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="N14" s="32" t="s">
         <v>313</v>
@@ -8268,7 +8264,7 @@
         <v>30</v>
       </c>
       <c r="M16" s="32" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="N16" s="32" t="s">
         <v>313</v>
@@ -8315,7 +8311,7 @@
         <v>30</v>
       </c>
       <c r="M17" s="26" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="N17" s="26" t="s">
         <v>313</v>
@@ -8362,7 +8358,7 @@
         <v>30</v>
       </c>
       <c r="M18" s="32" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="N18" s="32" t="s">
         <v>331</v>
@@ -8375,10 +8371,10 @@
     </row>
     <row r="19" spans="1:17" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="26" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C19" s="94">
         <v>100</v>
@@ -8411,13 +8407,13 @@
         <v>50</v>
       </c>
       <c r="M19" s="91" t="s">
+        <v>622</v>
+      </c>
+      <c r="N19" s="32" t="s">
         <v>623</v>
       </c>
-      <c r="N19" s="32" t="s">
-        <v>624</v>
-      </c>
       <c r="O19" s="32" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="P19" s="103"/>
       <c r="Q19" s="103"/>
@@ -8451,22 +8447,22 @@
         <v>333</v>
       </c>
       <c r="B1" s="44" t="s">
+        <v>336</v>
+      </c>
+      <c r="C1" s="44" t="s">
         <v>337</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="D1" s="44" t="s">
         <v>338</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="E1" s="44" t="s">
         <v>339</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="F1" s="44" t="s">
         <v>340</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="G1" s="44" t="s">
         <v>341</v>
-      </c>
-      <c r="G1" s="44" t="s">
-        <v>342</v>
       </c>
       <c r="H1" s="44" t="s">
         <v>237</v>
@@ -8475,7 +8471,7 @@
     </row>
     <row r="2" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="119" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B2" s="119" t="s">
         <v>298</v>
@@ -8484,19 +8480,19 @@
         <v>298</v>
       </c>
       <c r="D2" s="45" t="s">
+        <v>342</v>
+      </c>
+      <c r="E2" s="45" t="s">
+        <v>454</v>
+      </c>
+      <c r="F2" s="45" t="s">
+        <v>454</v>
+      </c>
+      <c r="G2" s="45" t="s">
         <v>343</v>
       </c>
-      <c r="E2" s="45" t="s">
-        <v>455</v>
-      </c>
-      <c r="F2" s="45" t="s">
-        <v>455</v>
-      </c>
-      <c r="G2" s="45" t="s">
+      <c r="H2" s="119" t="s">
         <v>344</v>
-      </c>
-      <c r="H2" s="119" t="s">
-        <v>345</v>
       </c>
       <c r="I2" s="62"/>
     </row>
@@ -8505,16 +8501,16 @@
       <c r="B3" s="117"/>
       <c r="C3" s="117"/>
       <c r="D3" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E3" s="46" t="s">
+        <v>455</v>
+      </c>
+      <c r="F3" s="46" t="s">
+        <v>455</v>
+      </c>
+      <c r="G3" s="46" t="s">
         <v>456</v>
-      </c>
-      <c r="F3" s="46" t="s">
-        <v>456</v>
-      </c>
-      <c r="G3" s="46" t="s">
-        <v>457</v>
       </c>
       <c r="H3" s="117"/>
     </row>
@@ -8523,16 +8519,16 @@
       <c r="B4" s="117"/>
       <c r="C4" s="117"/>
       <c r="D4" s="60" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E4" s="60" t="s">
+        <v>568</v>
+      </c>
+      <c r="F4" s="60" t="s">
+        <v>567</v>
+      </c>
+      <c r="G4" s="60" t="s">
         <v>569</v>
-      </c>
-      <c r="F4" s="60" t="s">
-        <v>568</v>
-      </c>
-      <c r="G4" s="60" t="s">
-        <v>570</v>
       </c>
       <c r="H4" s="117"/>
     </row>
@@ -8545,19 +8541,19 @@
         <v>299</v>
       </c>
       <c r="D5" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E5" s="61" t="s">
+        <v>556</v>
+      </c>
+      <c r="F5" s="61" t="s">
         <v>557</v>
       </c>
-      <c r="F5" s="61" t="s">
+      <c r="G5" s="61" t="s">
         <v>558</v>
       </c>
-      <c r="G5" s="61" t="s">
-        <v>559</v>
-      </c>
       <c r="H5" s="116" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8565,16 +8561,16 @@
       <c r="B6" s="117"/>
       <c r="C6" s="117"/>
       <c r="D6" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F6" s="46" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="G6" s="46" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="H6" s="117"/>
     </row>
@@ -8583,41 +8579,41 @@
       <c r="B7" s="118"/>
       <c r="C7" s="118"/>
       <c r="D7" s="59" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E7" s="59" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F7" s="59" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G7" s="59" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="H7" s="118"/>
     </row>
     <row r="8" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="117"/>
       <c r="B8" s="116" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C8" s="116" t="s">
         <v>315</v>
       </c>
       <c r="D8" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E8" s="61" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F8" s="61" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G8" s="61" t="s">
         <v>220</v>
       </c>
       <c r="H8" s="116" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8625,16 +8621,16 @@
       <c r="B9" s="117"/>
       <c r="C9" s="117"/>
       <c r="D9" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="F9" s="46" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="G9" s="46" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="H9" s="117"/>
     </row>
@@ -8643,41 +8639,41 @@
       <c r="B10" s="118"/>
       <c r="C10" s="118"/>
       <c r="D10" s="59" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E10" s="59" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F10" s="59" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G10" s="59" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H10" s="118"/>
     </row>
     <row r="11" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="117"/>
       <c r="B11" s="116" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C11" s="116" t="s">
         <v>317</v>
       </c>
       <c r="D11" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E11" s="61" t="s">
+        <v>586</v>
+      </c>
+      <c r="F11" s="61" t="s">
         <v>587</v>
       </c>
-      <c r="F11" s="61" t="s">
-        <v>588</v>
-      </c>
       <c r="G11" s="61" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H11" s="116" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8685,13 +8681,13 @@
       <c r="B12" s="117"/>
       <c r="C12" s="117"/>
       <c r="D12" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E12" s="46" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="F12" s="46" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="G12" s="46" t="s">
         <v>203</v>
@@ -8703,41 +8699,41 @@
       <c r="B13" s="117"/>
       <c r="C13" s="117"/>
       <c r="D13" s="60" t="s">
+        <v>346</v>
+      </c>
+      <c r="E13" s="60" t="s">
+        <v>354</v>
+      </c>
+      <c r="F13" s="60" t="s">
+        <v>349</v>
+      </c>
+      <c r="G13" s="60" t="s">
         <v>347</v>
-      </c>
-      <c r="E13" s="60" t="s">
-        <v>355</v>
-      </c>
-      <c r="F13" s="60" t="s">
-        <v>350</v>
-      </c>
-      <c r="G13" s="60" t="s">
-        <v>348</v>
       </c>
       <c r="H13" s="117"/>
     </row>
     <row r="14" spans="1:9" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="117"/>
       <c r="B14" s="116" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C14" s="116" t="s">
         <v>319</v>
       </c>
       <c r="D14" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E14" s="61" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="F14" s="61" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="G14" s="61" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="H14" s="116" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8745,16 +8741,16 @@
       <c r="B15" s="117"/>
       <c r="C15" s="117"/>
       <c r="D15" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E15" s="46" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F15" s="46" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="G15" s="46" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H15" s="117"/>
     </row>
@@ -8763,29 +8759,29 @@
       <c r="B16" s="118"/>
       <c r="C16" s="118"/>
       <c r="D16" s="59" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E16" s="59" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F16" s="59" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="G16" s="59" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="H16" s="118"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="117"/>
       <c r="B17" s="116" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C17" s="116" t="s">
         <v>321</v>
       </c>
       <c r="D17" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E17" s="61" t="s">
         <v>11</v>
@@ -8797,7 +8793,7 @@
         <v>111</v>
       </c>
       <c r="H17" s="116" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8805,16 +8801,16 @@
       <c r="B18" s="117"/>
       <c r="C18" s="117"/>
       <c r="D18" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E18" s="46" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F18" s="46" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="G18" s="46" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="H18" s="117"/>
     </row>
@@ -8823,41 +8819,41 @@
       <c r="B19" s="118"/>
       <c r="C19" s="118"/>
       <c r="D19" s="59" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E19" s="59" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F19" s="59" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G19" s="59" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H19" s="118"/>
     </row>
     <row r="20" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="117"/>
       <c r="B20" s="116" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C20" s="116" t="s">
         <v>323</v>
       </c>
       <c r="D20" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E20" s="61" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F20" s="61" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="G20" s="61" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="H20" s="116" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8865,16 +8861,16 @@
       <c r="B21" s="117"/>
       <c r="C21" s="117"/>
       <c r="D21" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E21" s="46" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="F21" s="46" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="G21" s="46" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="H21" s="117"/>
     </row>
@@ -8883,41 +8879,41 @@
       <c r="B22" s="117"/>
       <c r="C22" s="117"/>
       <c r="D22" s="60" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E22" s="60" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="F22" s="60" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="G22" s="60" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H22" s="120"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="117"/>
       <c r="B23" s="116" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C23" s="116" t="s">
         <v>324</v>
       </c>
       <c r="D23" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E23" s="61" t="s">
         <v>148</v>
       </c>
       <c r="F23" s="61" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="G23" s="61" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="H23" s="119" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -8925,16 +8921,16 @@
       <c r="B24" s="117"/>
       <c r="C24" s="117"/>
       <c r="D24" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E24" s="65" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="F24" s="46" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="G24" s="46" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="H24" s="117"/>
     </row>
@@ -8943,22 +8939,22 @@
       <c r="B25" s="120"/>
       <c r="C25" s="120"/>
       <c r="D25" s="47" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E25" s="47" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="F25" s="47" t="s">
+        <v>450</v>
+      </c>
+      <c r="G25" s="47" t="s">
         <v>451</v>
-      </c>
-      <c r="G25" s="47" t="s">
-        <v>452</v>
       </c>
       <c r="H25" s="120"/>
     </row>
     <row r="26" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="119" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B26" s="119" t="s">
         <v>298</v>
@@ -8967,7 +8963,7 @@
         <v>298</v>
       </c>
       <c r="D26" s="45" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E26" s="121"/>
       <c r="F26" s="122"/>
@@ -8979,7 +8975,7 @@
       <c r="B27" s="117"/>
       <c r="C27" s="117"/>
       <c r="D27" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E27" s="121"/>
       <c r="F27" s="122"/>
@@ -8991,7 +8987,7 @@
       <c r="B28" s="117"/>
       <c r="C28" s="117"/>
       <c r="D28" s="60" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E28" s="126"/>
       <c r="F28" s="127"/>
@@ -9007,19 +9003,19 @@
         <v>299</v>
       </c>
       <c r="D29" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E29" s="75" t="s">
+        <v>498</v>
+      </c>
+      <c r="F29" s="64" t="s">
         <v>499</v>
       </c>
-      <c r="F29" s="64" t="s">
-        <v>500</v>
-      </c>
       <c r="G29" s="76" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="H29" s="116" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9027,16 +9023,16 @@
       <c r="B30" s="117"/>
       <c r="C30" s="117"/>
       <c r="D30" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E30" s="79" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="F30" s="71" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="G30" s="77" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="H30" s="117"/>
     </row>
@@ -9045,41 +9041,41 @@
       <c r="B31" s="118"/>
       <c r="C31" s="118"/>
       <c r="D31" s="59" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E31" s="78" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F31" s="74" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="G31" s="78" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="H31" s="118"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="117"/>
       <c r="B32" s="117" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C32" s="117" t="s">
         <v>328</v>
       </c>
       <c r="D32" s="58" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E32" s="73" t="s">
+        <v>492</v>
+      </c>
+      <c r="F32" s="80" t="s">
         <v>493</v>
       </c>
-      <c r="F32" s="80" t="s">
+      <c r="G32" s="73" t="s">
         <v>494</v>
       </c>
-      <c r="G32" s="73" t="s">
-        <v>495</v>
-      </c>
       <c r="H32" s="117" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9087,16 +9083,16 @@
       <c r="B33" s="117"/>
       <c r="C33" s="117"/>
       <c r="D33" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E33" s="79" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F33" s="71" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G33" s="79" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H33" s="117"/>
     </row>
@@ -9105,41 +9101,41 @@
       <c r="B34" s="117"/>
       <c r="C34" s="117"/>
       <c r="D34" s="60" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E34" s="67" t="s">
+        <v>489</v>
+      </c>
+      <c r="F34" s="81" t="s">
         <v>490</v>
       </c>
-      <c r="F34" s="81" t="s">
-        <v>491</v>
-      </c>
       <c r="G34" s="67" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="H34" s="117"/>
     </row>
     <row r="35" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="117"/>
       <c r="B35" s="116" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C35" s="116" t="s">
         <v>317</v>
       </c>
       <c r="D35" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E35" s="75" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F35" s="75" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G35" s="75" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="H35" s="116" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9147,16 +9143,16 @@
       <c r="B36" s="117"/>
       <c r="C36" s="117"/>
       <c r="D36" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E36" s="79" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F36" s="79" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="G36" s="79" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="H36" s="117"/>
     </row>
@@ -9165,41 +9161,41 @@
       <c r="B37" s="117"/>
       <c r="C37" s="117"/>
       <c r="D37" s="60" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E37" s="90" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F37" s="90" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="G37" s="90" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="H37" s="117"/>
     </row>
     <row r="38" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="117"/>
       <c r="B38" s="116" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C38" s="116" t="s">
         <v>287</v>
       </c>
       <c r="D38" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E38" s="63" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="F38" s="85" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="G38" s="63" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="H38" s="116" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9207,16 +9203,16 @@
       <c r="B39" s="117"/>
       <c r="C39" s="117"/>
       <c r="D39" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E39" s="79" t="s">
+        <v>472</v>
+      </c>
+      <c r="F39" s="71" t="s">
         <v>473</v>
       </c>
-      <c r="F39" s="71" t="s">
-        <v>474</v>
-      </c>
       <c r="G39" s="79" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="H39" s="117"/>
     </row>
@@ -9225,41 +9221,41 @@
       <c r="B40" s="117"/>
       <c r="C40" s="117"/>
       <c r="D40" s="60" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E40" s="67" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="F40" s="81" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="G40" s="67" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="H40" s="117"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="117"/>
       <c r="B41" s="116" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C41" s="116" t="s">
         <v>321</v>
       </c>
       <c r="D41" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E41" s="86" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="F41" s="80" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="G41" s="86" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="H41" s="116" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9267,16 +9263,16 @@
       <c r="B42" s="117"/>
       <c r="C42" s="117"/>
       <c r="D42" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E42" s="87" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F42" s="88" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="G42" s="87" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="H42" s="117"/>
     </row>
@@ -9285,41 +9281,41 @@
       <c r="B43" s="117"/>
       <c r="C43" s="117"/>
       <c r="D43" s="60" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E43" s="67" t="s">
+        <v>466</v>
+      </c>
+      <c r="F43" s="89" t="s">
         <v>467</v>
       </c>
-      <c r="F43" s="89" t="s">
-        <v>468</v>
-      </c>
       <c r="G43" s="67" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H43" s="117"/>
     </row>
     <row r="44" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="117"/>
       <c r="B44" s="116" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C44" s="116" t="s">
         <v>315</v>
       </c>
       <c r="D44" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E44" s="68" t="s">
+        <v>487</v>
+      </c>
+      <c r="F44" s="82" t="s">
         <v>488</v>
       </c>
-      <c r="F44" s="82" t="s">
-        <v>489</v>
-      </c>
       <c r="G44" s="68" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="H44" s="116" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9327,16 +9323,16 @@
       <c r="B45" s="117"/>
       <c r="C45" s="117"/>
       <c r="D45" s="66" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E45" s="69" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F45" s="69" t="s">
+        <v>548</v>
+      </c>
+      <c r="G45" s="69" t="s">
         <v>549</v>
-      </c>
-      <c r="G45" s="69" t="s">
-        <v>550</v>
       </c>
       <c r="H45" s="117"/>
     </row>
@@ -9345,41 +9341,41 @@
       <c r="B46" s="117"/>
       <c r="C46" s="117"/>
       <c r="D46" s="60" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E46" s="67" t="s">
+        <v>546</v>
+      </c>
+      <c r="F46" s="81" t="s">
         <v>547</v>
       </c>
-      <c r="F46" s="81" t="s">
-        <v>548</v>
-      </c>
       <c r="G46" s="67" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="H46" s="117"/>
     </row>
     <row r="47" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="117"/>
       <c r="B47" s="116" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C47" s="116" t="s">
         <v>324</v>
       </c>
       <c r="D47" s="61" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E47" s="63" t="s">
         <v>158</v>
       </c>
       <c r="F47" s="80" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="G47" s="63" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="H47" s="116" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -9387,16 +9383,16 @@
       <c r="B48" s="117"/>
       <c r="C48" s="117"/>
       <c r="D48" s="46" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E48" s="70" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F48" s="83" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="G48" s="70" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="H48" s="117"/>
     </row>
@@ -9405,16 +9401,16 @@
       <c r="B49" s="120"/>
       <c r="C49" s="120"/>
       <c r="D49" s="47" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E49" s="84" t="s">
+        <v>483</v>
+      </c>
+      <c r="F49" s="72" t="s">
         <v>484</v>
       </c>
-      <c r="F49" s="72" t="s">
-        <v>485</v>
-      </c>
       <c r="G49" s="84" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="H49" s="120"/>
     </row>
@@ -9500,113 +9496,113 @@
         <v>236</v>
       </c>
       <c r="B1" s="20" t="s">
+        <v>363</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>364</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="D1" s="20" t="s">
         <v>365</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="E1" s="20" t="s">
         <v>366</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="F1" s="20" t="s">
         <v>367</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="G1" s="20" t="s">
         <v>368</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="H1" s="20" t="s">
         <v>369</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="I1" s="20" t="s">
         <v>370</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="J1" s="20" t="s">
         <v>371</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="K1" s="20" t="s">
         <v>372</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="L1" s="20" t="s">
         <v>373</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="M1" s="20" t="s">
         <v>374</v>
       </c>
-      <c r="M1" s="20" t="s">
+      <c r="N1" s="20" t="s">
         <v>375</v>
       </c>
-      <c r="N1" s="20" t="s">
+      <c r="O1" s="20" t="s">
         <v>376</v>
       </c>
-      <c r="O1" s="20" t="s">
+      <c r="P1" s="20" t="s">
         <v>377</v>
-      </c>
-      <c r="P1" s="20" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="32" t="s">
+        <v>378</v>
+      </c>
+      <c r="B2" s="32" t="s">
         <v>379</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>380</v>
       </c>
       <c r="C2" s="32">
         <v>3</v>
       </c>
       <c r="D2" s="32" t="s">
+        <v>380</v>
+      </c>
+      <c r="E2" s="32">
+        <v>0</v>
+      </c>
+      <c r="F2" s="32">
+        <v>0</v>
+      </c>
+      <c r="G2" s="49">
+        <v>0</v>
+      </c>
+      <c r="H2" s="49" t="s">
+        <v>404</v>
+      </c>
+      <c r="I2" s="49" t="s">
+        <v>404</v>
+      </c>
+      <c r="J2" s="49" t="s">
+        <v>402</v>
+      </c>
+      <c r="K2" s="49">
+        <v>0</v>
+      </c>
+      <c r="L2" s="49">
+        <v>0</v>
+      </c>
+      <c r="M2" s="32" t="s">
         <v>381</v>
       </c>
-      <c r="E2" s="32">
-        <v>0</v>
-      </c>
-      <c r="F2" s="32">
-        <v>0</v>
-      </c>
-      <c r="G2" s="49">
-        <v>0</v>
-      </c>
-      <c r="H2" s="49" t="s">
-        <v>405</v>
-      </c>
-      <c r="I2" s="49" t="s">
-        <v>405</v>
-      </c>
-      <c r="J2" s="49" t="s">
-        <v>403</v>
-      </c>
-      <c r="K2" s="49">
-        <v>0</v>
-      </c>
-      <c r="L2" s="49">
-        <v>0</v>
-      </c>
-      <c r="M2" s="32" t="s">
+      <c r="N2" s="32" t="s">
         <v>382</v>
-      </c>
-      <c r="N2" s="32" t="s">
-        <v>383</v>
       </c>
       <c r="O2" s="32">
         <v>300</v>
       </c>
       <c r="P2" s="32" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="C3" s="26">
         <v>12</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E3" s="26">
         <v>0</v>
@@ -9618,13 +9614,13 @@
         <v>0</v>
       </c>
       <c r="H3" s="50" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="I3" s="50" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="J3" s="50" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="K3" s="50">
         <v>0</v>
@@ -9633,80 +9629,80 @@
         <v>0</v>
       </c>
       <c r="M3" s="26" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="N3" s="26" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="O3" s="26">
         <v>400</v>
       </c>
       <c r="P3" s="26" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="32" t="s">
+        <v>386</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>600</v>
+      </c>
+      <c r="C4" s="32">
+        <v>0</v>
+      </c>
+      <c r="D4" s="32" t="s">
+        <v>380</v>
+      </c>
+      <c r="E4" s="32">
+        <v>0</v>
+      </c>
+      <c r="F4" s="32">
+        <v>1</v>
+      </c>
+      <c r="G4" s="49">
+        <v>1</v>
+      </c>
+      <c r="H4" s="49" t="s">
+        <v>405</v>
+      </c>
+      <c r="I4" s="49" t="s">
+        <v>405</v>
+      </c>
+      <c r="J4" s="49" t="s">
+        <v>601</v>
+      </c>
+      <c r="K4" s="49">
+        <v>0</v>
+      </c>
+      <c r="L4" s="49">
+        <v>0</v>
+      </c>
+      <c r="M4" s="32" t="s">
+        <v>385</v>
+      </c>
+      <c r="N4" s="32" t="s">
         <v>387</v>
       </c>
-      <c r="B4" s="32" t="s">
-        <v>601</v>
-      </c>
-      <c r="C4" s="32">
-        <v>0</v>
-      </c>
-      <c r="D4" s="32" t="s">
-        <v>381</v>
-      </c>
-      <c r="E4" s="32">
-        <v>0</v>
-      </c>
-      <c r="F4" s="32">
-        <v>1</v>
-      </c>
-      <c r="G4" s="49">
-        <v>1</v>
-      </c>
-      <c r="H4" s="49" t="s">
-        <v>406</v>
-      </c>
-      <c r="I4" s="49" t="s">
-        <v>406</v>
-      </c>
-      <c r="J4" s="49" t="s">
-        <v>602</v>
-      </c>
-      <c r="K4" s="49">
-        <v>0</v>
-      </c>
-      <c r="L4" s="49">
-        <v>0</v>
-      </c>
-      <c r="M4" s="32" t="s">
-        <v>386</v>
-      </c>
-      <c r="N4" s="32" t="s">
+      <c r="O4" s="32" t="s">
         <v>388</v>
       </c>
-      <c r="O4" s="32" t="s">
-        <v>389</v>
-      </c>
       <c r="P4" s="32" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
+        <v>389</v>
+      </c>
+      <c r="B5" s="26" t="s">
         <v>390</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>391</v>
       </c>
       <c r="C5" s="26">
         <v>20</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E5" s="26">
         <v>0</v>
@@ -9715,48 +9711,48 @@
         <v>1</v>
       </c>
       <c r="G5" s="50" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="H5" s="50" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="I5" s="50" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="J5" s="50" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="K5" s="50" t="s">
+        <v>407</v>
+      </c>
+      <c r="L5" s="50" t="s">
         <v>408</v>
       </c>
-      <c r="L5" s="50" t="s">
-        <v>409</v>
-      </c>
       <c r="M5" s="26" t="s">
+        <v>391</v>
+      </c>
+      <c r="N5" s="26" t="s">
+        <v>382</v>
+      </c>
+      <c r="O5" s="26" t="s">
         <v>392</v>
       </c>
-      <c r="N5" s="26" t="s">
+      <c r="P5" s="26" t="s">
         <v>383</v>
-      </c>
-      <c r="O5" s="26" t="s">
-        <v>393</v>
-      </c>
-      <c r="P5" s="26" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="32" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C6" s="32">
         <v>10</v>
       </c>
       <c r="D6" s="32" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E6" s="32">
         <v>0</v>
@@ -9765,48 +9761,48 @@
         <v>1</v>
       </c>
       <c r="G6" s="49" t="s">
+        <v>403</v>
+      </c>
+      <c r="H6" s="49" t="s">
+        <v>603</v>
+      </c>
+      <c r="I6" s="49" t="s">
+        <v>642</v>
+      </c>
+      <c r="J6" s="49" t="s">
+        <v>642</v>
+      </c>
+      <c r="K6" s="49" t="s">
+        <v>407</v>
+      </c>
+      <c r="L6" s="49" t="s">
         <v>404</v>
       </c>
-      <c r="H6" s="49" t="s">
-        <v>604</v>
-      </c>
-      <c r="I6" s="49" t="s">
-        <v>643</v>
-      </c>
-      <c r="J6" s="49" t="s">
-        <v>643</v>
-      </c>
-      <c r="K6" s="49" t="s">
-        <v>408</v>
-      </c>
-      <c r="L6" s="49" t="s">
-        <v>405</v>
-      </c>
       <c r="M6" s="32" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="N6" s="32" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="O6" s="32">
         <v>500</v>
       </c>
       <c r="P6" s="32" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="26" t="s">
+        <v>394</v>
+      </c>
+      <c r="B7" s="26" t="s">
         <v>395</v>
       </c>
-      <c r="B7" s="26" t="s">
-        <v>396</v>
-      </c>
       <c r="C7" s="26">
         <v>0</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E7" s="26">
         <v>1</v>
@@ -9815,48 +9811,48 @@
         <v>2</v>
       </c>
       <c r="G7" s="50" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H7" s="50" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="I7" s="50" t="s">
+        <v>406</v>
+      </c>
+      <c r="J7" s="50" t="s">
+        <v>606</v>
+      </c>
+      <c r="K7" s="50" t="s">
         <v>407</v>
       </c>
-      <c r="J7" s="50" t="s">
-        <v>607</v>
-      </c>
-      <c r="K7" s="50" t="s">
-        <v>408</v>
-      </c>
       <c r="L7" s="50" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="M7" s="26" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="N7" s="26" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="O7" s="26" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="P7" s="26" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="32" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B8" s="32" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C8" s="32">
         <v>4</v>
       </c>
       <c r="D8" s="32" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E8" s="32">
         <v>0</v>
@@ -9868,181 +9864,181 @@
         <v>0</v>
       </c>
       <c r="H8" s="49" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I8" s="49" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="J8" s="49" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="K8" s="49" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="L8" s="49">
         <v>0</v>
       </c>
       <c r="M8" s="32" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="N8" s="32" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="O8" s="32" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="P8" s="32" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="26" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="C9" s="26">
         <v>12</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="E9" s="26">
         <v>0</v>
       </c>
       <c r="F9" s="50" t="s">
+        <v>404</v>
+      </c>
+      <c r="G9" s="50" t="s">
         <v>405</v>
       </c>
-      <c r="G9" s="50" t="s">
-        <v>406</v>
-      </c>
       <c r="H9" s="50" t="s">
+        <v>601</v>
+      </c>
+      <c r="I9" s="50" t="s">
+        <v>601</v>
+      </c>
+      <c r="J9" s="50" t="s">
         <v>602</v>
       </c>
-      <c r="I9" s="50" t="s">
-        <v>602</v>
-      </c>
-      <c r="J9" s="50" t="s">
-        <v>603</v>
-      </c>
       <c r="K9" s="50" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="L9" s="50" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="M9" s="26" t="s">
+        <v>400</v>
+      </c>
+      <c r="N9" s="26" t="s">
+        <v>609</v>
+      </c>
+      <c r="O9" s="26" t="s">
         <v>401</v>
       </c>
-      <c r="N9" s="26" t="s">
-        <v>610</v>
-      </c>
-      <c r="O9" s="26" t="s">
-        <v>402</v>
-      </c>
       <c r="P9" s="26" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="32" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C10" s="32">
         <v>20</v>
       </c>
       <c r="D10" s="32" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E10" s="32">
         <v>1</v>
       </c>
       <c r="F10" s="92" t="s">
+        <v>403</v>
+      </c>
+      <c r="G10" s="93" t="s">
+        <v>403</v>
+      </c>
+      <c r="H10" s="49" t="s">
+        <v>603</v>
+      </c>
+      <c r="I10" s="49" t="s">
+        <v>603</v>
+      </c>
+      <c r="J10" s="49" t="s">
+        <v>607</v>
+      </c>
+      <c r="K10" s="49" t="s">
+        <v>408</v>
+      </c>
+      <c r="L10" s="49" t="s">
         <v>404</v>
       </c>
-      <c r="G10" s="93" t="s">
-        <v>404</v>
-      </c>
-      <c r="H10" s="49" t="s">
-        <v>604</v>
-      </c>
-      <c r="I10" s="49" t="s">
-        <v>604</v>
-      </c>
-      <c r="J10" s="49" t="s">
-        <v>608</v>
-      </c>
-      <c r="K10" s="49" t="s">
-        <v>409</v>
-      </c>
-      <c r="L10" s="49" t="s">
-        <v>405</v>
-      </c>
       <c r="M10" s="32" t="s">
+        <v>391</v>
+      </c>
+      <c r="N10" s="32" t="s">
+        <v>611</v>
+      </c>
+      <c r="O10" s="32" t="s">
         <v>392</v>
       </c>
-      <c r="N10" s="32" t="s">
-        <v>612</v>
-      </c>
-      <c r="O10" s="32" t="s">
-        <v>393</v>
-      </c>
       <c r="P10" s="32" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="26" t="s">
+        <v>612</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>390</v>
+      </c>
+      <c r="C11" s="26">
+        <v>0</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>380</v>
+      </c>
+      <c r="E11" s="26">
+        <v>0</v>
+      </c>
+      <c r="F11" s="26">
+        <v>1</v>
+      </c>
+      <c r="G11" s="50" t="s">
+        <v>403</v>
+      </c>
+      <c r="H11" s="50" t="s">
+        <v>603</v>
+      </c>
+      <c r="I11" s="50" t="s">
+        <v>603</v>
+      </c>
+      <c r="J11" s="50" t="s">
+        <v>602</v>
+      </c>
+      <c r="K11" s="50" t="s">
+        <v>407</v>
+      </c>
+      <c r="L11" s="50" t="s">
+        <v>408</v>
+      </c>
+      <c r="M11" s="26" t="s">
+        <v>391</v>
+      </c>
+      <c r="N11" s="26" t="s">
+        <v>382</v>
+      </c>
+      <c r="O11" s="26" t="s">
         <v>613</v>
       </c>
-      <c r="B11" s="26" t="s">
-        <v>391</v>
-      </c>
-      <c r="C11" s="26">
-        <v>0</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>381</v>
-      </c>
-      <c r="E11" s="26">
-        <v>0</v>
-      </c>
-      <c r="F11" s="26">
-        <v>1</v>
-      </c>
-      <c r="G11" s="50" t="s">
-        <v>404</v>
-      </c>
-      <c r="H11" s="50" t="s">
-        <v>604</v>
-      </c>
-      <c r="I11" s="50" t="s">
-        <v>604</v>
-      </c>
-      <c r="J11" s="50" t="s">
-        <v>603</v>
-      </c>
-      <c r="K11" s="50" t="s">
-        <v>408</v>
-      </c>
-      <c r="L11" s="50" t="s">
-        <v>409</v>
-      </c>
-      <c r="M11" s="26" t="s">
-        <v>392</v>
-      </c>
-      <c r="N11" s="26" t="s">
+      <c r="P11" s="26" t="s">
         <v>383</v>
-      </c>
-      <c r="O11" s="26" t="s">
-        <v>614</v>
-      </c>
-      <c r="P11" s="26" t="s">
-        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -10062,7 +10058,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="129" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B1" s="129"/>
       <c r="C1" s="51"/>
@@ -10085,19 +10081,19 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="105" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B4" s="52"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="106" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B5" s="14"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="106" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B6" s="14"/>
     </row>
@@ -10107,31 +10103,31 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="106" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B8" s="14"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="106" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B9" s="14"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="107" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B10" s="14"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="107" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B11" s="14"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B12" s="14"/>
     </row>
@@ -10140,144 +10136,144 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B14" s="14"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B15" s="14"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B16" s="14"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B17" s="14"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B18" s="14"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B19" s="14"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B20" s="14"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B21" s="14"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B22" s="14"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B23" s="14"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B24" s="14"/>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B25" s="14"/>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B26" s="14"/>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B27" s="14"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B28" s="14"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B29" s="14"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B30" s="14"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B31" s="14"/>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B32" s="14"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B33" s="14"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B34" s="14"/>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B35" s="14"/>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
   </sheetData>
@@ -10479,7 +10475,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B3">
         <v>16</v>
@@ -10542,7 +10538,7 @@
         <v>76</v>
       </c>
       <c r="V3" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="W3" cm="1">
         <f t="array" aca="1" ref="W3" ca="1">INDEX(Caliber!B2:'Caliber'!C10,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B2:'Caliber'!B10,0),2)</f>
@@ -10556,7 +10552,7 @@
         <v>92</v>
       </c>
       <c r="Z3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.3">
@@ -11433,7 +11429,7 @@
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B15">
         <v>8</v>
@@ -11512,7 +11508,7 @@
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B16">
         <v>12</v>
@@ -11785,7 +11781,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B3">
         <v>17</v>
@@ -12022,7 +12018,7 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B6">
         <v>23</v>
@@ -12259,7 +12255,7 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B9">
         <v>21</v>
@@ -12322,7 +12318,7 @@
         <v>7</v>
       </c>
       <c r="V9" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="W9" s="10" cm="1">
         <f t="array" aca="1" ref="W9" ca="1">INDEX(Caliber!B2:'Caliber'!C11,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B2:'Caliber'!B11,0),2)</f>
@@ -12333,7 +12329,7 @@
         <v>0.35</v>
       </c>
       <c r="Y9" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
@@ -12733,7 +12729,7 @@
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B15">
         <v>22</v>
@@ -12807,12 +12803,12 @@
         <v>0</v>
       </c>
       <c r="Y15" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B16">
         <v>19</v>
@@ -12891,7 +12887,7 @@
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B17">
         <v>26</v>
@@ -13501,7 +13497,7 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B7">
         <v>31</v>
@@ -13513,7 +13509,7 @@
         <v>76</v>
       </c>
       <c r="E7" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -13578,7 +13574,7 @@
         <v>0.3</v>
       </c>
       <c r="Z7" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
@@ -13665,7 +13661,7 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B9">
         <v>21</v>
@@ -13747,7 +13743,7 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B10">
         <v>19</v>
@@ -14737,7 +14733,7 @@
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B22">
         <v>23</v>
@@ -15311,7 +15307,7 @@
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B29">
         <v>30</v>
@@ -15393,7 +15389,7 @@
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B30">
         <v>32</v>
@@ -15557,7 +15553,7 @@
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B32">
         <v>30</v>
@@ -15569,7 +15565,7 @@
         <v>76</v>
       </c>
       <c r="E32" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F32" t="b">
         <v>1</v>
@@ -15639,7 +15635,7 @@
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B33">
         <v>24</v>
@@ -17525,7 +17521,7 @@
     </row>
     <row r="56" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B56">
         <v>24</v>
@@ -17607,7 +17603,7 @@
     </row>
     <row r="57" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B57">
         <v>22</v>
@@ -17689,7 +17685,7 @@
     </row>
     <row r="58" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B58">
         <v>23</v>
@@ -18876,7 +18872,7 @@
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B14">
         <v>35</v>
@@ -18942,7 +18938,7 @@
         <v>76</v>
       </c>
       <c r="W14" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="X14">
         <f>INDEX(Caliber!B13:'Caliber'!C24,MATCH(W14,Caliber!B13:'Caliber'!B24,0),2)</f>
@@ -18956,12 +18952,12 @@
         <v>178</v>
       </c>
       <c r="AA14" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B15">
         <v>37</v>
@@ -19027,7 +19023,7 @@
         <v>76</v>
       </c>
       <c r="W15" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="X15">
         <f>INDEX(Caliber!B13:'Caliber'!C24,MATCH(W15,Caliber!B13:'Caliber'!B24,0),2)</f>
@@ -19041,12 +19037,12 @@
         <v>178</v>
       </c>
       <c r="AA15" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" s="57" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B16">
         <v>24</v>
@@ -19128,7 +19124,7 @@
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B17">
         <v>27</v>
@@ -19635,7 +19631,7 @@
         <v>160</v>
       </c>
       <c r="AB3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
@@ -19724,7 +19720,7 @@
         <v>178</v>
       </c>
       <c r="AB4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -19813,7 +19809,7 @@
         <v>178</v>
       </c>
       <c r="AB5" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
@@ -20263,7 +20259,7 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B11">
         <v>24</v>
@@ -20347,12 +20343,12 @@
         <v>178</v>
       </c>
       <c r="AB11" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B12">
         <v>8</v>
@@ -20532,7 +20528,7 @@
         <v>73</v>
       </c>
       <c r="T1" s="19" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="U1" s="19" t="s">
         <v>86</v>
@@ -21156,7 +21152,7 @@
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B9">
         <v>24</v>
@@ -21225,7 +21221,7 @@
         <v>15</v>
       </c>
       <c r="X9" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="Y9" cm="1">
         <f t="array" aca="1" ref="Y9" ca="1">INDEX(Caliber!B2:'Caliber'!C11,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B2:'Caliber'!B11,0),2)</f>
@@ -21236,12 +21232,12 @@
         <v>0.35</v>
       </c>
       <c r="AA9" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B10">
         <v>78</v>
@@ -21326,7 +21322,7 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -21411,7 +21407,7 @@
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B12">
         <v>39</v>
@@ -21491,12 +21487,12 @@
         <v>0.4</v>
       </c>
       <c r="AA12" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B13">
         <v>30</v>
@@ -21576,12 +21572,12 @@
         <v>0.4</v>
       </c>
       <c r="AA13" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B14">
         <v>48</v>
@@ -21661,12 +21657,12 @@
         <v>0.4</v>
       </c>
       <c r="AA14" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B15">
         <v>47</v>
@@ -22382,7 +22378,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B8">
         <v>30</v>
@@ -22448,7 +22444,7 @@
         <v>76</v>
       </c>
       <c r="W8" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="X8" cm="1">
         <f t="array" aca="1" ref="X8" ca="1">INDEX(Caliber!B35:'Caliber'!C45,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B45,0),2)</f>
@@ -22462,12 +22458,12 @@
         <v>82</v>
       </c>
       <c r="AA8" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B9">
         <v>24</v>
@@ -22547,12 +22543,12 @@
         <v>82</v>
       </c>
       <c r="AA9" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B10">
         <v>48</v>
@@ -22618,7 +22614,7 @@
         <v>76</v>
       </c>
       <c r="W10" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="X10" cm="1">
         <f t="array" aca="1" ref="X10" ca="1">INDEX(Caliber!B35:'Caliber'!C47,MATCH(INDIRECT(ADDRESS(ROW(),COLUMN()-1)),Caliber!B35:'Caliber'!B47,0),2)</f>
@@ -22629,10 +22625,10 @@
         <v>0.4</v>
       </c>
       <c r="Z10" t="s">
+        <v>593</v>
+      </c>
+      <c r="AA10" t="s">
         <v>594</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>595</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.3">
@@ -22713,7 +22709,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>